<commit_message>
demo: restage the fixture after the review fixes
Still the synthetic fixture — Fixture Park, 180 units, TX — per the standing rule; 505 West
stays local. Gate clean against both the default denylist and the 505 West one.

Carries the ten review fixes: the mortgage-tax line now reads NOT ASSERTED without a loan
rather than asserting one at 100% LTV; the unit-mix TOTAL in-place rent is computed off the
roll so the workbook and the preview agree; the summary workbook gained the tax-evidence
rows and the closing-cost block that previously existed only in the preview; the audit trail
gained a "Value as published" column; and multi-series bars each get their own sub-track
instead of overflowing a 14px box by 30px onto the rows below.

npm run build green, 28 pages.
</commit_message>
<xml_diff>
--- a/public/downloads/underwriting-demo/sample-deal-summary.xlsx
+++ b/public/downloads/underwriting-demo/sample-deal-summary.xlsx
@@ -135,6 +135,7 @@
     <xf numFmtId="10" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -147,11 +148,10 @@
     <xf numFmtId="165" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -519,7 +519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H68"/>
+  <dimension ref="A1:H79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1033,178 +1033,325 @@
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
+          <t>Parcel / APN</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>SYN-000-00-000</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="inlineStr">
+        <is>
+          <t>The parcel the bill is issued against.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Tax area code</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>SYN-0000</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="inlineStr">
+        <is>
+          <t>Determines which published rate row applies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Basis label</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>Assessed value (synthetic)</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="inlineStr">
+        <is>
+          <t>Synthetic basis. On a real deal this row states what the basis IS in that state and whether it resets on sale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
           <t>Computed annual tax</t>
         </is>
       </c>
-      <c r="B50" s="7">
+      <c r="B53" s="7">
         <f>IFERROR(B46*B47/B48*B45-B49,"MISSING")</f>
         <v/>
       </c>
-      <c r="C50" s="6" t="inlineStr">
+      <c r="C53" s="6" t="inlineStr">
         <is>
           <t>Rate as billed, 2.148 per $100 of assessed value, read from the synthetic county bill for the 2025 tax year.</t>
         </is>
       </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="5" t="inlineStr">
-        <is>
-          <t>Computed tax per unit</t>
-        </is>
-      </c>
-      <c r="B51" s="7">
-        <f>IFERROR(B50/B18,"MISSING")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="4" t="inlineStr">
-        <is>
-          <t>Schools</t>
-        </is>
-      </c>
-      <c r="B53" s="4" t="n"/>
-      <c r="C53" s="4" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
         <is>
-          <t>Elementary school</t>
-        </is>
-      </c>
-      <c r="B54" s="5" t="inlineStr">
-        <is>
-          <t>Example Creek Elementary</t>
-        </is>
+          <t>Computed tax per unit</t>
+        </is>
+      </c>
+      <c r="B54" s="7">
+        <f>IFERROR(B53/B18,"MISSING")</f>
+        <v/>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t>Elementary rating</t>
-        </is>
-      </c>
-      <c r="B55" s="8" t="n">
-        <v>7</v>
+          <t>Billed by the county (2025)</t>
+        </is>
+      </c>
+      <c r="B55" s="7" t="n">
+        <v>494040</v>
+      </c>
+      <c r="C55" s="6" t="inlineStr">
+        <is>
+          <t>The county's own figure, for the cross-check below.</t>
+        </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="5" t="inlineStr">
         <is>
-          <t>Middle school</t>
-        </is>
-      </c>
-      <c r="B56" s="5" t="inlineStr">
-        <is>
-          <t>Example Ridge Middle</t>
+          <t>Check: computed vs billed</t>
+        </is>
+      </c>
+      <c r="B56" s="12">
+        <f>IF(B55=0,"NOT CHECKED",IF(ABS(B53-B55)/B55&lt;=0.02,"ties","REVIEW"))</f>
+        <v/>
+      </c>
+      <c r="C56" s="6" t="inlineStr">
+        <is>
+          <t>A computed tax that cannot be tied to the actual bill is an estimate wearing the clothes of a fact.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="5" t="inlineStr">
         <is>
-          <t>Middle rating</t>
-        </is>
-      </c>
-      <c r="B57" s="8" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="5" t="inlineStr">
-        <is>
-          <t>High school</t>
-        </is>
-      </c>
-      <c r="B58" s="5" t="inlineStr">
-        <is>
-          <t>Sample City High</t>
-        </is>
+          <t>Check: difference</t>
+        </is>
+      </c>
+      <c r="B57" s="7">
+        <f>IFERROR(B53-B55,"")</f>
+        <v/>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="5" t="inlineStr">
-        <is>
-          <t>High rating</t>
-        </is>
-      </c>
-      <c r="B59" s="8" t="n">
-        <v>7</v>
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>Closing costs at the illustrative price</t>
+        </is>
+      </c>
+      <c r="B59" s="4" t="n"/>
+      <c r="C59" s="4" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
+        <is>
+          <t>Transfer tax</t>
+        </is>
+      </c>
+      <c r="B60" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C60" s="6" t="inlineStr">
+        <is>
+          <t>No real-estate transfer tax · Tex. Const. art. VIII, sec. 29 (added 2015) · The bar is on enacting a transfer tax after 2016-01-01; Texas had none, so the rate is zero. The same section expressly permits a tax on title insurance, and Texas title premiums are state-promulgated and material — a zero here does not mean a cheap closing.</t>
+        </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="4" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-      <c r="B61" s="4" t="n"/>
-      <c r="C61" s="4" t="n"/>
+      <c r="A61" s="5" t="inlineStr">
+        <is>
+          <t>Mortgage / recording tax</t>
+        </is>
+      </c>
+      <c r="B61" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C61" s="6" t="inlineStr">
+        <is>
+          <t>No mortgage tax · No imposing statute; Tex. Loc. Gov't Code ch. 118 · Proven by absence of an imposing statute rather than by an affirmative constitutional bar, which is a weaker form of proof than Arizona's. Recording is a flat per-page schedule.</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
         <is>
-          <t>Notes</t>
-        </is>
-      </c>
-      <c r="B62" s="5" t="inlineStr">
-        <is>
-          <t>Synthetic deal built to exercise the output formats. Pricing is illustrative and no licensed data source was used. Comps come only from an operator's own weekly rent scrape.</t>
+          <t>Closing-cost basis</t>
+        </is>
+      </c>
+      <c r="B62" s="7" t="n">
+        <v>38700000</v>
+      </c>
+      <c r="C62" s="6" t="inlineStr">
+        <is>
+          <t>Transfer tax is computed on the purchase price. A mortgage or recording tax is computed on the LOAN AMOUNT, and is reported as not asserted when no loan is stated — never inferred from the price, which would assume 100% leverage. Rates are verified against a primary authority and carry the citation and the date confirmed; a state absent from the table reports as not asserted rather than as zero.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>Boundaries</t>
+          <t>Schools</t>
         </is>
       </c>
       <c r="B64" s="4" t="n"/>
       <c r="C64" s="4" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="12" t="inlineStr">
+      <c r="A65" s="5" t="inlineStr">
+        <is>
+          <t>Elementary school</t>
+        </is>
+      </c>
+      <c r="B65" s="5" t="inlineStr">
+        <is>
+          <t>Example Creek Elementary</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr">
+        <is>
+          <t>Elementary rating</t>
+        </is>
+      </c>
+      <c r="B66" s="8" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="5" t="inlineStr">
+        <is>
+          <t>Middle school</t>
+        </is>
+      </c>
+      <c r="B67" s="5" t="inlineStr">
+        <is>
+          <t>Example Ridge Middle</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="5" t="inlineStr">
+        <is>
+          <t>Middle rating</t>
+        </is>
+      </c>
+      <c r="B68" s="8" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="5" t="inlineStr">
+        <is>
+          <t>High school</t>
+        </is>
+      </c>
+      <c r="B69" s="5" t="inlineStr">
+        <is>
+          <t>Sample City High</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="5" t="inlineStr">
+        <is>
+          <t>High rating</t>
+        </is>
+      </c>
+      <c r="B70" s="8" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="B72" s="4" t="n"/>
+      <c r="C72" s="4" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="5" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="B73" s="5" t="inlineStr">
+        <is>
+          <t>Synthetic deal built to exercise the output formats. Pricing is illustrative and no licensed data source was used. Comps come only from an operator's own weekly rent scrape.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="4" t="inlineStr">
+        <is>
+          <t>Boundaries</t>
+        </is>
+      </c>
+      <c r="B75" s="4" t="n"/>
+      <c r="C75" s="4" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="13" t="inlineStr">
         <is>
           <t>Excluded by design</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr">
+      <c r="B76" t="inlineStr">
         <is>
           <t>Third-party licensed rent-comp feeds</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="12" t="inlineStr">
+    <row r="77">
+      <c r="A77" s="13" t="inlineStr">
         <is>
           <t>Excluded by design</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr">
+      <c r="B77" t="inlineStr">
         <is>
           <t>Subscription market-data providers</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="12" t="inlineStr">
+    <row r="78">
+      <c r="A78" s="13" t="inlineStr">
         <is>
           <t>Excluded by design</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr">
+      <c r="B78" t="inlineStr">
         <is>
           <t>Any employer-owned deal data or template</t>
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="12" t="inlineStr">
+    <row r="79">
+      <c r="A79" s="13" t="inlineStr">
         <is>
           <t>Synthetic deal</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr">
+      <c r="B79" t="inlineStr">
         <is>
           <t>Every figure is fabricated for demonstration. No real property is described.</t>
         </is>
@@ -1271,67 +1418,67 @@
       <c r="H4" s="3" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>Community</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="14" t="inlineStr">
         <is>
           <t>Distance (mi)</t>
         </is>
       </c>
-      <c r="C5" s="13" t="inlineStr">
+      <c r="C5" s="14" t="inlineStr">
         <is>
           <t>Floor plan</t>
         </is>
       </c>
-      <c r="D5" s="13" t="inlineStr">
+      <c r="D5" s="14" t="inlineStr">
         <is>
           <t>Beds</t>
         </is>
       </c>
-      <c r="E5" s="13" t="inlineStr">
+      <c r="E5" s="14" t="inlineStr">
         <is>
           <t>Baths</t>
         </is>
       </c>
-      <c r="F5" s="13" t="inlineStr">
+      <c r="F5" s="14" t="inlineStr">
         <is>
           <t>SF</t>
         </is>
       </c>
-      <c r="G5" s="13" t="inlineStr">
+      <c r="G5" s="14" t="inlineStr">
         <is>
           <t>Asking rent</t>
         </is>
       </c>
-      <c r="H5" s="13" t="inlineStr">
+      <c r="H5" s="14" t="inlineStr">
         <is>
           <t>Concession</t>
         </is>
       </c>
-      <c r="I5" s="13" t="inlineStr">
+      <c r="I5" s="14" t="inlineStr">
         <is>
           <t>Net effective rent</t>
         </is>
       </c>
-      <c r="J5" s="13" t="inlineStr">
+      <c r="J5" s="14" t="inlineStr">
         <is>
           <t>Asking $/SF</t>
         </is>
       </c>
-      <c r="K5" s="13" t="inlineStr">
+      <c r="K5" s="14" t="inlineStr">
         <is>
           <t>Occupancy</t>
         </is>
       </c>
-      <c r="L5" s="13" t="inlineStr">
+      <c r="L5" s="14" t="inlineStr">
         <is>
           <t>As-of date</t>
         </is>
       </c>
-      <c r="M5" s="13" t="inlineStr">
+      <c r="M5" s="14" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
@@ -1351,10 +1498,10 @@
           <t>1BR-A</t>
         </is>
       </c>
-      <c r="D6" s="14" t="n">
+      <c r="D6" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="E6" s="14" t="n">
+      <c r="E6" s="15" t="n">
         <v>1</v>
       </c>
       <c r="F6" s="7" t="n">
@@ -1369,14 +1516,14 @@
       <c r="I6" s="7" t="n">
         <v>1450</v>
       </c>
-      <c r="J6" s="15">
+      <c r="J6" s="16">
         <f>IFERROR(G6/F6,"")</f>
         <v/>
       </c>
       <c r="K6" s="11" t="n">
         <v>0.9399999999999999</v>
       </c>
-      <c r="L6" s="16" t="n">
+      <c r="L6" s="17" t="n">
         <v>46195</v>
       </c>
       <c r="M6" s="5" t="inlineStr">
@@ -1399,10 +1546,10 @@
           <t>2BR-B</t>
         </is>
       </c>
-      <c r="D7" s="14" t="n">
+      <c r="D7" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="E7" s="14" t="n">
+      <c r="E7" s="15" t="n">
         <v>2</v>
       </c>
       <c r="F7" s="7" t="n">
@@ -1417,14 +1564,14 @@
       <c r="I7" s="7" t="n">
         <v>1775</v>
       </c>
-      <c r="J7" s="15">
+      <c r="J7" s="16">
         <f>IFERROR(G7/F7,"")</f>
         <v/>
       </c>
       <c r="K7" s="11" t="n">
         <v>0.9399999999999999</v>
       </c>
-      <c r="L7" s="16" t="n">
+      <c r="L7" s="17" t="n">
         <v>46195</v>
       </c>
       <c r="M7" s="5" t="inlineStr">
@@ -1447,10 +1594,10 @@
           <t>A1</t>
         </is>
       </c>
-      <c r="D8" s="14" t="n">
+      <c r="D8" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="E8" s="14" t="n">
+      <c r="E8" s="15" t="n">
         <v>1</v>
       </c>
       <c r="F8" s="7" t="n">
@@ -1465,14 +1612,14 @@
       <c r="I8" s="7" t="n">
         <v>1440</v>
       </c>
-      <c r="J8" s="15">
+      <c r="J8" s="16">
         <f>IFERROR(G8/F8,"")</f>
         <v/>
       </c>
       <c r="K8" s="11" t="n">
         <v>0.96</v>
       </c>
-      <c r="L8" s="16" t="n">
+      <c r="L8" s="17" t="n">
         <v>46195</v>
       </c>
       <c r="M8" s="5" t="inlineStr">
@@ -1495,10 +1642,10 @@
           <t>B2</t>
         </is>
       </c>
-      <c r="D9" s="14" t="n">
+      <c r="D9" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="E9" s="14" t="n">
+      <c r="E9" s="15" t="n">
         <v>2</v>
       </c>
       <c r="F9" s="7" t="n">
@@ -1513,14 +1660,14 @@
       <c r="I9" s="7" t="n">
         <v>1720</v>
       </c>
-      <c r="J9" s="15">
+      <c r="J9" s="16">
         <f>IFERROR(G9/F9,"")</f>
         <v/>
       </c>
       <c r="K9" s="11" t="n">
         <v>0.9399999999999999</v>
       </c>
-      <c r="L9" s="16" t="n">
+      <c r="L9" s="17" t="n">
         <v>46195</v>
       </c>
       <c r="M9" s="5" t="inlineStr">
@@ -1543,10 +1690,10 @@
           <t>C1</t>
         </is>
       </c>
-      <c r="D10" s="14" t="n">
+      <c r="D10" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="E10" s="14" t="n">
+      <c r="E10" s="15" t="n">
         <v>2</v>
       </c>
       <c r="F10" s="7" t="n">
@@ -1561,14 +1708,14 @@
       <c r="I10" s="7" t="n">
         <v>2140</v>
       </c>
-      <c r="J10" s="15">
+      <c r="J10" s="16">
         <f>IFERROR(G10/F10,"")</f>
         <v/>
       </c>
       <c r="K10" s="11" t="n">
         <v>0.96</v>
       </c>
-      <c r="L10" s="16" t="n">
+      <c r="L10" s="17" t="n">
         <v>46195</v>
       </c>
       <c r="M10" s="5" t="inlineStr">
@@ -1591,10 +1738,10 @@
           <t>Aspen</t>
         </is>
       </c>
-      <c r="D11" s="14" t="n">
+      <c r="D11" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="E11" s="14" t="n">
+      <c r="E11" s="15" t="n">
         <v>1</v>
       </c>
       <c r="F11" s="7" t="n">
@@ -1609,14 +1756,14 @@
       <c r="I11" s="7" t="n">
         <v>1430</v>
       </c>
-      <c r="J11" s="15">
+      <c r="J11" s="16">
         <f>IFERROR(G11/F11,"")</f>
         <v/>
       </c>
       <c r="K11" s="11" t="n">
         <v>0.9399999999999999</v>
       </c>
-      <c r="L11" s="16" t="n">
+      <c r="L11" s="17" t="n">
         <v>46195</v>
       </c>
       <c r="M11" s="5" t="inlineStr">
@@ -1639,10 +1786,10 @@
           <t>Birch</t>
         </is>
       </c>
-      <c r="D12" s="14" t="n">
+      <c r="D12" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="E12" s="14" t="n">
+      <c r="E12" s="15" t="n">
         <v>2</v>
       </c>
       <c r="F12" s="7" t="n">
@@ -1657,14 +1804,14 @@
       <c r="I12" s="7" t="n">
         <v>1790</v>
       </c>
-      <c r="J12" s="15">
+      <c r="J12" s="16">
         <f>IFERROR(G12/F12,"")</f>
         <v/>
       </c>
       <c r="K12" s="11" t="n">
         <v>0.9399999999999999</v>
       </c>
-      <c r="L12" s="16" t="n">
+      <c r="L12" s="17" t="n">
         <v>46195</v>
       </c>
       <c r="M12" s="5" t="inlineStr">
@@ -1687,10 +1834,10 @@
           <t>One Bed</t>
         </is>
       </c>
-      <c r="D13" s="14" t="n">
+      <c r="D13" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="E13" s="14" t="n">
+      <c r="E13" s="15" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="7" t="n">
@@ -1705,14 +1852,14 @@
       <c r="I13" s="7" t="n">
         <v>1465</v>
       </c>
-      <c r="J13" s="15">
+      <c r="J13" s="16">
         <f>IFERROR(G13/F13,"")</f>
         <v/>
       </c>
       <c r="K13" s="11" t="n">
         <v>0.96</v>
       </c>
-      <c r="L13" s="16" t="n">
+      <c r="L13" s="17" t="n">
         <v>46195</v>
       </c>
       <c r="M13" s="5" t="inlineStr">
@@ -1735,10 +1882,10 @@
           <t>Two Bed</t>
         </is>
       </c>
-      <c r="D14" s="14" t="n">
+      <c r="D14" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="E14" s="14" t="n">
+      <c r="E14" s="15" t="n">
         <v>2.5</v>
       </c>
       <c r="F14" s="7" t="n">
@@ -1753,14 +1900,14 @@
       <c r="I14" s="7" t="n">
         <v>1860</v>
       </c>
-      <c r="J14" s="15">
+      <c r="J14" s="16">
         <f>IFERROR(G14/F14,"")</f>
         <v/>
       </c>
       <c r="K14" s="11" t="n">
         <v>0.9399999999999999</v>
       </c>
-      <c r="L14" s="16" t="n">
+      <c r="L14" s="17" t="n">
         <v>46195</v>
       </c>
       <c r="M14" s="5" t="inlineStr">
@@ -1783,10 +1930,10 @@
           <t>Three Bed</t>
         </is>
       </c>
-      <c r="D15" s="14" t="n">
+      <c r="D15" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="E15" s="14" t="n">
+      <c r="E15" s="15" t="n">
         <v>2.5</v>
       </c>
       <c r="F15" s="7" t="n">
@@ -1801,14 +1948,14 @@
       <c r="I15" s="7" t="n">
         <v>2385</v>
       </c>
-      <c r="J15" s="15">
+      <c r="J15" s="16">
         <f>IFERROR(G15/F15,"")</f>
         <v/>
       </c>
       <c r="K15" s="11" t="n">
         <v>0.96</v>
       </c>
-      <c r="L15" s="16" t="n">
+      <c r="L15" s="17" t="n">
         <v>46195</v>
       </c>
       <c r="M15" s="5" t="inlineStr">
@@ -1935,37 +2082,37 @@
       <c r="H4" s="3" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>Ring</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="14" t="inlineStr">
         <is>
           <t>Population</t>
         </is>
       </c>
-      <c r="C5" s="13" t="inlineStr">
+      <c r="C5" s="14" t="inlineStr">
         <is>
           <t>Households</t>
         </is>
       </c>
-      <c r="D5" s="13" t="inlineStr">
+      <c r="D5" s="14" t="inlineStr">
         <is>
           <t>Median household income</t>
         </is>
       </c>
-      <c r="E5" s="13" t="inlineStr">
+      <c r="E5" s="14" t="inlineStr">
         <is>
           <t>Total jobs</t>
         </is>
       </c>
-      <c r="F5" s="13" t="inlineStr">
+      <c r="F5" s="14" t="inlineStr">
         <is>
           <t>Population growth (5-yr)</t>
         </is>
       </c>
-      <c r="G5" s="13" t="inlineStr">
+      <c r="G5" s="14" t="inlineStr">
         <is>
           <t>Renter share</t>
         </is>
@@ -2072,27 +2219,27 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="17" t="inlineStr">
+      <c r="A10" s="18" t="inlineStr">
         <is>
           <t>MSA</t>
         </is>
       </c>
-      <c r="B10" s="18" t="n">
+      <c r="B10" s="19" t="n">
         <v>2418000</v>
       </c>
-      <c r="C10" s="18" t="n">
+      <c r="C10" s="19" t="n">
         <v>903400</v>
       </c>
-      <c r="D10" s="18" t="n">
+      <c r="D10" s="19" t="n">
         <v>86100</v>
       </c>
-      <c r="E10" s="18" t="n">
+      <c r="E10" s="19" t="n">
         <v>1284000</v>
       </c>
-      <c r="F10" s="19" t="n">
+      <c r="F10" s="20" t="n">
         <v>0.073</v>
       </c>
-      <c r="G10" s="19" t="n">
+      <c r="G10" s="20" t="n">
         <v>0.37</v>
       </c>
     </row>
@@ -2148,22 +2295,22 @@
       <c r="H4" s="3" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>Ring</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="14" t="inlineStr">
         <is>
           <t>Stage</t>
         </is>
       </c>
-      <c r="C5" s="13" t="inlineStr">
+      <c r="C5" s="14" t="inlineStr">
         <is>
           <t>Projects</t>
         </is>
       </c>
-      <c r="D5" s="13" t="inlineStr">
+      <c r="D5" s="14" t="inlineStr">
         <is>
           <t>Units</t>
         </is>
@@ -2397,22 +2544,22 @@
       <c r="D19" s="4" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="13" t="inlineStr">
+      <c r="A20" s="14" t="inlineStr">
         <is>
           <t>Ring</t>
         </is>
       </c>
-      <c r="B20" s="13" t="inlineStr">
+      <c r="B20" s="14" t="inlineStr">
         <is>
           <t>Pipeline units</t>
         </is>
       </c>
-      <c r="C20" s="13" t="inlineStr">
+      <c r="C20" s="14" t="inlineStr">
         <is>
           <t>Existing stock</t>
         </is>
       </c>
-      <c r="D20" s="13" t="inlineStr">
+      <c r="D20" s="14" t="inlineStr">
         <is>
           <t>Units as % of stock</t>
         </is>
@@ -2487,11 +2634,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="62" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="62" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2526,1150 +2674,1373 @@
       <c r="H4" s="3" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="13" t="inlineStr">
         <is>
           <t>Stamped values in this workbook</t>
         </is>
       </c>
-      <c r="B5" s="20" t="n">
+      <c r="B5" s="21" t="n">
         <v>42</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="13" t="inlineStr">
         <is>
           <t>Coverage of the required set</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>42/42 (100%)</t>
+          <t>50/50 (100%)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="inlineStr">
+      <c r="A8" s="14" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>Value as published</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="inlineStr">
         <is>
           <t>Source document</t>
         </is>
       </c>
-      <c r="C8" s="13" t="inlineStr">
+      <c r="D8" s="14" t="inlineStr">
         <is>
           <t>Where in it</t>
         </is>
       </c>
-      <c r="D8" s="13" t="inlineStr">
+      <c r="E8" s="14" t="inlineStr">
         <is>
           <t>How</t>
         </is>
       </c>
-      <c r="E8" s="13" t="inlineStr">
+      <c r="F8" s="14" t="inlineStr">
         <is>
           <t>Built from</t>
         </is>
       </c>
-      <c r="F8" s="13" t="inlineStr">
+      <c r="G8" s="14" t="inlineStr">
         <is>
           <t>Supporting quote / note</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="21" t="inlineStr">
+      <c r="A9" s="22" t="inlineStr">
         <is>
           <t>closing_costs.mortgage_tax.amount</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
           <t>Vendored state rate table</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>closing_costs.py</t>
-        </is>
-      </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
+          <t>closing_costs.MORTGAGE_TAX</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
           <t>computed</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>pricing.price_per_unit, summary.state</t>
-        </is>
-      </c>
-      <c r="F9" s="22" t="n"/>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>closing_costs.loan_amount, summary.state</t>
+        </is>
+      </c>
+      <c r="G9" s="23" t="inlineStr">
+        <is>
+          <t>Computed on the LOAN, never on the price. With no loan amount the line is reported as not asserted rather than inferred at 100% leverage.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="21" t="inlineStr">
+      <c r="A10" s="22" t="inlineStr">
         <is>
           <t>closing_costs.transfer_tax.amount</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
           <t>Vendored state rate table</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>closing_costs.py</t>
-        </is>
-      </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
+          <t>closing_costs.TRANSFER_TAX</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
           <t>computed</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>pricing.price_per_unit, summary.state</t>
-        </is>
-      </c>
-      <c r="F10" s="22" t="n"/>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>pricing.price_per_unit, pricing.unit_count, summary.state, closing_costs.price</t>
+        </is>
+      </c>
+      <c r="G10" s="23" t="inlineStr">
+        <is>
+          <t>Rate applied to price_per_unit x unit_count. Per-unit statutes round the consideration up.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="21" t="inlineStr">
+      <c r="A11" s="22" t="inlineStr">
         <is>
           <t>comps.rows</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
+          <t>10 entries</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
           <t>Synthetic weekly rent scrape</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="E11" s="5" t="inlineStr">
         <is>
           <t>read</t>
         </is>
       </c>
-      <c r="E11" s="23" t="n"/>
-      <c r="F11" s="24" t="inlineStr">
+      <c r="F11" s="12" t="n"/>
+      <c r="G11" s="23" t="inlineStr">
         <is>
           <t>Own weekly scrape; asking and net effective stated separately.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="21" t="inlineStr">
+      <c r="A12" s="22" t="inlineStr">
         <is>
           <t>demand.rings</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
+          <t>5 entries</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
           <t>Synthetic public data extract</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="E12" s="5" t="inlineStr">
         <is>
           <t>read</t>
         </is>
       </c>
-      <c r="E12" s="23" t="n"/>
-      <c r="F12" s="24" t="inlineStr">
+      <c r="F12" s="12" t="n"/>
+      <c r="G12" s="23" t="inlineStr">
         <is>
           <t>Ring demographics.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="21" t="inlineStr">
+      <c r="A13" s="22" t="inlineStr">
         <is>
           <t>pricing.price_per_unit</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
+          <t>215,000</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
           <t>Supplied by the operator</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="E13" s="5" t="inlineStr">
         <is>
           <t>read</t>
         </is>
       </c>
-      <c r="E13" s="23" t="n"/>
-      <c r="F13" s="24" t="inlineStr">
+      <c r="F13" s="12" t="n"/>
+      <c r="G13" s="23" t="inlineStr">
         <is>
           <t>Illustrative. Inside the band a per-unit sale price occupies.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="21" t="inlineStr">
+      <c r="A14" s="22" t="inlineStr">
         <is>
           <t>pricing.unit_count</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
+          <t>180</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
           <t>Synthetic rent roll export</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>Rent Roll!A:A</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="E14" s="5" t="inlineStr">
         <is>
           <t>derived</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="F14" s="5" t="inlineStr">
         <is>
           <t>summary.unit_count</t>
         </is>
       </c>
-      <c r="F14" s="22" t="n"/>
+      <c r="G14" s="24" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="21" t="inlineStr">
+      <c r="A15" s="22" t="inlineStr">
         <is>
           <t>summary.assessed_value_basis</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
+          <t>23,000,000</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
           <t>Synthetic county tax record</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>Valuation notice</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="E15" s="5" t="inlineStr">
         <is>
           <t>read</t>
         </is>
       </c>
-      <c r="E15" s="23" t="n"/>
-      <c r="F15" s="22" t="n"/>
+      <c r="F15" s="12" t="n"/>
+      <c r="G15" s="24" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="21" t="inlineStr">
+      <c r="A16" s="22" t="inlineStr">
         <is>
           <t>summary.assessment_ratio</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
           <t>Synthetic county tax record</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>Rate table</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="E16" s="5" t="inlineStr">
         <is>
           <t>read</t>
         </is>
       </c>
-      <c r="E16" s="23" t="n"/>
-      <c r="F16" s="22" t="n"/>
+      <c r="F16" s="12" t="n"/>
+      <c r="G16" s="24" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="21" t="inlineStr">
+      <c r="A17" s="22" t="inlineStr">
         <is>
           <t>summary.city</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
+          <t>Sample City</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
           <t>Synthetic offering memorandum</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>p.4</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="E17" s="5" t="inlineStr">
         <is>
           <t>read</t>
         </is>
       </c>
-      <c r="E17" s="23" t="n"/>
-      <c r="F17" s="22" t="n"/>
+      <c r="F17" s="12" t="n"/>
+      <c r="G17" s="24" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="21" t="inlineStr">
+      <c r="A18" s="22" t="inlineStr">
         <is>
           <t>summary.construction_status</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
+          <t>Stabilized</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
           <t>Synthetic offering memorandum</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr">
         <is>
           <t>p.6</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="E18" s="5" t="inlineStr">
         <is>
           <t>read</t>
         </is>
       </c>
-      <c r="E18" s="23" t="n"/>
-      <c r="F18" s="22" t="n"/>
+      <c r="F18" s="12" t="n"/>
+      <c r="G18" s="24" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="21" t="inlineStr">
+      <c r="A19" s="22" t="inlineStr">
         <is>
           <t>summary.county</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
+          <t>Example County</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
           <t>Synthetic offering memorandum</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="D19" s="5" t="inlineStr">
         <is>
           <t>p.4</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="E19" s="5" t="inlineStr">
         <is>
           <t>read</t>
         </is>
       </c>
-      <c r="E19" s="23" t="n"/>
-      <c r="F19" s="22" t="n"/>
+      <c r="F19" s="12" t="n"/>
+      <c r="G19" s="24" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="21" t="inlineStr">
+      <c r="A20" s="22" t="inlineStr">
         <is>
           <t>summary.deal_name</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
+          <t>Fixture Park</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
           <t>Synthetic offering memorandum</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr">
         <is>
           <t>p.1</t>
         </is>
       </c>
-      <c r="D20" s="5" t="inlineStr">
+      <c r="E20" s="5" t="inlineStr">
         <is>
           <t>read</t>
         </is>
       </c>
-      <c r="E20" s="23" t="n"/>
-      <c r="F20" s="24" t="inlineStr">
+      <c r="F20" s="12" t="n"/>
+      <c r="G20" s="23" t="inlineStr">
         <is>
           <t>Fixture Park</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="21" t="inlineStr">
+      <c r="A21" s="22" t="inlineStr">
         <is>
           <t>summary.deal_status</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
+          <t>On the market</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
           <t>Synthetic offering memorandum</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="D21" s="5" t="inlineStr">
         <is>
           <t>p.2</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="E21" s="5" t="inlineStr">
         <is>
           <t>read</t>
         </is>
       </c>
-      <c r="E21" s="23" t="n"/>
-      <c r="F21" s="22" t="n"/>
+      <c r="F21" s="12" t="n"/>
+      <c r="G21" s="24" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="21" t="inlineStr">
+      <c r="A22" s="22" t="inlineStr">
         <is>
           <t>summary.delivery_date</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
+          <t>Delivered 2019; fully stabilized since 2021</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
           <t>Synthetic offering memorandum</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>p.6</t>
         </is>
       </c>
-      <c r="D22" s="5" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr">
         <is>
           <t>read</t>
         </is>
       </c>
-      <c r="E22" s="23" t="n"/>
-      <c r="F22" s="22" t="n"/>
+      <c r="F22" s="12" t="n"/>
+      <c r="G22" s="24" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="21" t="inlineStr">
+      <c r="A23" s="22" t="inlineStr">
         <is>
           <t>summary.fair_market_value</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
+          <t>39,600,000</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
           <t>Supplied by the operator</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr">
+      <c r="E23" s="5" t="inlineStr">
         <is>
           <t>read</t>
         </is>
       </c>
-      <c r="E23" s="23" t="n"/>
-      <c r="F23" s="24" t="inlineStr">
+      <c r="F23" s="12" t="n"/>
+      <c r="G23" s="23" t="inlineStr">
         <is>
           <t>Operator's own estimate.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="21" t="inlineStr">
+      <c r="A24" s="22" t="inlineStr">
         <is>
           <t>summary.in_place_rent_avg</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
+          <t>1,795.36</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
           <t>Derived by the pipeline</t>
         </is>
       </c>
-      <c r="C24" s="5" t="inlineStr">
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Unit Mix Summary!E</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>computed</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>rent_roll.units</t>
+        </is>
+      </c>
+      <c r="G24" s="23" t="inlineStr">
+        <is>
+          <t>Occupied units, straight off the roll.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="22" t="inlineStr">
+        <is>
+          <t>summary.listing_brokerage</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Listing brokerage</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Derived by the pipeline</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>derived</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>summary.seller_entity</t>
+        </is>
+      </c>
+      <c r="G25" s="23" t="inlineStr">
+        <is>
+          <t>Generic label; no firm or individual is named in a published file.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="22" t="inlineStr">
+        <is>
+          <t>summary.market_rent_for_model</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>1,834.78</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Derived by the pipeline</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
         <is>
           <t>Unit Mix Summary!H</t>
         </is>
       </c>
-      <c r="D24" s="5" t="inlineStr">
+      <c r="E26" s="5" t="inlineStr">
         <is>
           <t>computed</t>
         </is>
       </c>
-      <c r="E24" s="5" t="inlineStr">
+      <c r="F26" s="5" t="inlineStr">
         <is>
           <t>rent_roll.units</t>
         </is>
       </c>
-      <c r="F24" s="24" t="inlineStr">
-        <is>
-          <t>Occupied units, weighted.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="21" t="inlineStr">
-        <is>
-          <t>summary.listing_brokerage</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="inlineStr">
+      <c r="G26" s="23" t="inlineStr">
+        <is>
+          <t>New-lease average where a plan has new leases in the window, else in-place. Never a blend.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="22" t="inlineStr">
+        <is>
+          <t>summary.msa</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Sample City MSA</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
         <is>
           <t>Derived by the pipeline</t>
         </is>
       </c>
-      <c r="C25" s="5" t="inlineStr">
+      <c r="D27" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D25" s="5" t="inlineStr">
+      <c r="E27" s="5" t="inlineStr">
         <is>
           <t>derived</t>
         </is>
       </c>
-      <c r="E25" s="5" t="inlineStr">
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>summary.city, summary.state</t>
+        </is>
+      </c>
+      <c r="G27" s="23" t="inlineStr">
+        <is>
+          <t>Metro assigned from the city/state pair.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="22" t="inlineStr">
+        <is>
+          <t>summary.pricing_guidance</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>$215,000 per unit (illustrative)</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Supplied by the operator</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F28" s="12" t="n"/>
+      <c r="G28" s="23" t="inlineStr">
+        <is>
+          <t>Illustrative figure supplied directly; not a quote or an offer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="22" t="inlineStr">
+        <is>
+          <t>summary.product_detail</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>180 units across six plans: 62 one-bedroom (720–795 SF), 78 two-bedroom (1,050–1,140 SF…</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>Synthetic offering memorandum</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>p.7</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F29" s="12" t="n"/>
+      <c r="G29" s="24" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="22" t="inlineStr">
+        <is>
+          <t>summary.product_type</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>MF</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Synthetic offering memorandum</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>p.6</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F30" s="12" t="n"/>
+      <c r="G30" s="24" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="22" t="inlineStr">
+        <is>
+          <t>summary.school_elementary_name</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>Example Creek Elementary</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>Synthetic public data extract</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>School attendance lookup</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F31" s="12" t="n"/>
+      <c r="G31" s="24" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="22" t="inlineStr">
+        <is>
+          <t>summary.school_high_name</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Sample City High</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>Synthetic public data extract</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>School attendance lookup</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F32" s="12" t="n"/>
+      <c r="G32" s="24" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="22" t="inlineStr">
+        <is>
+          <t>summary.school_middle_name</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>Example Ridge Middle</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>Synthetic public data extract</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>School attendance lookup</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F33" s="12" t="n"/>
+      <c r="G33" s="24" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="22" t="inlineStr">
         <is>
           <t>summary.seller_entity</t>
         </is>
       </c>
-      <c r="F25" s="24" t="inlineStr">
-        <is>
-          <t>Generic label; no firm or individual is named in a published file.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="21" t="inlineStr">
-        <is>
-          <t>summary.market_rent_for_model</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>Derived by the pipeline</t>
-        </is>
-      </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>Unit Mix Summary!K</t>
-        </is>
-      </c>
-      <c r="D26" s="5" t="inlineStr">
-        <is>
-          <t>computed</t>
-        </is>
-      </c>
-      <c r="E26" s="5" t="inlineStr">
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Sample City Residential Holdings LLC</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>Synthetic offering memorandum</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>p.2</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F34" s="12" t="n"/>
+      <c r="G34" s="24" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="22" t="inlineStr">
+        <is>
+          <t>summary.state</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>Synthetic offering memorandum</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>p.4</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F35" s="12" t="n"/>
+      <c r="G35" s="24" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="22" t="inlineStr">
+        <is>
+          <t>summary.street_address</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>1400 Example Parkway</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>Synthetic offering memorandum</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>p.4</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F36" s="12" t="n"/>
+      <c r="G36" s="23" t="inlineStr">
+        <is>
+          <t>1400 Example Parkway</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="22" t="inlineStr">
+        <is>
+          <t>summary.structure</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>Three-story garden, surface parked</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>Synthetic offering memorandum</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>p.6</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F37" s="12" t="n"/>
+      <c r="G37" s="23" t="inlineStr">
+        <is>
+          <t>Three-story garden, surface parked</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="22" t="inlineStr">
+        <is>
+          <t>summary.tax_area_code</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>SYN-0000</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>Synthetic county tax record</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Rate table</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F38" s="12" t="n"/>
+      <c r="G38" s="24" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="22" t="inlineStr">
+        <is>
+          <t>summary.tax_basis_label</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>Assessed value (synthetic)</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>Synthetic county tax record</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>Valuation notice</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F39" s="12" t="n"/>
+      <c r="G39" s="24" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="22" t="inlineStr">
+        <is>
+          <t>summary.tax_basis_note</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>Synthetic basis. On a real deal this row states what the basis IS in that state and whe…</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>Synthetic county tax record</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>Valuation notice</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F40" s="12" t="n"/>
+      <c r="G40" s="24" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="22" t="inlineStr">
+        <is>
+          <t>summary.tax_billed_amount</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>494,040</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>Synthetic county tax record</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>Tax bill</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F41" s="12" t="n"/>
+      <c r="G41" s="24" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="22" t="inlineStr">
+        <is>
+          <t>summary.tax_billed_year</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>2,025</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>Synthetic county tax record</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Tax bill</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F42" s="12" t="n"/>
+      <c r="G42" s="24" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="22" t="inlineStr">
+        <is>
+          <t>summary.tax_divisor</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>Synthetic county tax record</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>Rate table</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F43" s="12" t="n"/>
+      <c r="G43" s="24" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="22" t="inlineStr">
+        <is>
+          <t>summary.tax_exemption</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>Synthetic county tax record</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>Valuation notice</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F44" s="12" t="n"/>
+      <c r="G44" s="24" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="22" t="inlineStr">
+        <is>
+          <t>summary.tax_parcel_id</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>SYN-000-00-000</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>Synthetic county tax record</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>Parcel record</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F45" s="12" t="n"/>
+      <c r="G45" s="24" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="22" t="inlineStr">
+        <is>
+          <t>summary.tax_rate_as_billed</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>2.15</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>Synthetic county tax record</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>Rate table, synthetic district</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F46" s="12" t="n"/>
+      <c r="G46" s="24" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="22" t="inlineStr">
+        <is>
+          <t>summary.unit_count</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>180</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>Synthetic rent roll export</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>Rent Roll!A:A</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>derived</t>
+        </is>
+      </c>
+      <c r="F47" s="5" t="inlineStr">
         <is>
           <t>rent_roll.units</t>
         </is>
       </c>
-      <c r="F26" s="24" t="inlineStr">
-        <is>
-          <t>New-lease average where a plan has new leases in the window, else in-place. Never a blend.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="21" t="inlineStr">
-        <is>
-          <t>summary.msa</t>
-        </is>
-      </c>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>Derived by the pipeline</t>
-        </is>
-      </c>
-      <c r="C27" s="5" t="inlineStr">
+      <c r="G47" s="23" t="inlineStr">
+        <is>
+          <t>Distinct unit identifiers on the roll.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="22" t="inlineStr">
+        <is>
+          <t>summary.year_built</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>2,019</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>Synthetic offering memorandum</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>p.6</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F48" s="12" t="n"/>
+      <c r="G48" s="24" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="22" t="inlineStr">
+        <is>
+          <t>summary.zip</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>75000</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>Synthetic offering memorandum</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>p.4</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F49" s="12" t="n"/>
+      <c r="G49" s="24" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="22" t="inlineStr">
+        <is>
+          <t>supply.rings</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>12 entries</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>Synthetic public data extract</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D27" s="5" t="inlineStr">
-        <is>
-          <t>derived</t>
-        </is>
-      </c>
-      <c r="E27" s="5" t="inlineStr">
-        <is>
-          <t>summary.city, summary.state</t>
-        </is>
-      </c>
-      <c r="F27" s="24" t="inlineStr">
-        <is>
-          <t>Metro assigned from the city/state pair.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="21" t="inlineStr">
-        <is>
-          <t>summary.pricing_guidance</t>
-        </is>
-      </c>
-      <c r="B28" s="5" t="inlineStr">
-        <is>
-          <t>Supplied by the operator</t>
-        </is>
-      </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D28" s="5" t="inlineStr">
+      <c r="E50" s="5" t="inlineStr">
         <is>
           <t>read</t>
         </is>
       </c>
-      <c r="E28" s="23" t="n"/>
-      <c r="F28" s="24" t="inlineStr">
-        <is>
-          <t>Illustrative figure supplied directly; not a quote or an offer.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="21" t="inlineStr">
-        <is>
-          <t>summary.product_detail</t>
-        </is>
-      </c>
-      <c r="B29" s="5" t="inlineStr">
-        <is>
-          <t>Synthetic offering memorandum</t>
-        </is>
-      </c>
-      <c r="C29" s="5" t="inlineStr">
-        <is>
-          <t>p.7</t>
-        </is>
-      </c>
-      <c r="D29" s="5" t="inlineStr">
-        <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="E29" s="23" t="n"/>
-      <c r="F29" s="22" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="21" t="inlineStr">
-        <is>
-          <t>summary.product_type</t>
-        </is>
-      </c>
-      <c r="B30" s="5" t="inlineStr">
-        <is>
-          <t>Synthetic offering memorandum</t>
-        </is>
-      </c>
-      <c r="C30" s="5" t="inlineStr">
-        <is>
-          <t>p.6</t>
-        </is>
-      </c>
-      <c r="D30" s="5" t="inlineStr">
-        <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="E30" s="23" t="n"/>
-      <c r="F30" s="22" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="21" t="inlineStr">
-        <is>
-          <t>summary.school_elementary_name</t>
-        </is>
-      </c>
-      <c r="B31" s="5" t="inlineStr">
-        <is>
-          <t>Synthetic public data extract</t>
-        </is>
-      </c>
-      <c r="C31" s="5" t="inlineStr">
-        <is>
-          <t>School attendance lookup</t>
-        </is>
-      </c>
-      <c r="D31" s="5" t="inlineStr">
-        <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="E31" s="23" t="n"/>
-      <c r="F31" s="22" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="21" t="inlineStr">
-        <is>
-          <t>summary.school_high_name</t>
-        </is>
-      </c>
-      <c r="B32" s="5" t="inlineStr">
-        <is>
-          <t>Synthetic public data extract</t>
-        </is>
-      </c>
-      <c r="C32" s="5" t="inlineStr">
-        <is>
-          <t>School attendance lookup</t>
-        </is>
-      </c>
-      <c r="D32" s="5" t="inlineStr">
-        <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="E32" s="23" t="n"/>
-      <c r="F32" s="22" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="21" t="inlineStr">
-        <is>
-          <t>summary.school_middle_name</t>
-        </is>
-      </c>
-      <c r="B33" s="5" t="inlineStr">
-        <is>
-          <t>Synthetic public data extract</t>
-        </is>
-      </c>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>School attendance lookup</t>
-        </is>
-      </c>
-      <c r="D33" s="5" t="inlineStr">
-        <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="E33" s="23" t="n"/>
-      <c r="F33" s="22" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="21" t="inlineStr">
-        <is>
-          <t>summary.seller_entity</t>
-        </is>
-      </c>
-      <c r="B34" s="5" t="inlineStr">
-        <is>
-          <t>Synthetic offering memorandum</t>
-        </is>
-      </c>
-      <c r="C34" s="5" t="inlineStr">
-        <is>
-          <t>p.2</t>
-        </is>
-      </c>
-      <c r="D34" s="5" t="inlineStr">
-        <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="E34" s="23" t="n"/>
-      <c r="F34" s="22" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="21" t="inlineStr">
-        <is>
-          <t>summary.state</t>
-        </is>
-      </c>
-      <c r="B35" s="5" t="inlineStr">
-        <is>
-          <t>Synthetic offering memorandum</t>
-        </is>
-      </c>
-      <c r="C35" s="5" t="inlineStr">
-        <is>
-          <t>p.4</t>
-        </is>
-      </c>
-      <c r="D35" s="5" t="inlineStr">
-        <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="E35" s="23" t="n"/>
-      <c r="F35" s="22" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="21" t="inlineStr">
-        <is>
-          <t>summary.street_address</t>
-        </is>
-      </c>
-      <c r="B36" s="5" t="inlineStr">
-        <is>
-          <t>Synthetic offering memorandum</t>
-        </is>
-      </c>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>p.4</t>
-        </is>
-      </c>
-      <c r="D36" s="5" t="inlineStr">
-        <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="E36" s="23" t="n"/>
-      <c r="F36" s="24" t="inlineStr">
-        <is>
-          <t>1400 Example Parkway</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="21" t="inlineStr">
-        <is>
-          <t>summary.structure</t>
-        </is>
-      </c>
-      <c r="B37" s="5" t="inlineStr">
-        <is>
-          <t>Synthetic offering memorandum</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>p.6</t>
-        </is>
-      </c>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="E37" s="23" t="n"/>
-      <c r="F37" s="24" t="inlineStr">
-        <is>
-          <t>Three-story garden, surface parked</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="21" t="inlineStr">
-        <is>
-          <t>summary.tax_area_code</t>
-        </is>
-      </c>
-      <c r="B38" s="5" t="inlineStr">
-        <is>
-          <t>Synthetic county tax record</t>
-        </is>
-      </c>
-      <c r="C38" s="5" t="inlineStr">
-        <is>
-          <t>Rate table</t>
-        </is>
-      </c>
-      <c r="D38" s="5" t="inlineStr">
-        <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="E38" s="23" t="n"/>
-      <c r="F38" s="22" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="21" t="inlineStr">
-        <is>
-          <t>summary.tax_basis_label</t>
-        </is>
-      </c>
-      <c r="B39" s="5" t="inlineStr">
-        <is>
-          <t>Synthetic county tax record</t>
-        </is>
-      </c>
-      <c r="C39" s="5" t="inlineStr">
-        <is>
-          <t>Valuation notice</t>
-        </is>
-      </c>
-      <c r="D39" s="5" t="inlineStr">
-        <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="E39" s="23" t="n"/>
-      <c r="F39" s="22" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="21" t="inlineStr">
-        <is>
-          <t>summary.tax_basis_note</t>
-        </is>
-      </c>
-      <c r="B40" s="5" t="inlineStr">
-        <is>
-          <t>Synthetic county tax record</t>
-        </is>
-      </c>
-      <c r="C40" s="5" t="inlineStr">
-        <is>
-          <t>Valuation notice</t>
-        </is>
-      </c>
-      <c r="D40" s="5" t="inlineStr">
-        <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="E40" s="23" t="n"/>
-      <c r="F40" s="22" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="21" t="inlineStr">
-        <is>
-          <t>summary.tax_billed_amount</t>
-        </is>
-      </c>
-      <c r="B41" s="5" t="inlineStr">
-        <is>
-          <t>Synthetic county tax record</t>
-        </is>
-      </c>
-      <c r="C41" s="5" t="inlineStr">
-        <is>
-          <t>Tax bill</t>
-        </is>
-      </c>
-      <c r="D41" s="5" t="inlineStr">
-        <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="E41" s="23" t="n"/>
-      <c r="F41" s="22" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="21" t="inlineStr">
-        <is>
-          <t>summary.tax_billed_year</t>
-        </is>
-      </c>
-      <c r="B42" s="5" t="inlineStr">
-        <is>
-          <t>Synthetic county tax record</t>
-        </is>
-      </c>
-      <c r="C42" s="5" t="inlineStr">
-        <is>
-          <t>Tax bill</t>
-        </is>
-      </c>
-      <c r="D42" s="5" t="inlineStr">
-        <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="E42" s="23" t="n"/>
-      <c r="F42" s="22" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="21" t="inlineStr">
-        <is>
-          <t>summary.tax_divisor</t>
-        </is>
-      </c>
-      <c r="B43" s="5" t="inlineStr">
-        <is>
-          <t>Synthetic county tax record</t>
-        </is>
-      </c>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t>Rate table</t>
-        </is>
-      </c>
-      <c r="D43" s="5" t="inlineStr">
-        <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="E43" s="23" t="n"/>
-      <c r="F43" s="22" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="21" t="inlineStr">
-        <is>
-          <t>summary.tax_exemption</t>
-        </is>
-      </c>
-      <c r="B44" s="5" t="inlineStr">
-        <is>
-          <t>Synthetic county tax record</t>
-        </is>
-      </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t>Valuation notice</t>
-        </is>
-      </c>
-      <c r="D44" s="5" t="inlineStr">
-        <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="E44" s="23" t="n"/>
-      <c r="F44" s="22" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="21" t="inlineStr">
-        <is>
-          <t>summary.tax_parcel_id</t>
-        </is>
-      </c>
-      <c r="B45" s="5" t="inlineStr">
-        <is>
-          <t>Synthetic county tax record</t>
-        </is>
-      </c>
-      <c r="C45" s="5" t="inlineStr">
-        <is>
-          <t>Parcel record</t>
-        </is>
-      </c>
-      <c r="D45" s="5" t="inlineStr">
-        <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="E45" s="23" t="n"/>
-      <c r="F45" s="22" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="21" t="inlineStr">
-        <is>
-          <t>summary.tax_rate_as_billed</t>
-        </is>
-      </c>
-      <c r="B46" s="5" t="inlineStr">
-        <is>
-          <t>Synthetic county tax record</t>
-        </is>
-      </c>
-      <c r="C46" s="5" t="inlineStr">
-        <is>
-          <t>Rate table, synthetic district</t>
-        </is>
-      </c>
-      <c r="D46" s="5" t="inlineStr">
-        <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="E46" s="23" t="n"/>
-      <c r="F46" s="22" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="21" t="inlineStr">
-        <is>
-          <t>summary.unit_count</t>
-        </is>
-      </c>
-      <c r="B47" s="5" t="inlineStr">
-        <is>
-          <t>Synthetic rent roll export</t>
-        </is>
-      </c>
-      <c r="C47" s="5" t="inlineStr">
-        <is>
-          <t>Rent Roll!A:A</t>
-        </is>
-      </c>
-      <c r="D47" s="5" t="inlineStr">
-        <is>
-          <t>derived</t>
-        </is>
-      </c>
-      <c r="E47" s="5" t="inlineStr">
-        <is>
-          <t>rent_roll.units</t>
-        </is>
-      </c>
-      <c r="F47" s="24" t="inlineStr">
-        <is>
-          <t>Distinct unit identifiers on the roll.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="21" t="inlineStr">
-        <is>
-          <t>summary.year_built</t>
-        </is>
-      </c>
-      <c r="B48" s="5" t="inlineStr">
-        <is>
-          <t>Synthetic offering memorandum</t>
-        </is>
-      </c>
-      <c r="C48" s="5" t="inlineStr">
-        <is>
-          <t>p.6</t>
-        </is>
-      </c>
-      <c r="D48" s="5" t="inlineStr">
-        <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="E48" s="23" t="n"/>
-      <c r="F48" s="22" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="21" t="inlineStr">
-        <is>
-          <t>summary.zip</t>
-        </is>
-      </c>
-      <c r="B49" s="5" t="inlineStr">
-        <is>
-          <t>Synthetic offering memorandum</t>
-        </is>
-      </c>
-      <c r="C49" s="5" t="inlineStr">
-        <is>
-          <t>p.4</t>
-        </is>
-      </c>
-      <c r="D49" s="5" t="inlineStr">
-        <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="E49" s="23" t="n"/>
-      <c r="F49" s="22" t="n"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="21" t="inlineStr">
-        <is>
-          <t>supply.rings</t>
-        </is>
-      </c>
-      <c r="B50" s="5" t="inlineStr">
-        <is>
-          <t>Synthetic public data extract</t>
-        </is>
-      </c>
-      <c r="C50" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D50" s="5" t="inlineStr">
-        <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="E50" s="23" t="n"/>
-      <c r="F50" s="24" t="inlineStr">
+      <c r="F50" s="12" t="n"/>
+      <c r="G50" s="23" t="inlineStr">
         <is>
           <t>Permit and entitlement records.</t>
         </is>

</xml_diff>

<commit_message>
demo: restage the fixture with the comps consistency fixes
Still the synthetic fixture; 505 West stays local. Gate clean against both denylists.

The comps tab now carries the by-bed table, the mix-matched comp rent, the subject rent
restricted to the same bed counts, and mix coverage — and it publishes a spread only when
compute publishes one, showing WITHHELD with compute's own reason otherwise. Previously the
workbook divided a flat average and published a spread the preview was withholding.

npm run build green, 28 pages.
</commit_message>
<xml_diff>
--- a/public/downloads/underwriting-demo/sample-deal-summary.xlsx
+++ b/public/downloads/underwriting-demo/sample-deal-summary.xlsx
@@ -1368,14 +1368,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M21"/>
+  <dimension ref="A1:M30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
@@ -1968,62 +1968,203 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Subject versus comp set</t>
+          <t>By bed count — like for like</t>
         </is>
       </c>
       <c r="B17" s="4" t="n"/>
       <c r="C17" s="4" t="n"/>
+      <c r="D17" s="4" t="n"/>
+      <c r="E17" s="4" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>Subject market rent</t>
-        </is>
-      </c>
-      <c r="B18" s="7" t="n">
-        <v>1834.78</v>
-      </c>
-      <c r="C18" s="6" t="inlineStr">
-        <is>
-          <t>Unit-weighted market rent for model, from the rent-roll analysis.</t>
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>Beds</t>
+        </is>
+      </c>
+      <c r="B18" s="14" t="inlineStr">
+        <is>
+          <t>Communities</t>
+        </is>
+      </c>
+      <c r="C18" s="14" t="inlineStr">
+        <is>
+          <t>Plans</t>
+        </is>
+      </c>
+      <c r="D18" s="14" t="inlineStr">
+        <is>
+          <t>Avg asking</t>
+        </is>
+      </c>
+      <c r="E18" s="14" t="inlineStr">
+        <is>
+          <t>Avg net effective</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
+          <t>1 bed</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="C19" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="D19" s="7" t="n">
+        <v>1480</v>
+      </c>
+      <c r="E19" s="7" t="n">
+        <v>1446.25</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>2 bed</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="C20" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="D20" s="7" t="n">
+        <v>1855</v>
+      </c>
+      <c r="E20" s="7" t="n">
+        <v>1786.25</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>3 bed</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="C21" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D21" s="7" t="n">
+        <v>2262.5</v>
+      </c>
+      <c r="E21" s="7" t="n">
+        <v>2262.5</v>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Subject versus comp set</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="n"/>
+      <c r="C23" s="4" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Subject market rent</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="n">
+        <v>1834.78</v>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>Unit-weighted market rent for model, whole property.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
           <t>Comp-set average asking</t>
         </is>
       </c>
-      <c r="B19" s="7">
+      <c r="B25" s="7">
         <f>IFERROR(AVERAGE(G6:G15),"")</f>
         <v/>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t>Comp-set average net effective</t>
         </is>
       </c>
-      <c r="B20" s="7">
+      <c r="B26" s="7">
         <f>IFERROR(AVERAGE(I6:I15),"")</f>
         <v/>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>Subject vs comp-set net effective</t>
-        </is>
-      </c>
-      <c r="B21" s="11">
-        <f>IFERROR(B18/B20-1,"")</f>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Comp set, mix-matched</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="n">
+        <v>1774.972222222222</v>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>Each bed count's comp net-effective weighted by the subject's own unit mix, so both sides describe the same product.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Subject rent, same bed counts</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="n">
+        <v>1834.777777777778</v>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>Restricted to the bed counts the comp set covers: [1, 2, 3].</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Mix coverage</t>
+        </is>
+      </c>
+      <c r="B29" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>Share of the subject's units actually compared, by bed count and priced plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Subject vs comp set (mix-matched)</t>
+        </is>
+      </c>
+      <c r="B30" s="11">
+        <f>IFERROR(B28/B27-1,"")</f>
         <v/>
       </c>
-      <c r="C21" s="6" t="inlineStr">
-        <is>
-          <t>Positive means the subject is underwritten above the comp set.</t>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>Negative means the subject is underwritten BELOW the market — mark-to-market room rather than a stretch.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
restage the fixture with the three-tier comp display
Comps now render as Top comps / Additional comps / Also nearby. The third tier is
identity only - name, address, distance, units, product, year - with a column
saying why each community is not a comp: wrong product, vintage outside the band,
no quoted rent, excluded by the tracker, or simply beyond the closest twenty.

That last column is the point. "Why isn't the property across the street in your
comp set?" is the first question anyone asks a comp set, and one that cannot answer
it is asking to be trusted rather than read.

Still the synthetic fixture: 11 communities in the detailed tiers, 4 nearby, one of
them carrying no published year so the tier-1 header discloses that the vintage
filter ran only where a year was known.
</commit_message>
<xml_diff>
--- a/public/downloads/underwriting-demo/sample-deal-summary.xlsx
+++ b/public/downloads/underwriting-demo/sample-deal-summary.xlsx
@@ -1368,22 +1368,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M30"/>
+  <dimension ref="A1:N58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
     <col width="42" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="19" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="19" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1418,211 +1419,142 @@
       <c r="H4" s="3" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="14" t="inlineStr">
-        <is>
-          <t>Community</t>
-        </is>
-      </c>
-      <c r="B5" s="14" t="inlineStr">
-        <is>
-          <t>Distance (mi)</t>
-        </is>
-      </c>
-      <c r="C5" s="14" t="inlineStr">
-        <is>
-          <t>Floor plan</t>
-        </is>
-      </c>
-      <c r="D5" s="14" t="inlineStr">
-        <is>
-          <t>Beds</t>
-        </is>
-      </c>
-      <c r="E5" s="14" t="inlineStr">
-        <is>
-          <t>Baths</t>
-        </is>
-      </c>
-      <c r="F5" s="14" t="inlineStr">
-        <is>
-          <t>SF</t>
-        </is>
-      </c>
-      <c r="G5" s="14" t="inlineStr">
-        <is>
-          <t>Asking rent</t>
-        </is>
-      </c>
-      <c r="H5" s="14" t="inlineStr">
-        <is>
-          <t>Concession</t>
-        </is>
-      </c>
-      <c r="I5" s="14" t="inlineStr">
-        <is>
-          <t>Net effective rent</t>
-        </is>
-      </c>
-      <c r="J5" s="14" t="inlineStr">
-        <is>
-          <t>Asking $/SF</t>
-        </is>
-      </c>
-      <c r="K5" s="14" t="inlineStr">
-        <is>
-          <t>Occupancy</t>
-        </is>
-      </c>
-      <c r="L5" s="14" t="inlineStr">
-        <is>
-          <t>As-of date</t>
-        </is>
-      </c>
-      <c r="M5" s="14" t="inlineStr">
-        <is>
-          <t>Source</t>
-        </is>
-      </c>
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Tier 1 — Top comps: the closest 5 communities matching the subject's product and vintage</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n"/>
+      <c r="C5" s="4" t="n"/>
+      <c r="D5" s="4" t="n"/>
+      <c r="E5" s="4" t="n"/>
+      <c r="F5" s="4" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Alderwood Crossing</t>
-        </is>
-      </c>
-      <c r="B6" s="10" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>1BR-A</t>
-        </is>
-      </c>
-      <c r="D6" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="E6" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="F6" s="7" t="n">
-        <v>735</v>
-      </c>
-      <c r="G6" s="7" t="n">
-        <v>1495</v>
-      </c>
-      <c r="H6" s="7" t="n">
-        <v>45</v>
-      </c>
-      <c r="I6" s="7" t="n">
-        <v>1450</v>
-      </c>
-      <c r="J6" s="16">
-        <f>IFERROR(G6/F6,"")</f>
-        <v/>
-      </c>
-      <c r="K6" s="11" t="n">
-        <v>0.9399999999999999</v>
-      </c>
-      <c r="L6" s="17" t="n">
-        <v>46195</v>
-      </c>
-      <c r="M6" s="5" t="inlineStr">
-        <is>
-          <t>own weekly scrape</t>
+          <t>Vintage filter applied where year known: +/-10 years of the subject's year built. 1 of 11 communities shown carry no published year and were matched on distance and product only.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>Alderwood Crossing</t>
-        </is>
-      </c>
-      <c r="B7" s="10" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>2BR-B</t>
-        </is>
-      </c>
-      <c r="D7" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="E7" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="F7" s="7" t="n">
-        <v>1075</v>
-      </c>
-      <c r="G7" s="7" t="n">
-        <v>1835</v>
-      </c>
-      <c r="H7" s="7" t="n">
-        <v>60</v>
-      </c>
-      <c r="I7" s="7" t="n">
-        <v>1775</v>
-      </c>
-      <c r="J7" s="16">
-        <f>IFERROR(G7/F7,"")</f>
-        <v/>
-      </c>
-      <c r="K7" s="11" t="n">
-        <v>0.9399999999999999</v>
-      </c>
-      <c r="L7" s="17" t="n">
-        <v>46195</v>
-      </c>
-      <c r="M7" s="5" t="inlineStr">
-        <is>
-          <t>own weekly scrape</t>
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>Community</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>Distance (mi)</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="inlineStr">
+        <is>
+          <t>Year built</t>
+        </is>
+      </c>
+      <c r="D7" s="14" t="inlineStr">
+        <is>
+          <t>Floor plan</t>
+        </is>
+      </c>
+      <c r="E7" s="14" t="inlineStr">
+        <is>
+          <t>Beds</t>
+        </is>
+      </c>
+      <c r="F7" s="14" t="inlineStr">
+        <is>
+          <t>Baths</t>
+        </is>
+      </c>
+      <c r="G7" s="14" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="H7" s="14" t="inlineStr">
+        <is>
+          <t>Asking rent</t>
+        </is>
+      </c>
+      <c r="I7" s="14" t="inlineStr">
+        <is>
+          <t>Concession</t>
+        </is>
+      </c>
+      <c r="J7" s="14" t="inlineStr">
+        <is>
+          <t>Net effective rent</t>
+        </is>
+      </c>
+      <c r="K7" s="14" t="inlineStr">
+        <is>
+          <t>Asking $/SF</t>
+        </is>
+      </c>
+      <c r="L7" s="14" t="inlineStr">
+        <is>
+          <t>Occupancy</t>
+        </is>
+      </c>
+      <c r="M7" s="14" t="inlineStr">
+        <is>
+          <t>As-of date</t>
+        </is>
+      </c>
+      <c r="N7" s="14" t="inlineStr">
+        <is>
+          <t>Source</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Sable Point</t>
+          <t>Alderwood Crossing</t>
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>A1</t>
-        </is>
-      </c>
-      <c r="D8" s="15" t="n">
-        <v>1</v>
+        <v>0.4</v>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>2021</v>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>1BR-A</t>
+        </is>
       </c>
       <c r="E8" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="F8" s="7" t="n">
-        <v>700</v>
+      <c r="F8" s="15" t="n">
+        <v>1</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>1440</v>
+        <v>735</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>0</v>
+        <v>1450</v>
       </c>
       <c r="I8" s="7" t="n">
-        <v>1440</v>
-      </c>
-      <c r="J8" s="16">
-        <f>IFERROR(G8/F8,"")</f>
+        <v>45</v>
+      </c>
+      <c r="J8" s="7" t="n">
+        <v>1405</v>
+      </c>
+      <c r="K8" s="16">
+        <f>IFERROR(H8/G8,"")</f>
         <v/>
       </c>
-      <c r="K8" s="11" t="n">
-        <v>0.96</v>
-      </c>
-      <c r="L8" s="17" t="n">
+      <c r="L8" s="11" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="M8" s="17" t="n">
         <v>46195</v>
       </c>
-      <c r="M8" s="5" t="inlineStr">
+      <c r="N8" s="5" t="inlineStr">
         <is>
           <t>own weekly scrape</t>
         </is>
@@ -1631,46 +1563,49 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Sable Point</t>
+          <t>Alderwood Crossing</t>
         </is>
       </c>
       <c r="B9" s="10" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>B2</t>
-        </is>
-      </c>
-      <c r="D9" s="15" t="n">
-        <v>2</v>
+        <v>0.4</v>
+      </c>
+      <c r="C9" s="8" t="n">
+        <v>2021</v>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>2BR-B</t>
+        </is>
       </c>
       <c r="E9" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="F9" s="7" t="n">
-        <v>1100</v>
+      <c r="F9" s="15" t="n">
+        <v>2</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>1795</v>
+        <v>1075</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>75</v>
+        <v>1815</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>1720</v>
-      </c>
-      <c r="J9" s="16">
-        <f>IFERROR(G9/F9,"")</f>
+        <v>45</v>
+      </c>
+      <c r="J9" s="7" t="n">
+        <v>1770</v>
+      </c>
+      <c r="K9" s="16">
+        <f>IFERROR(H9/G9,"")</f>
         <v/>
       </c>
-      <c r="K9" s="11" t="n">
+      <c r="L9" s="11" t="n">
         <v>0.9399999999999999</v>
       </c>
-      <c r="L9" s="17" t="n">
+      <c r="M9" s="17" t="n">
         <v>46195</v>
       </c>
-      <c r="M9" s="5" t="inlineStr">
+      <c r="N9" s="5" t="inlineStr">
         <is>
           <t>own weekly scrape</t>
         </is>
@@ -1679,46 +1614,47 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Sable Point</t>
+          <t>Rowan Yard</t>
         </is>
       </c>
       <c r="B10" s="10" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>C1</t>
-        </is>
-      </c>
-      <c r="D10" s="15" t="n">
-        <v>3</v>
+        <v>0.6</v>
+      </c>
+      <c r="C10" s="12" t="n"/>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>1BR-A</t>
+        </is>
       </c>
       <c r="E10" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="F10" s="7" t="n">
-        <v>1355</v>
+        <v>1</v>
+      </c>
+      <c r="F10" s="15" t="n">
+        <v>1</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>2140</v>
+        <v>735</v>
       </c>
       <c r="H10" s="7" t="n">
+        <v>1455</v>
+      </c>
+      <c r="I10" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="I10" s="7" t="n">
-        <v>2140</v>
-      </c>
-      <c r="J10" s="16">
-        <f>IFERROR(G10/F10,"")</f>
+      <c r="J10" s="7" t="n">
+        <v>1455</v>
+      </c>
+      <c r="K10" s="16">
+        <f>IFERROR(H10/G10,"")</f>
         <v/>
       </c>
-      <c r="K10" s="11" t="n">
+      <c r="L10" s="11" t="n">
         <v>0.96</v>
       </c>
-      <c r="L10" s="17" t="n">
+      <c r="M10" s="17" t="n">
         <v>46195</v>
       </c>
-      <c r="M10" s="5" t="inlineStr">
+      <c r="N10" s="5" t="inlineStr">
         <is>
           <t>own weekly scrape</t>
         </is>
@@ -1727,46 +1663,47 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Harper Station</t>
+          <t>Rowan Yard</t>
         </is>
       </c>
       <c r="B11" s="10" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>Aspen</t>
-        </is>
-      </c>
-      <c r="D11" s="15" t="n">
-        <v>1</v>
+        <v>0.6</v>
+      </c>
+      <c r="C11" s="12" t="n"/>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>2BR-B</t>
+        </is>
       </c>
       <c r="E11" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="F11" s="7" t="n">
-        <v>760</v>
+        <v>2</v>
+      </c>
+      <c r="F11" s="15" t="n">
+        <v>2</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>1520</v>
+        <v>1075</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>90</v>
+        <v>1820</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>1430</v>
-      </c>
-      <c r="J11" s="16">
-        <f>IFERROR(G11/F11,"")</f>
+        <v>0</v>
+      </c>
+      <c r="J11" s="7" t="n">
+        <v>1820</v>
+      </c>
+      <c r="K11" s="16">
+        <f>IFERROR(H11/G11,"")</f>
         <v/>
       </c>
-      <c r="K11" s="11" t="n">
-        <v>0.9399999999999999</v>
-      </c>
-      <c r="L11" s="17" t="n">
+      <c r="L11" s="11" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="M11" s="17" t="n">
         <v>46195</v>
       </c>
-      <c r="M11" s="5" t="inlineStr">
+      <c r="N11" s="5" t="inlineStr">
         <is>
           <t>own weekly scrape</t>
         </is>
@@ -1775,46 +1712,49 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Harper Station</t>
+          <t>Sable Point</t>
         </is>
       </c>
       <c r="B12" s="10" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>Birch</t>
-        </is>
-      </c>
-      <c r="D12" s="15" t="n">
-        <v>2</v>
+        <v>0.9</v>
+      </c>
+      <c r="C12" s="8" t="n">
+        <v>2014</v>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>1BR-A</t>
+        </is>
       </c>
       <c r="E12" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="F12" s="7" t="n">
-        <v>1130</v>
+        <v>1</v>
+      </c>
+      <c r="F12" s="15" t="n">
+        <v>1</v>
       </c>
       <c r="G12" s="7" t="n">
-        <v>1880</v>
+        <v>735</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>90</v>
+        <v>1460</v>
       </c>
       <c r="I12" s="7" t="n">
-        <v>1790</v>
-      </c>
-      <c r="J12" s="16">
-        <f>IFERROR(G12/F12,"")</f>
+        <v>45</v>
+      </c>
+      <c r="J12" s="7" t="n">
+        <v>1415</v>
+      </c>
+      <c r="K12" s="16">
+        <f>IFERROR(H12/G12,"")</f>
         <v/>
       </c>
-      <c r="K12" s="11" t="n">
+      <c r="L12" s="11" t="n">
         <v>0.9399999999999999</v>
       </c>
-      <c r="L12" s="17" t="n">
+      <c r="M12" s="17" t="n">
         <v>46195</v>
       </c>
-      <c r="M12" s="5" t="inlineStr">
+      <c r="N12" s="5" t="inlineStr">
         <is>
           <t>own weekly scrape</t>
         </is>
@@ -1823,46 +1763,49 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Kestrel Ridge</t>
+          <t>Sable Point</t>
         </is>
       </c>
       <c r="B13" s="10" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>One Bed</t>
-        </is>
-      </c>
-      <c r="D13" s="15" t="n">
-        <v>1</v>
+        <v>0.9</v>
+      </c>
+      <c r="C13" s="8" t="n">
+        <v>2014</v>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>2BR-B</t>
+        </is>
       </c>
       <c r="E13" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="F13" s="7" t="n">
-        <v>715</v>
+        <v>2</v>
+      </c>
+      <c r="F13" s="15" t="n">
+        <v>2</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>1465</v>
+        <v>1075</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0</v>
+        <v>1825</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>1465</v>
-      </c>
-      <c r="J13" s="16">
-        <f>IFERROR(G13/F13,"")</f>
+        <v>45</v>
+      </c>
+      <c r="J13" s="7" t="n">
+        <v>1780</v>
+      </c>
+      <c r="K13" s="16">
+        <f>IFERROR(H13/G13,"")</f>
         <v/>
       </c>
-      <c r="K13" s="11" t="n">
-        <v>0.96</v>
-      </c>
-      <c r="L13" s="17" t="n">
+      <c r="L13" s="11" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="M13" s="17" t="n">
         <v>46195</v>
       </c>
-      <c r="M13" s="5" t="inlineStr">
+      <c r="N13" s="5" t="inlineStr">
         <is>
           <t>own weekly scrape</t>
         </is>
@@ -1871,46 +1814,49 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Kestrel Ridge</t>
+          <t>Sable Point</t>
         </is>
       </c>
       <c r="B14" s="10" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>Two Bed</t>
-        </is>
-      </c>
-      <c r="D14" s="15" t="n">
-        <v>2</v>
+        <v>0.9</v>
+      </c>
+      <c r="C14" s="8" t="n">
+        <v>2014</v>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>3BR-C</t>
+        </is>
       </c>
       <c r="E14" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="F14" s="15" t="n">
         <v>2.5</v>
       </c>
-      <c r="F14" s="7" t="n">
-        <v>1180</v>
-      </c>
       <c r="G14" s="7" t="n">
-        <v>1910</v>
+        <v>1355</v>
       </c>
       <c r="H14" s="7" t="n">
-        <v>50</v>
+        <v>2180</v>
       </c>
       <c r="I14" s="7" t="n">
-        <v>1860</v>
-      </c>
-      <c r="J14" s="16">
-        <f>IFERROR(G14/F14,"")</f>
+        <v>45</v>
+      </c>
+      <c r="J14" s="7" t="n">
+        <v>2135</v>
+      </c>
+      <c r="K14" s="16">
+        <f>IFERROR(H14/G14,"")</f>
         <v/>
       </c>
-      <c r="K14" s="11" t="n">
+      <c r="L14" s="11" t="n">
         <v>0.9399999999999999</v>
       </c>
-      <c r="L14" s="17" t="n">
+      <c r="M14" s="17" t="n">
         <v>46195</v>
       </c>
-      <c r="M14" s="5" t="inlineStr">
+      <c r="N14" s="5" t="inlineStr">
         <is>
           <t>own weekly scrape</t>
         </is>
@@ -1919,250 +1865,1392 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
+          <t>Harper Station</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="C15" s="8" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>1BR-A</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="7" t="n">
+        <v>735</v>
+      </c>
+      <c r="H15" s="7" t="n">
+        <v>1465</v>
+      </c>
+      <c r="I15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="7" t="n">
+        <v>1465</v>
+      </c>
+      <c r="K15" s="16">
+        <f>IFERROR(H15/G15,"")</f>
+        <v/>
+      </c>
+      <c r="L15" s="11" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="M15" s="17" t="n">
+        <v>46195</v>
+      </c>
+      <c r="N15" s="5" t="inlineStr">
+        <is>
+          <t>own weekly scrape</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Harper Station</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="C16" s="8" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>2BR-B</t>
+        </is>
+      </c>
+      <c r="E16" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="F16" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="G16" s="7" t="n">
+        <v>1075</v>
+      </c>
+      <c r="H16" s="7" t="n">
+        <v>1830</v>
+      </c>
+      <c r="I16" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="7" t="n">
+        <v>1830</v>
+      </c>
+      <c r="K16" s="16">
+        <f>IFERROR(H16/G16,"")</f>
+        <v/>
+      </c>
+      <c r="L16" s="11" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="M16" s="17" t="n">
+        <v>46195</v>
+      </c>
+      <c r="N16" s="5" t="inlineStr">
+        <is>
+          <t>own weekly scrape</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
           <t>Kestrel Ridge</t>
         </is>
       </c>
-      <c r="B15" s="10" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>Three Bed</t>
-        </is>
-      </c>
-      <c r="D15" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="E15" s="15" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="F15" s="7" t="n">
-        <v>1600</v>
-      </c>
-      <c r="G15" s="7" t="n">
-        <v>2385</v>
-      </c>
-      <c r="H15" s="7" t="n">
+      <c r="B17" s="10" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="C17" s="8" t="n">
+        <v>2019</v>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>1BR-A</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" s="7" t="n">
+        <v>735</v>
+      </c>
+      <c r="H17" s="7" t="n">
+        <v>1470</v>
+      </c>
+      <c r="I17" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="J17" s="7" t="n">
+        <v>1425</v>
+      </c>
+      <c r="K17" s="16">
+        <f>IFERROR(H17/G17,"")</f>
+        <v/>
+      </c>
+      <c r="L17" s="11" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="M17" s="17" t="n">
+        <v>46195</v>
+      </c>
+      <c r="N17" s="5" t="inlineStr">
+        <is>
+          <t>own weekly scrape</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Kestrel Ridge</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="C18" s="8" t="n">
+        <v>2019</v>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>2BR-B</t>
+        </is>
+      </c>
+      <c r="E18" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="F18" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="G18" s="7" t="n">
+        <v>1075</v>
+      </c>
+      <c r="H18" s="7" t="n">
+        <v>1835</v>
+      </c>
+      <c r="I18" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="J18" s="7" t="n">
+        <v>1790</v>
+      </c>
+      <c r="K18" s="16">
+        <f>IFERROR(H18/G18,"")</f>
+        <v/>
+      </c>
+      <c r="L18" s="11" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="M18" s="17" t="n">
+        <v>46195</v>
+      </c>
+      <c r="N18" s="5" t="inlineStr">
+        <is>
+          <t>own weekly scrape</t>
+        </is>
+      </c>
+    </row>
+    <row r="19"/>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Tier 2 — Additional comps: the next 6 communities matching the subject's product and vintage</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="n"/>
+      <c r="C20" s="4" t="n"/>
+      <c r="D20" s="4" t="n"/>
+      <c r="E20" s="4" t="n"/>
+      <c r="F20" s="4" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="14" t="inlineStr">
+        <is>
+          <t>Community</t>
+        </is>
+      </c>
+      <c r="B21" s="14" t="inlineStr">
+        <is>
+          <t>Distance (mi)</t>
+        </is>
+      </c>
+      <c r="C21" s="14" t="inlineStr">
+        <is>
+          <t>Year built</t>
+        </is>
+      </c>
+      <c r="D21" s="14" t="inlineStr">
+        <is>
+          <t>Floor plan</t>
+        </is>
+      </c>
+      <c r="E21" s="14" t="inlineStr">
+        <is>
+          <t>Beds</t>
+        </is>
+      </c>
+      <c r="F21" s="14" t="inlineStr">
+        <is>
+          <t>Baths</t>
+        </is>
+      </c>
+      <c r="G21" s="14" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="H21" s="14" t="inlineStr">
+        <is>
+          <t>Asking rent</t>
+        </is>
+      </c>
+      <c r="I21" s="14" t="inlineStr">
+        <is>
+          <t>Concession</t>
+        </is>
+      </c>
+      <c r="J21" s="14" t="inlineStr">
+        <is>
+          <t>Net effective rent</t>
+        </is>
+      </c>
+      <c r="K21" s="14" t="inlineStr">
+        <is>
+          <t>Asking $/SF</t>
+        </is>
+      </c>
+      <c r="L21" s="14" t="inlineStr">
+        <is>
+          <t>Occupancy</t>
+        </is>
+      </c>
+      <c r="M21" s="14" t="inlineStr">
+        <is>
+          <t>As-of date</t>
+        </is>
+      </c>
+      <c r="N21" s="14" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Linden Mill</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C22" s="8" t="n">
+        <v>2011</v>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>1BR-A</t>
+        </is>
+      </c>
+      <c r="E22" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" s="7" t="n">
+        <v>735</v>
+      </c>
+      <c r="H22" s="7" t="n">
+        <v>1475</v>
+      </c>
+      <c r="I22" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="I15" s="7" t="n">
-        <v>2385</v>
-      </c>
-      <c r="J15" s="16">
-        <f>IFERROR(G15/F15,"")</f>
+      <c r="J22" s="7" t="n">
+        <v>1475</v>
+      </c>
+      <c r="K22" s="16">
+        <f>IFERROR(H22/G22,"")</f>
         <v/>
       </c>
-      <c r="K15" s="11" t="n">
+      <c r="L22" s="11" t="n">
         <v>0.96</v>
       </c>
-      <c r="L15" s="17" t="n">
+      <c r="M22" s="17" t="n">
         <v>46195</v>
       </c>
-      <c r="M15" s="5" t="inlineStr">
+      <c r="N22" s="5" t="inlineStr">
         <is>
           <t>own weekly scrape</t>
         </is>
       </c>
     </row>
-    <row r="16"/>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>By bed count — like for like</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="n"/>
-      <c r="C17" s="4" t="n"/>
-      <c r="D17" s="4" t="n"/>
-      <c r="E17" s="4" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="14" t="inlineStr">
-        <is>
-          <t>Beds</t>
-        </is>
-      </c>
-      <c r="B18" s="14" t="inlineStr">
-        <is>
-          <t>Communities</t>
-        </is>
-      </c>
-      <c r="C18" s="14" t="inlineStr">
-        <is>
-          <t>Plans</t>
-        </is>
-      </c>
-      <c r="D18" s="14" t="inlineStr">
-        <is>
-          <t>Avg asking</t>
-        </is>
-      </c>
-      <c r="E18" s="14" t="inlineStr">
-        <is>
-          <t>Avg net effective</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>1 bed</t>
-        </is>
-      </c>
-      <c r="B19" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="C19" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="D19" s="7" t="n">
-        <v>1480</v>
-      </c>
-      <c r="E19" s="7" t="n">
-        <v>1446.25</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>2 bed</t>
-        </is>
-      </c>
-      <c r="B20" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="C20" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="D20" s="7" t="n">
-        <v>1855</v>
-      </c>
-      <c r="E20" s="7" t="n">
-        <v>1786.25</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>3 bed</t>
-        </is>
-      </c>
-      <c r="B21" s="7" t="n">
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Linden Mill</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C23" s="8" t="n">
+        <v>2011</v>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>2BR-B</t>
+        </is>
+      </c>
+      <c r="E23" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="C21" s="7" t="n">
+      <c r="F23" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="D21" s="7" t="n">
-        <v>2262.5</v>
-      </c>
-      <c r="E21" s="7" t="n">
-        <v>2262.5</v>
-      </c>
-    </row>
-    <row r="22"/>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>Subject versus comp set</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="n"/>
-      <c r="C23" s="4" t="n"/>
+      <c r="G23" s="7" t="n">
+        <v>1075</v>
+      </c>
+      <c r="H23" s="7" t="n">
+        <v>1840</v>
+      </c>
+      <c r="I23" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" s="7" t="n">
+        <v>1840</v>
+      </c>
+      <c r="K23" s="16">
+        <f>IFERROR(H23/G23,"")</f>
+        <v/>
+      </c>
+      <c r="L23" s="11" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="M23" s="17" t="n">
+        <v>46195</v>
+      </c>
+      <c r="N23" s="5" t="inlineStr">
+        <is>
+          <t>own weekly scrape</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Subject market rent</t>
-        </is>
-      </c>
-      <c r="B24" s="7" t="n">
-        <v>1834.78</v>
-      </c>
-      <c r="C24" s="6" t="inlineStr">
-        <is>
-          <t>Unit-weighted market rent for model, whole property.</t>
+          <t>Linden Mill</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C24" s="8" t="n">
+        <v>2011</v>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>3BR-C</t>
+        </is>
+      </c>
+      <c r="E24" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="F24" s="15" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G24" s="7" t="n">
+        <v>1355</v>
+      </c>
+      <c r="H24" s="7" t="n">
+        <v>2195</v>
+      </c>
+      <c r="I24" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" s="7" t="n">
+        <v>2195</v>
+      </c>
+      <c r="K24" s="16">
+        <f>IFERROR(H24/G24,"")</f>
+        <v/>
+      </c>
+      <c r="L24" s="11" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="M24" s="17" t="n">
+        <v>46195</v>
+      </c>
+      <c r="N24" s="5" t="inlineStr">
+        <is>
+          <t>own weekly scrape</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>Comp-set average asking</t>
-        </is>
-      </c>
-      <c r="B25" s="7">
-        <f>IFERROR(AVERAGE(G6:G15),"")</f>
+          <t>Pinegate Commons</t>
+        </is>
+      </c>
+      <c r="B25" s="10" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="C25" s="8" t="n">
+        <v>2009</v>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>1BR-A</t>
+        </is>
+      </c>
+      <c r="E25" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" s="7" t="n">
+        <v>735</v>
+      </c>
+      <c r="H25" s="7" t="n">
+        <v>1480</v>
+      </c>
+      <c r="I25" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="J25" s="7" t="n">
+        <v>1435</v>
+      </c>
+      <c r="K25" s="16">
+        <f>IFERROR(H25/G25,"")</f>
         <v/>
+      </c>
+      <c r="L25" s="11" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="M25" s="17" t="n">
+        <v>46195</v>
+      </c>
+      <c r="N25" s="5" t="inlineStr">
+        <is>
+          <t>own weekly scrape</t>
+        </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>Comp-set average net effective</t>
-        </is>
-      </c>
-      <c r="B26" s="7">
-        <f>IFERROR(AVERAGE(I6:I15),"")</f>
+          <t>Pinegate Commons</t>
+        </is>
+      </c>
+      <c r="B26" s="10" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="C26" s="8" t="n">
+        <v>2009</v>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>2BR-B</t>
+        </is>
+      </c>
+      <c r="E26" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="F26" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="G26" s="7" t="n">
+        <v>1075</v>
+      </c>
+      <c r="H26" s="7" t="n">
+        <v>1845</v>
+      </c>
+      <c r="I26" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="J26" s="7" t="n">
+        <v>1800</v>
+      </c>
+      <c r="K26" s="16">
+        <f>IFERROR(H26/G26,"")</f>
         <v/>
+      </c>
+      <c r="L26" s="11" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="M26" s="17" t="n">
+        <v>46195</v>
+      </c>
+      <c r="N26" s="5" t="inlineStr">
+        <is>
+          <t>own weekly scrape</t>
+        </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>Comp set, mix-matched</t>
-        </is>
-      </c>
-      <c r="B27" s="7" t="n">
-        <v>1774.972222222222</v>
-      </c>
-      <c r="C27" s="6" t="inlineStr">
-        <is>
-          <t>Each bed count's comp net-effective weighted by the subject's own unit mix, so both sides describe the same product.</t>
+          <t>Quarry Flats</t>
+        </is>
+      </c>
+      <c r="B27" s="10" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="C27" s="8" t="n">
+        <v>2029</v>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>1BR-A</t>
+        </is>
+      </c>
+      <c r="E27" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F27" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" s="7" t="n">
+        <v>735</v>
+      </c>
+      <c r="H27" s="7" t="n">
+        <v>1485</v>
+      </c>
+      <c r="I27" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" s="7" t="n">
+        <v>1485</v>
+      </c>
+      <c r="K27" s="16">
+        <f>IFERROR(H27/G27,"")</f>
+        <v/>
+      </c>
+      <c r="L27" s="11" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="M27" s="17" t="n">
+        <v>46195</v>
+      </c>
+      <c r="N27" s="5" t="inlineStr">
+        <is>
+          <t>own weekly scrape</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Subject rent, same bed counts</t>
-        </is>
-      </c>
-      <c r="B28" s="7" t="n">
-        <v>1834.777777777778</v>
-      </c>
-      <c r="C28" s="6" t="inlineStr">
-        <is>
-          <t>Restricted to the bed counts the comp set covers: [1, 2, 3].</t>
+          <t>Quarry Flats</t>
+        </is>
+      </c>
+      <c r="B28" s="10" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="C28" s="8" t="n">
+        <v>2029</v>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>2BR-B</t>
+        </is>
+      </c>
+      <c r="E28" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="F28" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="G28" s="7" t="n">
+        <v>1075</v>
+      </c>
+      <c r="H28" s="7" t="n">
+        <v>1850</v>
+      </c>
+      <c r="I28" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" s="7" t="n">
+        <v>1850</v>
+      </c>
+      <c r="K28" s="16">
+        <f>IFERROR(H28/G28,"")</f>
+        <v/>
+      </c>
+      <c r="L28" s="11" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="M28" s="17" t="n">
+        <v>46195</v>
+      </c>
+      <c r="N28" s="5" t="inlineStr">
+        <is>
+          <t>own weekly scrape</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>Mix coverage</t>
-        </is>
-      </c>
-      <c r="B29" s="11" t="n">
+          <t>Marrow Bend</t>
+        </is>
+      </c>
+      <c r="B29" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="C29" s="8" t="n">
+        <v>2028</v>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>1BR-A</t>
+        </is>
+      </c>
+      <c r="E29" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="C29" s="6" t="inlineStr">
-        <is>
-          <t>Share of the subject's units actually compared, by bed count and priced plan.</t>
+      <c r="F29" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G29" s="7" t="n">
+        <v>735</v>
+      </c>
+      <c r="H29" s="7" t="n">
+        <v>1490</v>
+      </c>
+      <c r="I29" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="J29" s="7" t="n">
+        <v>1445</v>
+      </c>
+      <c r="K29" s="16">
+        <f>IFERROR(H29/G29,"")</f>
+        <v/>
+      </c>
+      <c r="L29" s="11" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="M29" s="17" t="n">
+        <v>46195</v>
+      </c>
+      <c r="N29" s="5" t="inlineStr">
+        <is>
+          <t>own weekly scrape</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
+          <t>Marrow Bend</t>
+        </is>
+      </c>
+      <c r="B30" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="C30" s="8" t="n">
+        <v>2028</v>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>2BR-B</t>
+        </is>
+      </c>
+      <c r="E30" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="F30" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="G30" s="7" t="n">
+        <v>1075</v>
+      </c>
+      <c r="H30" s="7" t="n">
+        <v>1855</v>
+      </c>
+      <c r="I30" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="J30" s="7" t="n">
+        <v>1810</v>
+      </c>
+      <c r="K30" s="16">
+        <f>IFERROR(H30/G30,"")</f>
+        <v/>
+      </c>
+      <c r="L30" s="11" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="M30" s="17" t="n">
+        <v>46195</v>
+      </c>
+      <c r="N30" s="5" t="inlineStr">
+        <is>
+          <t>own weekly scrape</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Marrow Bend</t>
+        </is>
+      </c>
+      <c r="B31" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="C31" s="8" t="n">
+        <v>2028</v>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>3BR-C</t>
+        </is>
+      </c>
+      <c r="E31" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="F31" s="15" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G31" s="7" t="n">
+        <v>1355</v>
+      </c>
+      <c r="H31" s="7" t="n">
+        <v>2210</v>
+      </c>
+      <c r="I31" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="J31" s="7" t="n">
+        <v>2165</v>
+      </c>
+      <c r="K31" s="16">
+        <f>IFERROR(H31/G31,"")</f>
+        <v/>
+      </c>
+      <c r="L31" s="11" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="M31" s="17" t="n">
+        <v>46195</v>
+      </c>
+      <c r="N31" s="5" t="inlineStr">
+        <is>
+          <t>own weekly scrape</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>Nyland Court</t>
+        </is>
+      </c>
+      <c r="B32" s="10" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="C32" s="8" t="n">
+        <v>2016</v>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>1BR-A</t>
+        </is>
+      </c>
+      <c r="E32" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F32" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G32" s="7" t="n">
+        <v>735</v>
+      </c>
+      <c r="H32" s="7" t="n">
+        <v>1495</v>
+      </c>
+      <c r="I32" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J32" s="7" t="n">
+        <v>1495</v>
+      </c>
+      <c r="K32" s="16">
+        <f>IFERROR(H32/G32,"")</f>
+        <v/>
+      </c>
+      <c r="L32" s="11" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="M32" s="17" t="n">
+        <v>46195</v>
+      </c>
+      <c r="N32" s="5" t="inlineStr">
+        <is>
+          <t>own weekly scrape</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Nyland Court</t>
+        </is>
+      </c>
+      <c r="B33" s="10" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="C33" s="8" t="n">
+        <v>2016</v>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>2BR-B</t>
+        </is>
+      </c>
+      <c r="E33" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="F33" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="G33" s="7" t="n">
+        <v>1075</v>
+      </c>
+      <c r="H33" s="7" t="n">
+        <v>1860</v>
+      </c>
+      <c r="I33" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J33" s="7" t="n">
+        <v>1860</v>
+      </c>
+      <c r="K33" s="16">
+        <f>IFERROR(H33/G33,"")</f>
+        <v/>
+      </c>
+      <c r="L33" s="11" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="M33" s="17" t="n">
+        <v>46195</v>
+      </c>
+      <c r="N33" s="5" t="inlineStr">
+        <is>
+          <t>own weekly scrape</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Orchard Vale</t>
+        </is>
+      </c>
+      <c r="B34" s="10" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="C34" s="8" t="n">
+        <v>2023</v>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>1BR-A</t>
+        </is>
+      </c>
+      <c r="E34" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F34" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G34" s="7" t="n">
+        <v>735</v>
+      </c>
+      <c r="H34" s="7" t="n">
+        <v>1500</v>
+      </c>
+      <c r="I34" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="J34" s="7" t="n">
+        <v>1455</v>
+      </c>
+      <c r="K34" s="16">
+        <f>IFERROR(H34/G34,"")</f>
+        <v/>
+      </c>
+      <c r="L34" s="11" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="M34" s="17" t="n">
+        <v>46195</v>
+      </c>
+      <c r="N34" s="5" t="inlineStr">
+        <is>
+          <t>own weekly scrape</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Orchard Vale</t>
+        </is>
+      </c>
+      <c r="B35" s="10" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="C35" s="8" t="n">
+        <v>2023</v>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>2BR-B</t>
+        </is>
+      </c>
+      <c r="E35" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="F35" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="G35" s="7" t="n">
+        <v>1075</v>
+      </c>
+      <c r="H35" s="7" t="n">
+        <v>1865</v>
+      </c>
+      <c r="I35" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="J35" s="7" t="n">
+        <v>1820</v>
+      </c>
+      <c r="K35" s="16">
+        <f>IFERROR(H35/G35,"")</f>
+        <v/>
+      </c>
+      <c r="L35" s="11" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="M35" s="17" t="n">
+        <v>46195</v>
+      </c>
+      <c r="N35" s="5" t="inlineStr">
+        <is>
+          <t>own weekly scrape</t>
+        </is>
+      </c>
+    </row>
+    <row r="36"/>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Tier 3 — Also nearby: 4 tracked communities inside the radius that are not comps, and why</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="n"/>
+      <c r="C37" s="4" t="n"/>
+      <c r="D37" s="4" t="n"/>
+      <c r="E37" s="4" t="n"/>
+      <c r="F37" s="4" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Identity only, by design. No rent is shown for these — a rent on a row that did not pass the comp criteria reads as a comp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="14" t="inlineStr">
+        <is>
+          <t>Community</t>
+        </is>
+      </c>
+      <c r="B39" s="14" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="C39" s="14" t="inlineStr">
+        <is>
+          <t>Distance (mi)</t>
+        </is>
+      </c>
+      <c r="D39" s="14" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="E39" s="14" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="F39" s="14" t="inlineStr">
+        <is>
+          <t>Year built</t>
+        </is>
+      </c>
+      <c r="G39" s="14" t="inlineStr">
+        <is>
+          <t>Not a comp because</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Rushmere Townhomes</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>375 Sample Street, Demo City</t>
+        </is>
+      </c>
+      <c r="C40" s="10" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D40" s="7" t="n">
+        <v>96</v>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>bfr</t>
+        </is>
+      </c>
+      <c r="F40" s="8" t="n">
+        <v>2022</v>
+      </c>
+      <c r="G40" s="5" t="inlineStr">
+        <is>
+          <t>different product: tracked as bfr, subject is MF</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Stonecrest Lofts</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>400 Sample Street, Demo City</t>
+        </is>
+      </c>
+      <c r="C41" s="10" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="D41" s="7" t="n">
+        <v>132</v>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>mf</t>
+        </is>
+      </c>
+      <c r="F41" s="8" t="n">
+        <v>1998</v>
+      </c>
+      <c r="G41" s="5" t="inlineStr">
+        <is>
+          <t>vintage 1998 is 21 years from the subject's 2019, outside the +/-10-year band</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Tallow Creek</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>425 Sample Street, Demo City</t>
+        </is>
+      </c>
+      <c r="C42" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" s="7" t="n">
+        <v>144</v>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>mf</t>
+        </is>
+      </c>
+      <c r="F42" s="8" t="n">
+        <v>2018</v>
+      </c>
+      <c r="G42" s="5" t="inlineStr">
+        <is>
+          <t>no quoted rent in the latest scrape of this community</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Underhill Residences</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>450 Sample Street, Demo City</t>
+        </is>
+      </c>
+      <c r="C43" s="10" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="D43" s="7" t="n">
+        <v>88</v>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>mf</t>
+        </is>
+      </c>
+      <c r="F43" s="8" t="n">
+        <v>2020</v>
+      </c>
+      <c r="G43" s="5" t="inlineStr">
+        <is>
+          <t>excluded from comp sets by the tracker: income_restricted</t>
+        </is>
+      </c>
+    </row>
+    <row r="44"/>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>By bed count — like for like</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="n"/>
+      <c r="C45" s="4" t="n"/>
+      <c r="D45" s="4" t="n"/>
+      <c r="E45" s="4" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="14" t="inlineStr">
+        <is>
+          <t>Beds</t>
+        </is>
+      </c>
+      <c r="B46" s="14" t="inlineStr">
+        <is>
+          <t>Communities</t>
+        </is>
+      </c>
+      <c r="C46" s="14" t="inlineStr">
+        <is>
+          <t>Plans</t>
+        </is>
+      </c>
+      <c r="D46" s="14" t="inlineStr">
+        <is>
+          <t>Avg asking</t>
+        </is>
+      </c>
+      <c r="E46" s="14" t="inlineStr">
+        <is>
+          <t>Avg net effective</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>1 bed</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="C47" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="D47" s="7" t="n">
+        <v>1475</v>
+      </c>
+      <c r="E47" s="7" t="n">
+        <v>1450.454545454545</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>2 bed</t>
+        </is>
+      </c>
+      <c r="B48" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="C48" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="D48" s="7" t="n">
+        <v>1840</v>
+      </c>
+      <c r="E48" s="7" t="n">
+        <v>1815.454545454545</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>3 bed</t>
+        </is>
+      </c>
+      <c r="B49" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="C49" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D49" s="7" t="n">
+        <v>2195</v>
+      </c>
+      <c r="E49" s="7" t="n">
+        <v>2165</v>
+      </c>
+    </row>
+    <row r="50"/>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Subject versus comp set — detailed tiers only</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="n"/>
+      <c r="C51" s="4" t="n"/>
+      <c r="D51" s="4" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Subject market rent</t>
+        </is>
+      </c>
+      <c r="B52" s="7" t="n">
+        <v>1834.78</v>
+      </c>
+      <c r="C52" s="6" t="inlineStr">
+        <is>
+          <t>Unit-weighted market rent for model, whole property.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Comp-set average asking</t>
+        </is>
+      </c>
+      <c r="B53" s="7">
+        <f>IFERROR(AVERAGE(H8:H18,H22:H35),"")</f>
+        <v/>
+      </c>
+      <c r="C53" s="6" t="inlineStr">
+        <is>
+          <t>Over 11 communities in the detailed tiers (top 5 plus next 15) — never the whole radius.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Comp-set average net effective</t>
+        </is>
+      </c>
+      <c r="B54" s="7">
+        <f>IFERROR(AVERAGE(J8:J18,J22:J35),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Comp set, mix-matched</t>
+        </is>
+      </c>
+      <c r="B55" s="7" t="n">
+        <v>1767.409090909091</v>
+      </c>
+      <c r="C55" s="6" t="inlineStr">
+        <is>
+          <t>Each bed count's comp net-effective weighted by the subject's own unit mix, so both sides describe the same product.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>Subject rent, same bed counts</t>
+        </is>
+      </c>
+      <c r="B56" s="7" t="n">
+        <v>1834.777777777778</v>
+      </c>
+      <c r="C56" s="6" t="inlineStr">
+        <is>
+          <t>Restricted to the bed counts the comp set covers: [1, 2, 3].</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>Mix coverage</t>
+        </is>
+      </c>
+      <c r="B57" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="C57" s="6" t="inlineStr">
+        <is>
+          <t>Share of the subject's units actually compared, by bed count and priced plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
           <t>Subject vs comp set (mix-matched)</t>
         </is>
       </c>
-      <c r="B30" s="11">
-        <f>IFERROR(B28/B27-1,"")</f>
+      <c r="B58" s="11">
+        <f>IFERROR(B56/B55-1,"")</f>
         <v/>
       </c>
-      <c r="C30" s="6" t="inlineStr">
+      <c r="C58" s="6" t="inlineStr">
         <is>
           <t>Negative means the subject is underwritten BELOW the market — mark-to-market room rather than a stretch.</t>
         </is>
@@ -2771,7 +3859,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H50"/>
+  <dimension ref="A1:H52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2821,7 +3909,7 @@
         </is>
       </c>
       <c r="B5" s="21" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="6">
@@ -2832,7 +3920,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>50/50 (100%)</t>
+          <t>52/52 (100%)</t>
         </is>
       </c>
     </row>
@@ -2950,50 +4038,54 @@
     <row r="11">
       <c r="A11" s="22" t="inlineStr">
         <is>
-          <t>comps.rows</t>
+          <t>comps.nearby</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>10 entries</t>
+          <t>4 entries</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Synthetic weekly rent scrape</t>
+          <t>Tracked-community registry</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>rents.communities within the radius</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="F11" s="12" t="n"/>
+          <t>derived</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>comps.rows.tier</t>
+        </is>
+      </c>
       <c r="G11" s="23" t="inlineStr">
         <is>
-          <t>Own weekly scrape; asking and net effective stated separately.</t>
+          <t>Every tracked community inside the radius that is not a detail row, with the reason it is not. No rent columns.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="22" t="inlineStr">
         <is>
-          <t>demand.rings</t>
+          <t>comps.rows</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>5 entries</t>
+          <t>25 entries</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Synthetic public data extract</t>
+          <t>Synthetic weekly rent scrape</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
@@ -3009,95 +4101,99 @@
       <c r="F12" s="12" t="n"/>
       <c r="G12" s="23" t="inlineStr">
         <is>
-          <t>Ring demographics.</t>
+          <t>Own weekly scrape; asking and net effective stated separately.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="22" t="inlineStr">
         <is>
-          <t>pricing.price_per_unit</t>
+          <t>comps.rows.tier</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>215,000</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Supplied by the operator</t>
+          <t>Tracked-community registry + the scrape</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>comp_tiers.assign</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="F13" s="12" t="n"/>
+          <t>derived</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>comps.rows.distance_mi, comps.tiering.subject_product, comps.tiering.subject_year_built, comps.tiering.year_band, comps.tiering.top_n, comps.tiering.additional_n</t>
+        </is>
+      </c>
       <c r="G13" s="23" t="inlineStr">
         <is>
-          <t>Illustrative. Inside the band a per-unit sale price occupies.</t>
+          <t>Tier 1 = the closest 5 matching product and vintage; tier 2 = the next 15; everything else is tier 3, identity only. An unknown year does not disqualify — it is disclosed on the tier header instead.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="22" t="inlineStr">
         <is>
-          <t>pricing.unit_count</t>
+          <t>demand.rings</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>5 entries</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Synthetic rent roll export</t>
+          <t>Synthetic public data extract</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Rent Roll!A:A</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>derived</t>
-        </is>
-      </c>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t>summary.unit_count</t>
-        </is>
-      </c>
-      <c r="G14" s="24" t="n"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F14" s="12" t="n"/>
+      <c r="G14" s="23" t="inlineStr">
+        <is>
+          <t>Ring demographics.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="22" t="inlineStr">
         <is>
-          <t>summary.assessed_value_basis</t>
+          <t>pricing.price_per_unit</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>23,000,000</t>
+          <t>215,000</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Synthetic county tax record</t>
+          <t>Supplied by the operator</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Valuation notice</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
@@ -3106,56 +4202,64 @@
         </is>
       </c>
       <c r="F15" s="12" t="n"/>
-      <c r="G15" s="24" t="n"/>
+      <c r="G15" s="23" t="inlineStr">
+        <is>
+          <t>Illustrative. Inside the band a per-unit sale price occupies.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="22" t="inlineStr">
         <is>
-          <t>summary.assessment_ratio</t>
+          <t>pricing.unit_count</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>180</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Synthetic county tax record</t>
+          <t>Synthetic rent roll export</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Rate table</t>
+          <t>Rent Roll!A:A</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="F16" s="12" t="n"/>
+          <t>derived</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>summary.unit_count</t>
+        </is>
+      </c>
       <c r="G16" s="24" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="22" t="inlineStr">
         <is>
-          <t>summary.city</t>
+          <t>summary.assessed_value_basis</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Sample City</t>
+          <t>23,000,000</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Synthetic offering memorandum</t>
+          <t>Synthetic county tax record</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>p.4</t>
+          <t>Valuation notice</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -3169,22 +4273,22 @@
     <row r="18">
       <c r="A18" s="22" t="inlineStr">
         <is>
-          <t>summary.construction_status</t>
+          <t>summary.assessment_ratio</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Stabilized</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Synthetic offering memorandum</t>
+          <t>Synthetic county tax record</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>p.6</t>
+          <t>Rate table</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -3198,12 +4302,12 @@
     <row r="19">
       <c r="A19" s="22" t="inlineStr">
         <is>
-          <t>summary.county</t>
+          <t>summary.city</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Example County</t>
+          <t>Sample City</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
@@ -3227,12 +4331,12 @@
     <row r="20">
       <c r="A20" s="22" t="inlineStr">
         <is>
-          <t>summary.deal_name</t>
+          <t>summary.construction_status</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Fixture Park</t>
+          <t>Stabilized</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
@@ -3242,7 +4346,7 @@
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>p.1</t>
+          <t>p.6</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -3251,21 +4355,17 @@
         </is>
       </c>
       <c r="F20" s="12" t="n"/>
-      <c r="G20" s="23" t="inlineStr">
-        <is>
-          <t>Fixture Park</t>
-        </is>
-      </c>
+      <c r="G20" s="24" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="22" t="inlineStr">
         <is>
-          <t>summary.deal_status</t>
+          <t>summary.county</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>On the market</t>
+          <t>Example County</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
@@ -3275,7 +4375,7 @@
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>p.2</t>
+          <t>p.4</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
@@ -3289,12 +4389,12 @@
     <row r="22">
       <c r="A22" s="22" t="inlineStr">
         <is>
-          <t>summary.delivery_date</t>
+          <t>summary.deal_name</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Delivered 2019; fully stabilized since 2021</t>
+          <t>Fixture Park</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
@@ -3304,7 +4404,7 @@
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>p.6</t>
+          <t>p.1</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -3313,27 +4413,31 @@
         </is>
       </c>
       <c r="F22" s="12" t="n"/>
-      <c r="G22" s="24" t="n"/>
+      <c r="G22" s="23" t="inlineStr">
+        <is>
+          <t>Fixture Park</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="22" t="inlineStr">
         <is>
-          <t>summary.fair_market_value</t>
+          <t>summary.deal_status</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>39,600,000</t>
+          <t>On the market</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Supplied by the operator</t>
+          <t>Synthetic offering memorandum</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>p.2</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
@@ -3342,63 +4446,51 @@
         </is>
       </c>
       <c r="F23" s="12" t="n"/>
-      <c r="G23" s="23" t="inlineStr">
-        <is>
-          <t>Operator's own estimate.</t>
-        </is>
-      </c>
+      <c r="G23" s="24" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="22" t="inlineStr">
         <is>
-          <t>summary.in_place_rent_avg</t>
+          <t>summary.delivery_date</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>1,795.36</t>
+          <t>Delivered 2019; fully stabilized since 2021</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Derived by the pipeline</t>
+          <t>Synthetic offering memorandum</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Unit Mix Summary!E</t>
+          <t>p.6</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>computed</t>
-        </is>
-      </c>
-      <c r="F24" s="5" t="inlineStr">
-        <is>
-          <t>rent_roll.units</t>
-        </is>
-      </c>
-      <c r="G24" s="23" t="inlineStr">
-        <is>
-          <t>Occupied units, straight off the roll.</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F24" s="12" t="n"/>
+      <c r="G24" s="24" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="22" t="inlineStr">
         <is>
-          <t>summary.listing_brokerage</t>
+          <t>summary.fair_market_value</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Listing brokerage</t>
+          <t>39,600,000</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Derived by the pipeline</t>
+          <t>Supplied by the operator</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
@@ -3408,29 +4500,25 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>derived</t>
-        </is>
-      </c>
-      <c r="F25" s="5" t="inlineStr">
-        <is>
-          <t>summary.seller_entity</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F25" s="12" t="n"/>
       <c r="G25" s="23" t="inlineStr">
         <is>
-          <t>Generic label; no firm or individual is named in a published file.</t>
+          <t>Operator's own estimate.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="22" t="inlineStr">
         <is>
-          <t>summary.market_rent_for_model</t>
+          <t>summary.in_place_rent_avg</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>1,834.78</t>
+          <t>1,795.36</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
@@ -3440,7 +4528,7 @@
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Unit Mix Summary!H</t>
+          <t>Unit Mix Summary!E</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -3455,19 +4543,19 @@
       </c>
       <c r="G26" s="23" t="inlineStr">
         <is>
-          <t>New-lease average where a plan has new leases in the window, else in-place. Never a blend.</t>
+          <t>Occupied units, straight off the roll.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="22" t="inlineStr">
         <is>
-          <t>summary.msa</t>
+          <t>summary.listing_brokerage</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Sample City MSA</t>
+          <t>Listing brokerage</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
@@ -3487,96 +4575,108 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>summary.city, summary.state</t>
+          <t>summary.seller_entity</t>
         </is>
       </c>
       <c r="G27" s="23" t="inlineStr">
         <is>
-          <t>Metro assigned from the city/state pair.</t>
+          <t>Generic label; no firm or individual is named in a published file.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="22" t="inlineStr">
         <is>
-          <t>summary.pricing_guidance</t>
+          <t>summary.market_rent_for_model</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>$215,000 per unit (illustrative)</t>
+          <t>1,834.78</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Supplied by the operator</t>
+          <t>Derived by the pipeline</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Unit Mix Summary!H</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="F28" s="12" t="n"/>
+          <t>computed</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>rent_roll.units</t>
+        </is>
+      </c>
       <c r="G28" s="23" t="inlineStr">
         <is>
-          <t>Illustrative figure supplied directly; not a quote or an offer.</t>
+          <t>New-lease average where a plan has new leases in the window, else in-place. Never a blend.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="22" t="inlineStr">
         <is>
-          <t>summary.product_detail</t>
+          <t>summary.msa</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>180 units across six plans: 62 one-bedroom (720–795 SF), 78 two-bedroom (1,050–1,140 SF…</t>
+          <t>Sample City MSA</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Synthetic offering memorandum</t>
+          <t>Derived by the pipeline</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>p.7</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="F29" s="12" t="n"/>
-      <c r="G29" s="24" t="n"/>
+          <t>derived</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>summary.city, summary.state</t>
+        </is>
+      </c>
+      <c r="G29" s="23" t="inlineStr">
+        <is>
+          <t>Metro assigned from the city/state pair.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="22" t="inlineStr">
         <is>
-          <t>summary.product_type</t>
+          <t>summary.pricing_guidance</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>MF</t>
+          <t>$215,000 per unit (illustrative)</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>Synthetic offering memorandum</t>
+          <t>Supplied by the operator</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>p.6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -3585,27 +4685,31 @@
         </is>
       </c>
       <c r="F30" s="12" t="n"/>
-      <c r="G30" s="24" t="n"/>
+      <c r="G30" s="23" t="inlineStr">
+        <is>
+          <t>Illustrative figure supplied directly; not a quote or an offer.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="22" t="inlineStr">
         <is>
-          <t>summary.school_elementary_name</t>
+          <t>summary.product_detail</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Example Creek Elementary</t>
+          <t>180 units across six plans: 62 one-bedroom (720–795 SF), 78 two-bedroom (1,050–1,140 SF…</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Synthetic public data extract</t>
+          <t>Synthetic offering memorandum</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>School attendance lookup</t>
+          <t>p.7</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
@@ -3619,22 +4723,22 @@
     <row r="32">
       <c r="A32" s="22" t="inlineStr">
         <is>
-          <t>summary.school_high_name</t>
+          <t>summary.product_type</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Sample City High</t>
+          <t>MF</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>Synthetic public data extract</t>
+          <t>Synthetic offering memorandum</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>School attendance lookup</t>
+          <t>p.6</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -3648,12 +4752,12 @@
     <row r="33">
       <c r="A33" s="22" t="inlineStr">
         <is>
-          <t>summary.school_middle_name</t>
+          <t>summary.school_elementary_name</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>Example Ridge Middle</t>
+          <t>Example Creek Elementary</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
@@ -3677,22 +4781,22 @@
     <row r="34">
       <c r="A34" s="22" t="inlineStr">
         <is>
-          <t>summary.seller_entity</t>
+          <t>summary.school_high_name</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>Sample City Residential Holdings LLC</t>
+          <t>Sample City High</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>Synthetic offering memorandum</t>
+          <t>Synthetic public data extract</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>p.2</t>
+          <t>School attendance lookup</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -3706,22 +4810,22 @@
     <row r="35">
       <c r="A35" s="22" t="inlineStr">
         <is>
-          <t>summary.state</t>
+          <t>summary.school_middle_name</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>Example Ridge Middle</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Synthetic offering memorandum</t>
+          <t>Synthetic public data extract</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>p.4</t>
+          <t>School attendance lookup</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
@@ -3735,12 +4839,12 @@
     <row r="36">
       <c r="A36" s="22" t="inlineStr">
         <is>
-          <t>summary.street_address</t>
+          <t>summary.seller_entity</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>1400 Example Parkway</t>
+          <t>Sample City Residential Holdings LLC</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
@@ -3750,7 +4854,7 @@
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>p.4</t>
+          <t>p.2</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -3759,21 +4863,17 @@
         </is>
       </c>
       <c r="F36" s="12" t="n"/>
-      <c r="G36" s="23" t="inlineStr">
-        <is>
-          <t>1400 Example Parkway</t>
-        </is>
-      </c>
+      <c r="G36" s="24" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="22" t="inlineStr">
         <is>
-          <t>summary.structure</t>
+          <t>summary.state</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>Three-story garden, surface parked</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
@@ -3783,7 +4883,7 @@
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>p.6</t>
+          <t>p.4</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
@@ -3792,31 +4892,27 @@
         </is>
       </c>
       <c r="F37" s="12" t="n"/>
-      <c r="G37" s="23" t="inlineStr">
-        <is>
-          <t>Three-story garden, surface parked</t>
-        </is>
-      </c>
+      <c r="G37" s="24" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="22" t="inlineStr">
         <is>
-          <t>summary.tax_area_code</t>
+          <t>summary.street_address</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>SYN-0000</t>
+          <t>1400 Example Parkway</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>Synthetic county tax record</t>
+          <t>Synthetic offering memorandum</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>Rate table</t>
+          <t>p.4</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
@@ -3825,27 +4921,31 @@
         </is>
       </c>
       <c r="F38" s="12" t="n"/>
-      <c r="G38" s="24" t="n"/>
+      <c r="G38" s="23" t="inlineStr">
+        <is>
+          <t>1400 Example Parkway</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="22" t="inlineStr">
         <is>
-          <t>summary.tax_basis_label</t>
+          <t>summary.structure</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>Assessed value (synthetic)</t>
+          <t>Three-story garden, surface parked</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Synthetic county tax record</t>
+          <t>Synthetic offering memorandum</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>Valuation notice</t>
+          <t>p.6</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
@@ -3854,17 +4954,21 @@
         </is>
       </c>
       <c r="F39" s="12" t="n"/>
-      <c r="G39" s="24" t="n"/>
+      <c r="G39" s="23" t="inlineStr">
+        <is>
+          <t>Three-story garden, surface parked</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="22" t="inlineStr">
         <is>
-          <t>summary.tax_basis_note</t>
+          <t>summary.tax_area_code</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>Synthetic basis. On a real deal this row states what the basis IS in that state and whe…</t>
+          <t>SYN-0000</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
@@ -3874,7 +4978,7 @@
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>Valuation notice</t>
+          <t>Rate table</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -3888,12 +4992,12 @@
     <row r="41">
       <c r="A41" s="22" t="inlineStr">
         <is>
-          <t>summary.tax_billed_amount</t>
+          <t>summary.tax_basis_label</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>494,040</t>
+          <t>Assessed value (synthetic)</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
@@ -3903,7 +5007,7 @@
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>Tax bill</t>
+          <t>Valuation notice</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
@@ -3917,12 +5021,12 @@
     <row r="42">
       <c r="A42" s="22" t="inlineStr">
         <is>
-          <t>summary.tax_billed_year</t>
+          <t>summary.tax_basis_note</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>2,025</t>
+          <t>Synthetic basis. On a real deal this row states what the basis IS in that state and whe…</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
@@ -3932,7 +5036,7 @@
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>Tax bill</t>
+          <t>Valuation notice</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
@@ -3946,12 +5050,12 @@
     <row r="43">
       <c r="A43" s="22" t="inlineStr">
         <is>
-          <t>summary.tax_divisor</t>
+          <t>summary.tax_billed_amount</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>494,040</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
@@ -3961,7 +5065,7 @@
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>Rate table</t>
+          <t>Tax bill</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
@@ -3975,12 +5079,12 @@
     <row r="44">
       <c r="A44" s="22" t="inlineStr">
         <is>
-          <t>summary.tax_exemption</t>
+          <t>summary.tax_billed_year</t>
         </is>
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2,025</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
@@ -3990,7 +5094,7 @@
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>Valuation notice</t>
+          <t>Tax bill</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
@@ -4004,12 +5108,12 @@
     <row r="45">
       <c r="A45" s="22" t="inlineStr">
         <is>
-          <t>summary.tax_parcel_id</t>
+          <t>summary.tax_divisor</t>
         </is>
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>SYN-000-00-000</t>
+          <t>100</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
@@ -4019,7 +5123,7 @@
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>Parcel record</t>
+          <t>Rate table</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
@@ -4033,12 +5137,12 @@
     <row r="46">
       <c r="A46" s="22" t="inlineStr">
         <is>
-          <t>summary.tax_rate_as_billed</t>
+          <t>summary.tax_exemption</t>
         </is>
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>2.15</t>
+          <t>0</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
@@ -4048,7 +5152,7 @@
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>Rate table, synthetic district</t>
+          <t>Valuation notice</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
@@ -4062,59 +5166,51 @@
     <row r="47">
       <c r="A47" s="22" t="inlineStr">
         <is>
-          <t>summary.unit_count</t>
+          <t>summary.tax_parcel_id</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>SYN-000-00-000</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Synthetic rent roll export</t>
+          <t>Synthetic county tax record</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>Rent Roll!A:A</t>
+          <t>Parcel record</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t>derived</t>
-        </is>
-      </c>
-      <c r="F47" s="5" t="inlineStr">
-        <is>
-          <t>rent_roll.units</t>
-        </is>
-      </c>
-      <c r="G47" s="23" t="inlineStr">
-        <is>
-          <t>Distinct unit identifiers on the roll.</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F47" s="12" t="n"/>
+      <c r="G47" s="24" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="22" t="inlineStr">
         <is>
-          <t>summary.year_built</t>
+          <t>summary.tax_rate_as_billed</t>
         </is>
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>2,019</t>
+          <t>2.15</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>Synthetic offering memorandum</t>
+          <t>Synthetic county tax record</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>p.6</t>
+          <t>Rate table, synthetic district</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
@@ -4128,60 +5224,126 @@
     <row r="49">
       <c r="A49" s="22" t="inlineStr">
         <is>
-          <t>summary.zip</t>
+          <t>summary.unit_count</t>
         </is>
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>75000</t>
+          <t>180</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>Synthetic offering memorandum</t>
+          <t>Synthetic rent roll export</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>p.4</t>
+          <t>Rent Roll!A:A</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="F49" s="12" t="n"/>
-      <c r="G49" s="24" t="n"/>
+          <t>derived</t>
+        </is>
+      </c>
+      <c r="F49" s="5" t="inlineStr">
+        <is>
+          <t>rent_roll.units</t>
+        </is>
+      </c>
+      <c r="G49" s="23" t="inlineStr">
+        <is>
+          <t>Distinct unit identifiers on the roll.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="22" t="inlineStr">
         <is>
+          <t>summary.year_built</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>2,019</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>Synthetic offering memorandum</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>p.6</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F50" s="12" t="n"/>
+      <c r="G50" s="24" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="22" t="inlineStr">
+        <is>
+          <t>summary.zip</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>75000</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>Synthetic offering memorandum</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>p.4</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F51" s="12" t="n"/>
+      <c r="G51" s="24" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="22" t="inlineStr">
+        <is>
           <t>supply.rings</t>
         </is>
       </c>
-      <c r="B50" s="5" t="inlineStr">
+      <c r="B52" s="5" t="inlineStr">
         <is>
           <t>12 entries</t>
         </is>
       </c>
-      <c r="C50" s="5" t="inlineStr">
+      <c r="C52" s="5" t="inlineStr">
         <is>
           <t>Synthetic public data extract</t>
         </is>
       </c>
-      <c r="D50" s="5" t="inlineStr">
+      <c r="D52" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E50" s="5" t="inlineStr">
+      <c r="E52" s="5" t="inlineStr">
         <is>
           <t>read</t>
         </is>
       </c>
-      <c r="F50" s="12" t="n"/>
-      <c r="G50" s="23" t="inlineStr">
+      <c r="F52" s="12" t="n"/>
+      <c r="G52" s="23" t="inlineStr">
         <is>
           <t>Permit and entitlement records.</t>
         </is>

</xml_diff>

<commit_message>
restage the fixture: property tax, notes, and the full demand report
Two new tabs (Property tax, Notes & disclosures) and demand expanded from a five-row
ring table to the complete seven-column, seven-section report the engine produces -
including the two sections that do not share the ring geometry: ZIP home value, which
is one figure and not seven, and the metro labor history, which is a year-by-year
table.

The 1-mile column carries its overcount caveat above the data on every surface. It is
a known limit of the engine, and a reader of a published page has no other way to
know.

Provenance now renders beside each value as a muted line, not only in the audit-trail
tab. The trail tab stays as the complete registry.

Still the synthetic fixture set - the guard checks outputs/fixture/deal_outputs.json
and would refuse anything else.
</commit_message>
<xml_diff>
--- a/public/downloads/underwriting-demo/sample-deal-summary.xlsx
+++ b/public/downloads/underwriting-demo/sample-deal-summary.xlsx
@@ -9,9 +9,11 @@
   <sheets>
     <sheet name="Deal Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Rent Comps" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Demand" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Supply" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Audit Trail" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Property Tax" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Demand" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Supply" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Notes &amp; Disclosures" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Audit Trail" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,12 +22,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="#,##0.0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
     <numFmt numFmtId="167" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="168" formatCode="mm/dd/yyyy"/>
+    <numFmt numFmtId="169" formatCode="0.00&quot;x&quot;"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -66,7 +69,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -81,11 +84,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9D9D9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -120,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -143,14 +141,12 @@
     <xf numFmtId="166" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -578,6 +574,11 @@
           <t>Fixture Park</t>
         </is>
       </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>Synthetic offering memorandum — p.1</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -590,6 +591,11 @@
           <t>1400 Example Parkway</t>
         </is>
       </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Synthetic offering memorandum — p.4</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -602,6 +608,11 @@
           <t>Sample City</t>
         </is>
       </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>Synthetic offering memorandum — p.4</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -614,6 +625,11 @@
           <t>TX</t>
         </is>
       </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Synthetic offering memorandum — p.4</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -626,6 +642,11 @@
           <t>75000</t>
         </is>
       </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>Synthetic offering memorandum — p.4</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -638,6 +659,11 @@
           <t>Example County</t>
         </is>
       </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>Synthetic offering memorandum — p.4</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -650,6 +676,11 @@
           <t>Sample City MSA</t>
         </is>
       </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>Derived by the pipeline (derived)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -688,6 +719,11 @@
           <t>MF</t>
         </is>
       </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>Synthetic offering memorandum — p.6</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -700,6 +736,11 @@
           <t>Three-story garden, surface parked</t>
         </is>
       </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>Synthetic offering memorandum — p.6</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -715,6 +756,11 @@
           <t>Divisor for every per-unit figure in the output set.</t>
         </is>
       </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>Synthetic rent roll export — Rent Roll!A:A (derived)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -725,6 +771,11 @@
       <c r="B19" s="8" t="n">
         <v>2019</v>
       </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>Synthetic offering memorandum — p.6</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -737,6 +788,11 @@
           <t>180 units across six plans: 62 one-bedroom (720–795 SF), 78 two-bedroom (1,050–1,140 SF), 26 three-bedroom flats (1,380 SF), 14 three-bedroom townhomes (1,620 SF). Washer/dryer in unit; detached garages on 24 units.</t>
         </is>
       </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>Synthetic offering memorandum — p.7</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -749,6 +805,11 @@
           <t>Stabilized</t>
         </is>
       </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>Synthetic offering memorandum — p.6</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
@@ -761,6 +822,11 @@
           <t>Delivered 2019; fully stabilized since 2021</t>
         </is>
       </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>Synthetic offering memorandum — p.6</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -782,6 +848,11 @@
           <t>Sample City Residential Holdings LLC</t>
         </is>
       </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>Synthetic offering memorandum — p.2</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
@@ -794,6 +865,11 @@
           <t>Listing brokerage</t>
         </is>
       </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>Derived by the pipeline (derived)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
@@ -806,6 +882,11 @@
           <t>On the market</t>
         </is>
       </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>Synthetic offering memorandum — p.2</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -825,6 +906,11 @@
       <c r="B30" s="5" t="inlineStr">
         <is>
           <t>$215,000 per unit (illustrative)</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>Supplied by the operator</t>
         </is>
       </c>
     </row>
@@ -940,6 +1026,11 @@
       <c r="B40" s="7" t="n">
         <v>1795.36</v>
       </c>
+      <c r="D40" s="6" t="inlineStr">
+        <is>
+          <t>Derived by the pipeline — Unit Mix Summary!E (computed)</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
@@ -955,6 +1046,11 @@
           <t>New-lease average where the plan has new leases in the lookback window, otherwise in-place. Never a blend of new and renewal.</t>
         </is>
       </c>
+      <c r="D41" s="6" t="inlineStr">
+        <is>
+          <t>Derived by the pipeline — Unit Mix Summary!H (computed)</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
@@ -965,6 +1061,11 @@
       <c r="B42" s="7" t="n">
         <v>39600000</v>
       </c>
+      <c r="D42" s="6" t="inlineStr">
+        <is>
+          <t>Supplied by the operator</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
@@ -989,6 +1090,11 @@
           <t>Rate as actually billed — not a statutory or effective rate.</t>
         </is>
       </c>
+      <c r="D45" s="6" t="inlineStr">
+        <is>
+          <t>Synthetic county tax record — Rate table, synthetic district</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
@@ -999,6 +1105,11 @@
       <c r="B46" s="7" t="n">
         <v>23000000</v>
       </c>
+      <c r="D46" s="6" t="inlineStr">
+        <is>
+          <t>Synthetic county tax record — Valuation notice</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
@@ -1009,6 +1120,11 @@
       <c r="B47" s="11" t="n">
         <v>1</v>
       </c>
+      <c r="D47" s="6" t="inlineStr">
+        <is>
+          <t>Synthetic county tax record — Rate table</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
@@ -1019,6 +1135,11 @@
       <c r="B48" s="7" t="n">
         <v>100</v>
       </c>
+      <c r="D48" s="6" t="inlineStr">
+        <is>
+          <t>Synthetic county tax record — Rate table</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
@@ -1028,6 +1149,11 @@
       </c>
       <c r="B49" s="7" t="n">
         <v>0</v>
+      </c>
+      <c r="D49" s="6" t="inlineStr">
+        <is>
+          <t>Synthetic county tax record — Valuation notice</t>
+        </is>
       </c>
     </row>
     <row r="50">
@@ -1224,6 +1350,11 @@
           <t>Example Creek Elementary</t>
         </is>
       </c>
+      <c r="D65" s="6" t="inlineStr">
+        <is>
+          <t>Synthetic public data extract — School attendance lookup</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
@@ -1246,6 +1377,11 @@
           <t>Example Ridge Middle</t>
         </is>
       </c>
+      <c r="D67" s="6" t="inlineStr">
+        <is>
+          <t>Synthetic public data extract — School attendance lookup</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="5" t="inlineStr">
@@ -1266,6 +1402,11 @@
       <c r="B69" s="5" t="inlineStr">
         <is>
           <t>Sample City High</t>
+        </is>
+      </c>
+      <c r="D69" s="6" t="inlineStr">
+        <is>
+          <t>Synthetic public data extract — School attendance lookup</t>
         </is>
       </c>
     </row>
@@ -3267,22 +3408,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Demand</t>
+          <t>Property tax</t>
         </is>
       </c>
     </row>
@@ -3296,7 +3434,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Summary table by drive-ring. Public demographic data.</t>
+          <t>Rates as actually billed, not statutory or effective. The current-year block is checked against the county's own bill; the assumption block is what a buyer should carry at the illustrative price.</t>
         </is>
       </c>
     </row>
@@ -3311,165 +3449,397 @@
       <c r="H4" s="3" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="14" t="inlineStr">
-        <is>
-          <t>Ring</t>
-        </is>
-      </c>
-      <c r="B5" s="14" t="inlineStr">
-        <is>
-          <t>Population</t>
-        </is>
-      </c>
-      <c r="C5" s="14" t="inlineStr">
-        <is>
-          <t>Households</t>
-        </is>
-      </c>
-      <c r="D5" s="14" t="inlineStr">
-        <is>
-          <t>Median household income</t>
-        </is>
-      </c>
-      <c r="E5" s="14" t="inlineStr">
-        <is>
-          <t>Total jobs</t>
-        </is>
-      </c>
-      <c r="F5" s="14" t="inlineStr">
-        <is>
-          <t>Population growth (5-yr)</t>
-        </is>
-      </c>
-      <c r="G5" s="14" t="inlineStr">
-        <is>
-          <t>Renter share</t>
-        </is>
-      </c>
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>The rate, as billed</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n"/>
+      <c r="C5" s="4" t="n"/>
+      <c r="D5" s="4" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>1 mi</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="n">
-        <v>9840</v>
-      </c>
-      <c r="C6" s="7" t="n">
-        <v>4020</v>
-      </c>
-      <c r="D6" s="7" t="n">
-        <v>78400</v>
-      </c>
-      <c r="E6" s="7" t="n">
-        <v>3150</v>
-      </c>
-      <c r="F6" s="11" t="n">
-        <v>0.061</v>
-      </c>
-      <c r="G6" s="11" t="n">
-        <v>0.44</v>
+          <t>Parcel</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>SYN-000-00-000</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>Synthetic county tax record — Parcel record</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>3 mi</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="n">
-        <v>61250</v>
-      </c>
-      <c r="C7" s="7" t="n">
-        <v>24100</v>
-      </c>
-      <c r="D7" s="7" t="n">
-        <v>84900</v>
-      </c>
-      <c r="E7" s="7" t="n">
-        <v>27400</v>
-      </c>
-      <c r="F7" s="11" t="n">
-        <v>0.078</v>
-      </c>
-      <c r="G7" s="11" t="n">
-        <v>0.39</v>
+          <t>Tax area code</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>SYN-0000</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Synthetic county tax record — Rate table</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>5 mi</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="n">
-        <v>148300</v>
-      </c>
-      <c r="C8" s="7" t="n">
-        <v>57600</v>
-      </c>
-      <c r="D8" s="7" t="n">
-        <v>89200</v>
-      </c>
-      <c r="E8" s="7" t="n">
-        <v>71800</v>
-      </c>
-      <c r="F8" s="11" t="n">
-        <v>0.08400000000000001</v>
-      </c>
-      <c r="G8" s="11" t="n">
-        <v>0.36</v>
+          <t>Combined rate (per $100 of assessed value)</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="n">
+        <v>2.148</v>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Rate as actually billed — not a statutory or effective rate.</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>Synthetic county tax record — Rate table, synthetic district</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>10 mi</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="n">
-        <v>402700</v>
-      </c>
-      <c r="C9" s="7" t="n">
-        <v>154900</v>
-      </c>
-      <c r="D9" s="7" t="n">
-        <v>92600</v>
-      </c>
-      <c r="E9" s="7" t="n">
-        <v>214500</v>
-      </c>
-      <c r="F9" s="11" t="n">
-        <v>0.091</v>
-      </c>
-      <c r="G9" s="11" t="n">
-        <v>0.34</v>
+          <t>Assessment ratio (legal class)</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Synthetic county tax record — Rate table</t>
+        </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="inlineStr">
-        <is>
-          <t>MSA</t>
-        </is>
-      </c>
-      <c r="B10" s="19" t="n">
-        <v>2418000</v>
-      </c>
-      <c r="C10" s="19" t="n">
-        <v>903400</v>
-      </c>
-      <c r="D10" s="19" t="n">
-        <v>86100</v>
-      </c>
-      <c r="E10" s="19" t="n">
-        <v>1284000</v>
-      </c>
-      <c r="F10" s="20" t="n">
-        <v>0.073</v>
-      </c>
-      <c r="G10" s="20" t="n">
-        <v>0.37</v>
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Rate divisor</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>Synthetic county tax record — Rate table</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Rate evidence</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="n"/>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Rate as billed, 2.148 per $100 of assessed value, read from the synthetic county bill for the 2025 tax year.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12"/>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Current year — computed, then checked against the bill</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="n"/>
+      <c r="C13" s="4" t="n"/>
+      <c r="D13" s="4" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Assessed-value basis</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="n">
+        <v>23000000</v>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>Assessed value (synthetic)</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>Synthetic county tax record — Valuation notice</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Assessment ratio</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Assessed value</t>
+        </is>
+      </c>
+      <c r="B16" s="7">
+        <f>B14*B15</f>
+        <v/>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>Basis times the legal-class ratio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Combined rate</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="n">
+        <v>2.148</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Computed annual tax</t>
+        </is>
+      </c>
+      <c r="B18" s="7">
+        <f>B16*B17/100</f>
+        <v/>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>Assessed value times rate, per $100.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>County billed amount</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="n">
+        <v>494040</v>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>As billed for 2025.</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>Synthetic county tax record — Tax bill</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Computed less billed</t>
+        </is>
+      </c>
+      <c r="B20" s="7">
+        <f>IF(AND(ISNUMBER(B18),ISNUMBER(B19)),B18-B19,"NOT CHECKED")</f>
+        <v/>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>Guarded: a missing input renders NOT CHECKED rather than a difference of zero.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>ties</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>Ties within 2% of the billed figure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Underwriting assumption at the illustrative price</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="n"/>
+      <c r="C23" s="4" t="n"/>
+      <c r="D23" s="4" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Does the basis reset on sale?</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>TX reassesses toward the transaction price, so the generic pattern applies: assessed value is the purchase price times the statutory assessment ratio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Illustrative purchase price (illustrative)</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="n">
+        <v>38700000</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Year-one basis</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="n">
+        <v>38700000</v>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>Purchase price x assessment ratio</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Year-one assessed value</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="n">
+        <v>38700000</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Year-one tax (illustrative)</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="n">
+        <v>831276.0000000001</v>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>The figure to carry into the model.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Year-one tax per unit (illustrative)</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="n">
+        <v>4618.200000000001</v>
+      </c>
+    </row>
+    <row r="31"/>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>What the generic shortcut would have said</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="n"/>
+      <c r="C32" s="4" t="n"/>
+      <c r="D32" s="4" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Assessed value if it reset to the price</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="n">
+        <v>38700000</v>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>Purchase price times the assessment ratio — the pattern that holds in most states.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Tax on that basis</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="n">
+        <v>831276.0000000001</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Overstatement versus the correct approach</t>
+        </is>
+      </c>
+      <c r="B35" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>Shown because the size of the error is the point. Carrying the generic pattern into an Arizona model does not shade the answer, it changes it: a tax line this far out fails a deal that works.</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -3483,7 +3853,1782 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:I86"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="46" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Demand</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Fixture Park — as of 2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Synthetic ring demographics in the shape the real engine produces: ACS 5-year, a 2020 decennial baseline, LODES workplace counts and BLS metro series. All public sources; no licensed provider.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n"/>
+      <c r="B4" s="3" t="n"/>
+      <c r="C4" s="3" t="n"/>
+      <c r="D4" s="3" t="n"/>
+      <c r="E4" s="3" t="n"/>
+      <c r="F4" s="3" t="n"/>
+      <c r="G4" s="3" t="n"/>
+      <c r="H4" s="3" t="n"/>
+    </row>
+    <row r="5" ht="46" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Read this before the 1-mile column: The 1-mile column overstates levels. Ring membership is decided by each census block group's internal point and then the whole block group is counted, so at 1 mile a single large block group can sit mostly outside the ring and still be counted whole. Measured against a commercial source, 1-mile population reads roughly 2.3x and households roughly 1.9x too high; the 3-, 5- and 10-mile columns do not have this problem. Read the 1-mile column for mix and shares, which are ratios and survive the overcount, and read levels off the 3-mile column.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Households</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n"/>
+      <c r="C7" s="4" t="n"/>
+      <c r="D7" s="4" t="n"/>
+      <c r="E7" s="4" t="n"/>
+      <c r="F7" s="4" t="n"/>
+      <c r="G7" s="4" t="n"/>
+      <c r="H7" s="4" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>2020 Census baseline, 2024 ACS actual, and a 2026 projection.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr"/>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>1 mi</t>
+        </is>
+      </c>
+      <c r="C9" s="14" t="inlineStr">
+        <is>
+          <t>3 mi</t>
+        </is>
+      </c>
+      <c r="D9" s="14" t="inlineStr">
+        <is>
+          <t>5 mi</t>
+        </is>
+      </c>
+      <c r="E9" s="14" t="inlineStr">
+        <is>
+          <t>10 mi</t>
+        </is>
+      </c>
+      <c r="F9" s="14" t="inlineStr">
+        <is>
+          <t>Demo MSA</t>
+        </is>
+      </c>
+      <c r="G9" s="14" t="inlineStr">
+        <is>
+          <t>Demo State</t>
+        </is>
+      </c>
+      <c r="H9" s="14" t="inlineStr">
+        <is>
+          <t>U.S.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Households (2020 Census)</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="n">
+        <v>3780</v>
+      </c>
+      <c r="C10" s="7" t="n">
+        <v>20520</v>
+      </c>
+      <c r="D10" s="7" t="n">
+        <v>49680</v>
+      </c>
+      <c r="E10" s="7" t="n">
+        <v>146700</v>
+      </c>
+      <c r="F10" s="7" t="n">
+        <v>774000</v>
+      </c>
+      <c r="G10" s="7" t="n">
+        <v>1170000</v>
+      </c>
+      <c r="H10" s="7" t="n">
+        <v>54000000</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Households (2024 actual)</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="n">
+        <v>4011</v>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>21774</v>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>52716</v>
+      </c>
+      <c r="E11" s="7" t="n">
+        <v>155665</v>
+      </c>
+      <c r="F11" s="7" t="n">
+        <v>821300</v>
+      </c>
+      <c r="G11" s="7" t="n">
+        <v>1241500</v>
+      </c>
+      <c r="H11" s="7" t="n">
+        <v>57300000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Growth 2020 to 2024</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="n">
+        <v>0.0611</v>
+      </c>
+      <c r="C12" s="11" t="n">
+        <v>0.0611</v>
+      </c>
+      <c r="D12" s="11" t="n">
+        <v>0.0611</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>0.0611</v>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>0.0611</v>
+      </c>
+      <c r="G12" s="11" t="n">
+        <v>0.0611</v>
+      </c>
+      <c r="H12" s="11" t="n">
+        <v>0.0611</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Est. annual growth rate (to 2026)</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="n">
+        <v>0.0225</v>
+      </c>
+      <c r="C13" s="12" t="n"/>
+      <c r="D13" s="12" t="n"/>
+      <c r="E13" s="12" t="n"/>
+      <c r="F13" s="12" t="n"/>
+      <c r="G13" s="12" t="n"/>
+      <c r="H13" s="12" t="n"/>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>An assumption, not a measurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Households (2026 est.)</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="n">
+        <v>4194</v>
+      </c>
+      <c r="C14" s="7" t="n">
+        <v>22765</v>
+      </c>
+      <c r="D14" s="7" t="n">
+        <v>55115</v>
+      </c>
+      <c r="E14" s="7" t="n">
+        <v>162749</v>
+      </c>
+      <c r="F14" s="7" t="n">
+        <v>858674</v>
+      </c>
+      <c r="G14" s="7" t="n">
+        <v>1297996</v>
+      </c>
+      <c r="H14" s="7" t="n">
+        <v>59907508</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Population</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="n"/>
+      <c r="C16" s="4" t="n"/>
+      <c r="D16" s="4" t="n"/>
+      <c r="E16" s="4" t="n"/>
+      <c r="F16" s="4" t="n"/>
+      <c r="G16" s="4" t="n"/>
+      <c r="H16" s="4" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="14" t="inlineStr"/>
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>1 mi</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="inlineStr">
+        <is>
+          <t>3 mi</t>
+        </is>
+      </c>
+      <c r="D17" s="14" t="inlineStr">
+        <is>
+          <t>5 mi</t>
+        </is>
+      </c>
+      <c r="E17" s="14" t="inlineStr">
+        <is>
+          <t>10 mi</t>
+        </is>
+      </c>
+      <c r="F17" s="14" t="inlineStr">
+        <is>
+          <t>Demo MSA</t>
+        </is>
+      </c>
+      <c r="G17" s="14" t="inlineStr">
+        <is>
+          <t>Demo State</t>
+        </is>
+      </c>
+      <c r="H17" s="14" t="inlineStr">
+        <is>
+          <t>U.S.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Population (2020 Census)</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="n">
+        <v>9555</v>
+      </c>
+      <c r="C18" s="7" t="n">
+        <v>51870</v>
+      </c>
+      <c r="D18" s="7" t="n">
+        <v>125580</v>
+      </c>
+      <c r="E18" s="7" t="n">
+        <v>370825</v>
+      </c>
+      <c r="F18" s="7" t="n">
+        <v>1956500</v>
+      </c>
+      <c r="G18" s="7" t="n">
+        <v>2957500</v>
+      </c>
+      <c r="H18" s="7" t="n">
+        <v>136500000</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Population (2024 actual)</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="n">
+        <v>10017</v>
+      </c>
+      <c r="C19" s="7" t="n">
+        <v>54378</v>
+      </c>
+      <c r="D19" s="7" t="n">
+        <v>131652</v>
+      </c>
+      <c r="E19" s="7" t="n">
+        <v>388755</v>
+      </c>
+      <c r="F19" s="7" t="n">
+        <v>2051100</v>
+      </c>
+      <c r="G19" s="7" t="n">
+        <v>3100500</v>
+      </c>
+      <c r="H19" s="7" t="n">
+        <v>143100000</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Growth 2020 to 2024</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="n">
+        <v>0.0484</v>
+      </c>
+      <c r="C20" s="11" t="n">
+        <v>0.0484</v>
+      </c>
+      <c r="D20" s="11" t="n">
+        <v>0.0484</v>
+      </c>
+      <c r="E20" s="11" t="n">
+        <v>0.0484</v>
+      </c>
+      <c r="F20" s="11" t="n">
+        <v>0.0484</v>
+      </c>
+      <c r="G20" s="11" t="n">
+        <v>0.0484</v>
+      </c>
+      <c r="H20" s="11" t="n">
+        <v>0.0484</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Est. annual growth rate (to 2026)</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="C21" s="12" t="n"/>
+      <c r="D21" s="12" t="n"/>
+      <c r="E21" s="12" t="n"/>
+      <c r="F21" s="12" t="n"/>
+      <c r="G21" s="12" t="n"/>
+      <c r="H21" s="12" t="n"/>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>An assumption, not a measurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Population (2026 est.)</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="n">
+        <v>10239</v>
+      </c>
+      <c r="C22" s="7" t="n">
+        <v>55581</v>
+      </c>
+      <c r="D22" s="7" t="n">
+        <v>134564</v>
+      </c>
+      <c r="E22" s="7" t="n">
+        <v>397355</v>
+      </c>
+      <c r="F22" s="7" t="n">
+        <v>2096472</v>
+      </c>
+      <c r="G22" s="7" t="n">
+        <v>3169086</v>
+      </c>
+      <c r="H22" s="7" t="n">
+        <v>146265515</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Households by income (2024 actual)</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="n"/>
+      <c r="C24" s="4" t="n"/>
+      <c r="D24" s="4" t="n"/>
+      <c r="E24" s="4" t="n"/>
+      <c r="F24" s="4" t="n"/>
+      <c r="G24" s="4" t="n"/>
+      <c r="H24" s="4" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>Eight brackets, with the two affordability subtotals underneath.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="14" t="inlineStr"/>
+      <c r="B26" s="14" t="inlineStr">
+        <is>
+          <t>1 mi</t>
+        </is>
+      </c>
+      <c r="C26" s="14" t="inlineStr">
+        <is>
+          <t>3 mi</t>
+        </is>
+      </c>
+      <c r="D26" s="14" t="inlineStr">
+        <is>
+          <t>5 mi</t>
+        </is>
+      </c>
+      <c r="E26" s="14" t="inlineStr">
+        <is>
+          <t>10 mi</t>
+        </is>
+      </c>
+      <c r="F26" s="14" t="inlineStr">
+        <is>
+          <t>Demo MSA</t>
+        </is>
+      </c>
+      <c r="G26" s="14" t="inlineStr">
+        <is>
+          <t>Demo State</t>
+        </is>
+      </c>
+      <c r="H26" s="14" t="inlineStr">
+        <is>
+          <t>U.S.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Less than $25,000</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="n">
+        <v>473</v>
+      </c>
+      <c r="C27" s="7" t="n">
+        <v>2569</v>
+      </c>
+      <c r="D27" s="7" t="n">
+        <v>6220</v>
+      </c>
+      <c r="E27" s="7" t="n">
+        <v>18368</v>
+      </c>
+      <c r="F27" s="7" t="n">
+        <v>96913</v>
+      </c>
+      <c r="G27" s="7" t="n">
+        <v>146497</v>
+      </c>
+      <c r="H27" s="7" t="n">
+        <v>6761400</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    $25,000 - $49,999</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="n">
+        <v>586</v>
+      </c>
+      <c r="C28" s="7" t="n">
+        <v>3179</v>
+      </c>
+      <c r="D28" s="7" t="n">
+        <v>7697</v>
+      </c>
+      <c r="E28" s="7" t="n">
+        <v>22727</v>
+      </c>
+      <c r="F28" s="7" t="n">
+        <v>119910</v>
+      </c>
+      <c r="G28" s="7" t="n">
+        <v>181259</v>
+      </c>
+      <c r="H28" s="7" t="n">
+        <v>8365800</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    $50,000 - $74,999</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="n">
+        <v>610</v>
+      </c>
+      <c r="C29" s="7" t="n">
+        <v>3310</v>
+      </c>
+      <c r="D29" s="7" t="n">
+        <v>8013</v>
+      </c>
+      <c r="E29" s="7" t="n">
+        <v>23661</v>
+      </c>
+      <c r="F29" s="7" t="n">
+        <v>124838</v>
+      </c>
+      <c r="G29" s="7" t="n">
+        <v>188708</v>
+      </c>
+      <c r="H29" s="7" t="n">
+        <v>8709600</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    $75,000 - $99,999</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="n">
+        <v>558</v>
+      </c>
+      <c r="C30" s="7" t="n">
+        <v>3027</v>
+      </c>
+      <c r="D30" s="7" t="n">
+        <v>7328</v>
+      </c>
+      <c r="E30" s="7" t="n">
+        <v>21637</v>
+      </c>
+      <c r="F30" s="7" t="n">
+        <v>114161</v>
+      </c>
+      <c r="G30" s="7" t="n">
+        <v>172569</v>
+      </c>
+      <c r="H30" s="7" t="n">
+        <v>7964700</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    $100,000 - $124,999</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="n">
+        <v>485</v>
+      </c>
+      <c r="C31" s="7" t="n">
+        <v>2635</v>
+      </c>
+      <c r="D31" s="7" t="n">
+        <v>6379</v>
+      </c>
+      <c r="E31" s="7" t="n">
+        <v>18835</v>
+      </c>
+      <c r="F31" s="7" t="n">
+        <v>99377</v>
+      </c>
+      <c r="G31" s="7" t="n">
+        <v>150222</v>
+      </c>
+      <c r="H31" s="7" t="n">
+        <v>6933300</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    $125,000 - $149,999</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="n">
+        <v>369</v>
+      </c>
+      <c r="C32" s="7" t="n">
+        <v>2003</v>
+      </c>
+      <c r="D32" s="7" t="n">
+        <v>4850</v>
+      </c>
+      <c r="E32" s="7" t="n">
+        <v>14321</v>
+      </c>
+      <c r="F32" s="7" t="n">
+        <v>75560</v>
+      </c>
+      <c r="G32" s="7" t="n">
+        <v>114218</v>
+      </c>
+      <c r="H32" s="7" t="n">
+        <v>5271600</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    $150,000 - $199,999</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="n">
+        <v>457</v>
+      </c>
+      <c r="C33" s="7" t="n">
+        <v>2482</v>
+      </c>
+      <c r="D33" s="7" t="n">
+        <v>6010</v>
+      </c>
+      <c r="E33" s="7" t="n">
+        <v>17746</v>
+      </c>
+      <c r="F33" s="7" t="n">
+        <v>93628</v>
+      </c>
+      <c r="G33" s="7" t="n">
+        <v>141531</v>
+      </c>
+      <c r="H33" s="7" t="n">
+        <v>6532200</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    $200,000 and over</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="n">
+        <v>473</v>
+      </c>
+      <c r="C34" s="7" t="n">
+        <v>2569</v>
+      </c>
+      <c r="D34" s="7" t="n">
+        <v>6220</v>
+      </c>
+      <c r="E34" s="7" t="n">
+        <v>18368</v>
+      </c>
+      <c r="F34" s="7" t="n">
+        <v>96913</v>
+      </c>
+      <c r="G34" s="7" t="n">
+        <v>146497</v>
+      </c>
+      <c r="H34" s="7" t="n">
+        <v>6761400</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Subtotal $50,000 and over</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="n">
+        <v>2952</v>
+      </c>
+      <c r="C35" s="7" t="n">
+        <v>16026</v>
+      </c>
+      <c r="D35" s="7" t="n">
+        <v>38799</v>
+      </c>
+      <c r="E35" s="7" t="n">
+        <v>114569</v>
+      </c>
+      <c r="F35" s="7" t="n">
+        <v>604477</v>
+      </c>
+      <c r="G35" s="7" t="n">
+        <v>913744</v>
+      </c>
+      <c r="H35" s="7" t="n">
+        <v>42172800</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   share of households</t>
+        </is>
+      </c>
+      <c r="B36" s="11" t="n">
+        <v>0.736</v>
+      </c>
+      <c r="C36" s="11" t="n">
+        <v>0.736</v>
+      </c>
+      <c r="D36" s="11" t="n">
+        <v>0.736</v>
+      </c>
+      <c r="E36" s="11" t="n">
+        <v>0.736</v>
+      </c>
+      <c r="F36" s="11" t="n">
+        <v>0.736</v>
+      </c>
+      <c r="G36" s="11" t="n">
+        <v>0.736</v>
+      </c>
+      <c r="H36" s="11" t="n">
+        <v>0.736</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Subtotal $100,000 and over</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="n">
+        <v>1785</v>
+      </c>
+      <c r="C37" s="7" t="n">
+        <v>9689</v>
+      </c>
+      <c r="D37" s="7" t="n">
+        <v>23459</v>
+      </c>
+      <c r="E37" s="7" t="n">
+        <v>69271</v>
+      </c>
+      <c r="F37" s="7" t="n">
+        <v>365478</v>
+      </c>
+      <c r="G37" s="7" t="n">
+        <v>552468</v>
+      </c>
+      <c r="H37" s="7" t="n">
+        <v>25498500</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   share of households</t>
+        </is>
+      </c>
+      <c r="B38" s="11" t="n">
+        <v>0.445</v>
+      </c>
+      <c r="C38" s="11" t="n">
+        <v>0.445</v>
+      </c>
+      <c r="D38" s="11" t="n">
+        <v>0.445</v>
+      </c>
+      <c r="E38" s="11" t="n">
+        <v>0.445</v>
+      </c>
+      <c r="F38" s="11" t="n">
+        <v>0.445</v>
+      </c>
+      <c r="G38" s="11" t="n">
+        <v>0.445</v>
+      </c>
+      <c r="H38" s="11" t="n">
+        <v>0.445</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Income and affordability</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="n"/>
+      <c r="C40" s="4" t="n"/>
+      <c r="D40" s="4" t="n"/>
+      <c r="E40" s="4" t="n"/>
+      <c r="F40" s="4" t="n"/>
+      <c r="G40" s="4" t="n"/>
+      <c r="H40" s="4" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>Median interpolated from the brackets above, so the two cannot disagree.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="14" t="inlineStr"/>
+      <c r="B42" s="14" t="inlineStr">
+        <is>
+          <t>1 mi</t>
+        </is>
+      </c>
+      <c r="C42" s="14" t="inlineStr">
+        <is>
+          <t>3 mi</t>
+        </is>
+      </c>
+      <c r="D42" s="14" t="inlineStr">
+        <is>
+          <t>5 mi</t>
+        </is>
+      </c>
+      <c r="E42" s="14" t="inlineStr">
+        <is>
+          <t>10 mi</t>
+        </is>
+      </c>
+      <c r="F42" s="14" t="inlineStr">
+        <is>
+          <t>Demo MSA</t>
+        </is>
+      </c>
+      <c r="G42" s="14" t="inlineStr">
+        <is>
+          <t>Demo State</t>
+        </is>
+      </c>
+      <c r="H42" s="14" t="inlineStr">
+        <is>
+          <t>U.S.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Average household income (2024)</t>
+        </is>
+      </c>
+      <c r="B43" s="7" t="n">
+        <v>81200</v>
+      </c>
+      <c r="C43" s="7" t="n">
+        <v>103400</v>
+      </c>
+      <c r="D43" s="7" t="n">
+        <v>107900</v>
+      </c>
+      <c r="E43" s="7" t="n">
+        <v>112600</v>
+      </c>
+      <c r="F43" s="7" t="n">
+        <v>118800</v>
+      </c>
+      <c r="G43" s="7" t="n">
+        <v>108100</v>
+      </c>
+      <c r="H43" s="7" t="n">
+        <v>113900</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Median household income (2024)</t>
+        </is>
+      </c>
+      <c r="B44" s="7" t="n">
+        <v>66500</v>
+      </c>
+      <c r="C44" s="7" t="n">
+        <v>81900</v>
+      </c>
+      <c r="D44" s="7" t="n">
+        <v>83100</v>
+      </c>
+      <c r="E44" s="7" t="n">
+        <v>83400</v>
+      </c>
+      <c r="F44" s="7" t="n">
+        <v>88900</v>
+      </c>
+      <c r="G44" s="7" t="n">
+        <v>80600</v>
+      </c>
+      <c r="H44" s="7" t="n">
+        <v>81400</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Est. annual income growth (to 2026)</t>
+        </is>
+      </c>
+      <c r="B45" s="9" t="n">
+        <v>0.062</v>
+      </c>
+      <c r="C45" s="12" t="n"/>
+      <c r="D45" s="12" t="n"/>
+      <c r="E45" s="12" t="n"/>
+      <c r="F45" s="12" t="n"/>
+      <c r="G45" s="12" t="n"/>
+      <c r="H45" s="12" t="n"/>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>An assumption, not a measurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>Average household income (2026 est.)</t>
+        </is>
+      </c>
+      <c r="B46" s="7" t="n">
+        <v>91581</v>
+      </c>
+      <c r="C46" s="7" t="n">
+        <v>116619</v>
+      </c>
+      <c r="D46" s="7" t="n">
+        <v>121694</v>
+      </c>
+      <c r="E46" s="7" t="n">
+        <v>126995</v>
+      </c>
+      <c r="F46" s="7" t="n">
+        <v>133988</v>
+      </c>
+      <c r="G46" s="7" t="n">
+        <v>121920</v>
+      </c>
+      <c r="H46" s="7" t="n">
+        <v>128461</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Renter share</t>
+        </is>
+      </c>
+      <c r="B47" s="11" t="n">
+        <v>0.654</v>
+      </c>
+      <c r="C47" s="11" t="n">
+        <v>0.512</v>
+      </c>
+      <c r="D47" s="11" t="n">
+        <v>0.518</v>
+      </c>
+      <c r="E47" s="11" t="n">
+        <v>0.481</v>
+      </c>
+      <c r="F47" s="11" t="n">
+        <v>0.334</v>
+      </c>
+      <c r="G47" s="11" t="n">
+        <v>0.331</v>
+      </c>
+      <c r="H47" s="11" t="n">
+        <v>0.352</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Rent-to-income at $1,795/mo</t>
+        </is>
+      </c>
+      <c r="B48" s="11" t="n">
+        <v>0.265</v>
+      </c>
+      <c r="C48" s="11" t="n">
+        <v>0.208</v>
+      </c>
+      <c r="D48" s="11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E48" s="11" t="n">
+        <v>0.191</v>
+      </c>
+      <c r="F48" s="11" t="n">
+        <v>0.181</v>
+      </c>
+      <c r="G48" s="11" t="n">
+        <v>0.199</v>
+      </c>
+      <c r="H48" s="11" t="n">
+        <v>0.189</v>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>Against projected 2026 income, so it is a forward ratio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Home value — ZIP 00000 vs Demo MSA</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="n"/>
+      <c r="C50" s="4" t="n"/>
+      <c r="D50" s="4" t="n"/>
+      <c r="E50" s="4" t="n"/>
+      <c r="F50" s="4" t="n"/>
+      <c r="G50" s="4" t="n"/>
+      <c r="H50" s="4" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t>ZIP geography, not a drive ring — the only section that does not share the columns above, so it is shown as its own three figures rather than stretched across headers it does not describe.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="14" t="inlineStr"/>
+      <c r="B52" s="14" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>ZIP home value</t>
+        </is>
+      </c>
+      <c r="B53" s="7" t="n">
+        <v>451600</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Metro home value</t>
+        </is>
+      </c>
+      <c r="B54" s="7" t="n">
+        <v>446200</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>ZIP vs metro</t>
+        </is>
+      </c>
+      <c r="B55" s="11" t="n">
+        <v>0.0121</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Labor market</t>
+        </is>
+      </c>
+      <c r="B57" s="4" t="n"/>
+      <c r="C57" s="4" t="n"/>
+      <c r="D57" s="4" t="n"/>
+      <c r="E57" s="4" t="n"/>
+      <c r="F57" s="4" t="n"/>
+      <c r="G57" s="4" t="n"/>
+      <c r="H57" s="4" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>Ring job counts are WORKPLACE counts — jobs located inside the ring, not residents who hold jobs. The unemployment row is the opposite: residents.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="14" t="inlineStr"/>
+      <c r="B59" s="14" t="inlineStr">
+        <is>
+          <t>1 mi</t>
+        </is>
+      </c>
+      <c r="C59" s="14" t="inlineStr">
+        <is>
+          <t>3 mi</t>
+        </is>
+      </c>
+      <c r="D59" s="14" t="inlineStr">
+        <is>
+          <t>5 mi</t>
+        </is>
+      </c>
+      <c r="E59" s="14" t="inlineStr">
+        <is>
+          <t>10 mi</t>
+        </is>
+      </c>
+      <c r="F59" s="14" t="inlineStr">
+        <is>
+          <t>Demo MSA</t>
+        </is>
+      </c>
+      <c r="G59" s="14" t="inlineStr">
+        <is>
+          <t>Demo State</t>
+        </is>
+      </c>
+      <c r="H59" s="14" t="inlineStr">
+        <is>
+          <t>U.S.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
+        <is>
+          <t>Unemployment rate (residents, ACS)</t>
+        </is>
+      </c>
+      <c r="B60" s="11" t="n">
+        <v>0.066</v>
+      </c>
+      <c r="C60" s="11" t="n">
+        <v>0.052</v>
+      </c>
+      <c r="D60" s="11" t="n">
+        <v>0.048</v>
+      </c>
+      <c r="E60" s="11" t="n">
+        <v>0.046</v>
+      </c>
+      <c r="F60" s="11" t="n">
+        <v>0.047</v>
+      </c>
+      <c r="G60" s="11" t="n">
+        <v>0.051</v>
+      </c>
+      <c r="H60" s="11" t="n">
+        <v>0.052</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="13" t="inlineStr">
+        <is>
+          <t>Jobs located inside the ring — LODES workplace counts</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    2021</t>
+        </is>
+      </c>
+      <c r="B62" s="7" t="n">
+        <v>10370</v>
+      </c>
+      <c r="C62" s="7" t="n">
+        <v>122100</v>
+      </c>
+      <c r="D62" s="7" t="n">
+        <v>352300</v>
+      </c>
+      <c r="E62" s="7" t="n">
+        <v>903200</v>
+      </c>
+      <c r="F62" s="12" t="n"/>
+      <c r="G62" s="12" t="n"/>
+      <c r="H62" s="12" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    2022</t>
+        </is>
+      </c>
+      <c r="B63" s="7" t="n">
+        <v>11300</v>
+      </c>
+      <c r="C63" s="7" t="n">
+        <v>127600</v>
+      </c>
+      <c r="D63" s="7" t="n">
+        <v>361400</v>
+      </c>
+      <c r="E63" s="7" t="n">
+        <v>921800</v>
+      </c>
+      <c r="F63" s="12" t="n"/>
+      <c r="G63" s="12" t="n"/>
+      <c r="H63" s="12" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    2023  (latest)</t>
+        </is>
+      </c>
+      <c r="B64" s="7" t="n">
+        <v>11644</v>
+      </c>
+      <c r="C64" s="7" t="n">
+        <v>140800</v>
+      </c>
+      <c r="D64" s="7" t="n">
+        <v>382500</v>
+      </c>
+      <c r="E64" s="7" t="n">
+        <v>990700</v>
+      </c>
+      <c r="F64" s="12" t="n"/>
+      <c r="G64" s="12" t="n"/>
+      <c r="H64" s="12" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Job growth 2021 to 2023</t>
+        </is>
+      </c>
+      <c r="B65" s="11" t="n">
+        <v>0.1229</v>
+      </c>
+      <c r="C65" s="11" t="n">
+        <v>0.1531</v>
+      </c>
+      <c r="D65" s="11" t="n">
+        <v>0.0858</v>
+      </c>
+      <c r="E65" s="11" t="n">
+        <v>0.0968</v>
+      </c>
+      <c r="F65" s="12" t="n"/>
+      <c r="G65" s="12" t="n"/>
+      <c r="H65" s="12" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="13" t="inlineStr">
+        <is>
+          <t>Metro nonfarm employment and unemployment — Demo County, Demo State</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="14" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="B68" s="14" t="inlineStr">
+        <is>
+          <t>Nonfarm jobs (000s)</t>
+        </is>
+      </c>
+      <c r="C68" s="14" t="inlineStr">
+        <is>
+          <t>Job growth</t>
+        </is>
+      </c>
+      <c r="D68" s="14" t="inlineStr">
+        <is>
+          <t>Unemployment</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="12" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B69" s="10" t="n">
+        <v>2462.5</v>
+      </c>
+      <c r="C69" s="11" t="n">
+        <v>0.0026</v>
+      </c>
+      <c r="D69" s="11" t="n">
+        <v>0.0423</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="12" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B70" s="10" t="n">
+        <v>2456</v>
+      </c>
+      <c r="C70" s="11" t="n">
+        <v>0.0224</v>
+      </c>
+      <c r="D70" s="11" t="n">
+        <v>0.0367</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="12" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B71" s="10" t="n">
+        <v>2402.2</v>
+      </c>
+      <c r="C71" s="11" t="n">
+        <v>0.0311</v>
+      </c>
+      <c r="D71" s="11" t="n">
+        <v>0.0338</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="12" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B72" s="10" t="n">
+        <v>2329.7</v>
+      </c>
+      <c r="C72" s="11" t="n">
+        <v>0.0512</v>
+      </c>
+      <c r="D72" s="11" t="n">
+        <v>0.0311</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="4" t="inlineStr">
+        <is>
+          <t>Jobs by industry (2023)</t>
+        </is>
+      </c>
+      <c r="B74" s="4" t="n"/>
+      <c r="C74" s="4" t="n"/>
+      <c r="D74" s="4" t="n"/>
+      <c r="E74" s="4" t="n"/>
+      <c r="F74" s="4" t="n"/>
+      <c r="G74" s="4" t="n"/>
+      <c r="H74" s="4" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="6" t="inlineStr">
+        <is>
+          <t>Share of jobs by sector, sorted by the metro's own concentration. Ring, MSA and state shares come from LODES workplace counts; the U.S. column is QCEW, a different survey, so read it as a benchmark rather than the same measurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="14" t="inlineStr"/>
+      <c r="B76" s="14" t="inlineStr">
+        <is>
+          <t>1 mi</t>
+        </is>
+      </c>
+      <c r="C76" s="14" t="inlineStr">
+        <is>
+          <t>3 mi</t>
+        </is>
+      </c>
+      <c r="D76" s="14" t="inlineStr">
+        <is>
+          <t>5 mi</t>
+        </is>
+      </c>
+      <c r="E76" s="14" t="inlineStr">
+        <is>
+          <t>10 mi</t>
+        </is>
+      </c>
+      <c r="F76" s="14" t="inlineStr">
+        <is>
+          <t>Demo MSA</t>
+        </is>
+      </c>
+      <c r="G76" s="14" t="inlineStr">
+        <is>
+          <t>Demo State</t>
+        </is>
+      </c>
+      <c r="H76" s="14" t="inlineStr">
+        <is>
+          <t>U.S.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="5" t="inlineStr">
+        <is>
+          <t>Health Care/Social Asst</t>
+        </is>
+      </c>
+      <c r="B77" s="11" t="n">
+        <v>0.079</v>
+      </c>
+      <c r="C77" s="11" t="n">
+        <v>0.089</v>
+      </c>
+      <c r="D77" s="11" t="n">
+        <v>0.104</v>
+      </c>
+      <c r="E77" s="11" t="n">
+        <v>0.127</v>
+      </c>
+      <c r="F77" s="11" t="n">
+        <v>0.144</v>
+      </c>
+      <c r="G77" s="11" t="n">
+        <v>0.148</v>
+      </c>
+      <c r="H77" s="11" t="n">
+        <v>0.152</v>
+      </c>
+      <c r="I77" s="2" t="inlineStr">
+        <is>
+          <t>Location quotient vs U.S.: 0.95x — less concentrated here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="5" t="inlineStr">
+        <is>
+          <t>Retail Trade</t>
+        </is>
+      </c>
+      <c r="B78" s="11" t="n">
+        <v>0.091</v>
+      </c>
+      <c r="C78" s="11" t="n">
+        <v>0.091</v>
+      </c>
+      <c r="D78" s="11" t="n">
+        <v>0.08599999999999999</v>
+      </c>
+      <c r="E78" s="11" t="n">
+        <v>0.083</v>
+      </c>
+      <c r="F78" s="11" t="n">
+        <v>0.109</v>
+      </c>
+      <c r="G78" s="11" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="H78" s="11" t="n">
+        <v>0.102</v>
+      </c>
+      <c r="I78" s="2" t="inlineStr">
+        <is>
+          <t>Location quotient vs U.S.: 1.07x — more concentrated here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="5" t="inlineStr">
+        <is>
+          <t>Accommodation/Food Svcs</t>
+        </is>
+      </c>
+      <c r="B79" s="11" t="n">
+        <v>0.049</v>
+      </c>
+      <c r="C79" s="11" t="n">
+        <v>0.068</v>
+      </c>
+      <c r="D79" s="11" t="n">
+        <v>0.058</v>
+      </c>
+      <c r="E79" s="11" t="n">
+        <v>0.076</v>
+      </c>
+      <c r="F79" s="11" t="n">
+        <v>0.092</v>
+      </c>
+      <c r="G79" s="11" t="n">
+        <v>0.098</v>
+      </c>
+      <c r="H79" s="11" t="n">
+        <v>0.092</v>
+      </c>
+      <c r="I79" s="2" t="inlineStr">
+        <is>
+          <t>Location quotient vs U.S.: 1.00x — less concentrated here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="5" t="inlineStr">
+        <is>
+          <t>Professional/Scientific/Tech</t>
+        </is>
+      </c>
+      <c r="B80" s="11" t="n">
+        <v>0.061</v>
+      </c>
+      <c r="C80" s="11" t="n">
+        <v>0.074</v>
+      </c>
+      <c r="D80" s="11" t="n">
+        <v>0.081</v>
+      </c>
+      <c r="E80" s="11" t="n">
+        <v>0.07199999999999999</v>
+      </c>
+      <c r="F80" s="11" t="n">
+        <v>0.077</v>
+      </c>
+      <c r="G80" s="11" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="H80" s="11" t="n">
+        <v>0.08599999999999999</v>
+      </c>
+      <c r="I80" s="2" t="inlineStr">
+        <is>
+          <t>Location quotient vs U.S.: 0.90x — less concentrated here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="5" t="inlineStr">
+        <is>
+          <t>Educational Services</t>
+        </is>
+      </c>
+      <c r="B81" s="11" t="n">
+        <v>0.207</v>
+      </c>
+      <c r="C81" s="11" t="n">
+        <v>0.118</v>
+      </c>
+      <c r="D81" s="11" t="n">
+        <v>0.092</v>
+      </c>
+      <c r="E81" s="11" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="F81" s="11" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="G81" s="11" t="n">
+        <v>0.081</v>
+      </c>
+      <c r="H81" s="11" t="n">
+        <v>0.092</v>
+      </c>
+      <c r="I81" s="2" t="inlineStr">
+        <is>
+          <t>Location quotient vs U.S.: 0.82x — less concentrated here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="5" t="inlineStr">
+        <is>
+          <t>Admin/Support/Waste</t>
+        </is>
+      </c>
+      <c r="B82" s="11" t="n">
+        <v>0.038</v>
+      </c>
+      <c r="C82" s="11" t="n">
+        <v>0.052</v>
+      </c>
+      <c r="D82" s="11" t="n">
+        <v>0.061</v>
+      </c>
+      <c r="E82" s="11" t="n">
+        <v>0.058</v>
+      </c>
+      <c r="F82" s="11" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="G82" s="11" t="n">
+        <v>0.066</v>
+      </c>
+      <c r="H82" s="11" t="n">
+        <v>0.058</v>
+      </c>
+      <c r="I82" s="2" t="inlineStr">
+        <is>
+          <t>Location quotient vs U.S.: 1.21x — more concentrated here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="5" t="inlineStr">
+        <is>
+          <t>Finance/Insurance</t>
+        </is>
+      </c>
+      <c r="B83" s="11" t="n">
+        <v>0.021</v>
+      </c>
+      <c r="C83" s="11" t="n">
+        <v>0.038</v>
+      </c>
+      <c r="D83" s="11" t="n">
+        <v>0.049</v>
+      </c>
+      <c r="E83" s="11" t="n">
+        <v>0.043</v>
+      </c>
+      <c r="F83" s="11" t="n">
+        <v>0.061</v>
+      </c>
+      <c r="G83" s="11" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="H83" s="11" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="I83" s="2" t="inlineStr">
+        <is>
+          <t>Location quotient vs U.S.: 1.36x — more concentrated here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="5" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="B84" s="11" t="n">
+        <v>0.031</v>
+      </c>
+      <c r="C84" s="11" t="n">
+        <v>0.041</v>
+      </c>
+      <c r="D84" s="11" t="n">
+        <v>0.047</v>
+      </c>
+      <c r="E84" s="11" t="n">
+        <v>0.052</v>
+      </c>
+      <c r="F84" s="11" t="n">
+        <v>0.058</v>
+      </c>
+      <c r="G84" s="11" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="H84" s="11" t="n">
+        <v>0.052</v>
+      </c>
+      <c r="I84" s="2" t="inlineStr">
+        <is>
+          <t>Location quotient vs U.S.: 1.12x — more concentrated here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="5" t="inlineStr">
+        <is>
+          <t>Manufacturing</t>
+        </is>
+      </c>
+      <c r="B85" s="11" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="C85" s="11" t="n">
+        <v>0.029</v>
+      </c>
+      <c r="D85" s="11" t="n">
+        <v>0.038</v>
+      </c>
+      <c r="E85" s="11" t="n">
+        <v>0.049</v>
+      </c>
+      <c r="F85" s="11" t="n">
+        <v>0.052</v>
+      </c>
+      <c r="G85" s="11" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="H85" s="11" t="n">
+        <v>0.08599999999999999</v>
+      </c>
+      <c r="I85" s="2" t="inlineStr">
+        <is>
+          <t>Location quotient vs U.S.: 0.60x — less concentrated here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="5" t="inlineStr">
+        <is>
+          <t>Transportation/Warehousing</t>
+        </is>
+      </c>
+      <c r="B86" s="11" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="C86" s="11" t="n">
+        <v>0.024</v>
+      </c>
+      <c r="D86" s="11" t="n">
+        <v>0.031</v>
+      </c>
+      <c r="E86" s="11" t="n">
+        <v>0.041</v>
+      </c>
+      <c r="F86" s="11" t="n">
+        <v>0.046</v>
+      </c>
+      <c r="G86" s="11" t="n">
+        <v>0.044</v>
+      </c>
+      <c r="H86" s="11" t="n">
+        <v>0.042</v>
+      </c>
+      <c r="I86" s="2" t="inlineStr">
+        <is>
+          <t>Location quotient vs U.S.: 1.10x — more concentrated here.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -3523,62 +5668,34 @@
       <c r="G4" s="3" t="n"/>
       <c r="H4" s="3" t="n"/>
     </row>
-    <row r="5">
-      <c r="A5" s="14" t="inlineStr">
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Coverage note: these rings and stages are real and unmodified, and a zero is a genuine zero for the sources covered so far — not a gap left blank. Coverage of the permit and entitlement pipeline is an area of ongoing work and will be expanded, so read this section as a FLOOR on competing supply rather than a census of it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6"/>
+    <row r="7">
+      <c r="A7" s="14" t="inlineStr">
         <is>
           <t>Ring</t>
         </is>
       </c>
-      <c r="B5" s="14" t="inlineStr">
+      <c r="B7" s="14" t="inlineStr">
         <is>
           <t>Stage</t>
         </is>
       </c>
-      <c r="C5" s="14" t="inlineStr">
+      <c r="C7" s="14" t="inlineStr">
         <is>
           <t>Projects</t>
         </is>
       </c>
-      <c r="D5" s="14" t="inlineStr">
+      <c r="D7" s="14" t="inlineStr">
         <is>
           <t>Units</t>
         </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>1 mi</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>Entitlement</t>
-        </is>
-      </c>
-      <c r="C6" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" s="7" t="n">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>1 mi</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Permitted</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D7" s="7" t="n">
-        <v>148</v>
       </c>
     </row>
     <row r="8">
@@ -3589,14 +5706,14 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Under construction</t>
+          <t>Entitlement</t>
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>0</v>
+        <v>220</v>
       </c>
     </row>
     <row r="9">
@@ -3607,50 +5724,50 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Delivered (24 mo)</t>
+          <t>Permitted</t>
         </is>
       </c>
       <c r="C9" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>96</v>
+        <v>148</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>3 mi</t>
+          <t>1 mi</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Entitlement</t>
+          <t>Under construction</t>
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>742</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>3 mi</t>
+          <t>1 mi</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Permitted</t>
+          <t>Delivered (24 mo)</t>
         </is>
       </c>
       <c r="C11" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D11" s="7" t="n">
-        <v>410</v>
+        <v>96</v>
       </c>
     </row>
     <row r="12">
@@ -3661,14 +5778,14 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Under construction</t>
+          <t>Entitlement</t>
         </is>
       </c>
       <c r="C12" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D12" s="7" t="n">
-        <v>508</v>
+        <v>742</v>
       </c>
     </row>
     <row r="13">
@@ -3679,50 +5796,50 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Delivered (24 mo)</t>
+          <t>Permitted</t>
         </is>
       </c>
       <c r="C13" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D13" s="7" t="n">
-        <v>624</v>
+        <v>410</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>5 mi</t>
+          <t>3 mi</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Entitlement</t>
+          <t>Under construction</t>
         </is>
       </c>
       <c r="C14" s="7" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D14" s="7" t="n">
-        <v>1485</v>
+        <v>508</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>5 mi</t>
+          <t>3 mi</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Permitted</t>
+          <t>Delivered (24 mo)</t>
         </is>
       </c>
       <c r="C15" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D15" s="7" t="n">
-        <v>903</v>
+        <v>624</v>
       </c>
     </row>
     <row r="16">
@@ -3733,14 +5850,14 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Under construction</t>
+          <t>Entitlement</t>
         </is>
       </c>
       <c r="C16" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D16" s="7" t="n">
-        <v>1240</v>
+        <v>1485</v>
       </c>
     </row>
     <row r="17">
@@ -3751,100 +5868,136 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
+          <t>Permitted</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="D17" s="7" t="n">
+        <v>903</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>5 mi</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Under construction</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="D18" s="7" t="n">
+        <v>1240</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>5 mi</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
           <t>Delivered (24 mo)</t>
         </is>
       </c>
-      <c r="C17" s="7" t="n">
+      <c r="C19" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="D17" s="7" t="n">
+      <c r="D19" s="7" t="n">
         <v>1608</v>
       </c>
     </row>
-    <row r="18"/>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+    <row r="20"/>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>Ring totals</t>
         </is>
       </c>
-      <c r="B19" s="4" t="n"/>
-      <c r="C19" s="4" t="n"/>
-      <c r="D19" s="4" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="14" t="inlineStr">
+      <c r="B21" s="4" t="n"/>
+      <c r="C21" s="4" t="n"/>
+      <c r="D21" s="4" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="14" t="inlineStr">
         <is>
           <t>Ring</t>
         </is>
       </c>
-      <c r="B20" s="14" t="inlineStr">
+      <c r="B22" s="14" t="inlineStr">
         <is>
           <t>Pipeline units</t>
         </is>
       </c>
-      <c r="C20" s="14" t="inlineStr">
+      <c r="C22" s="14" t="inlineStr">
         <is>
           <t>Existing stock</t>
         </is>
       </c>
-      <c r="D20" s="14" t="inlineStr">
+      <c r="D22" s="14" t="inlineStr">
         <is>
           <t>Units as % of stock</t>
         </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>1 mi</t>
-        </is>
-      </c>
-      <c r="B21" s="7">
-        <f>SUMIF($A$6:$A$17,$A21,$D$6:$D$17)</f>
-        <v/>
-      </c>
-      <c r="C21" s="7" t="n">
-        <v>3140</v>
-      </c>
-      <c r="D21" s="11">
-        <f>IFERROR(B21/C21,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>3 mi</t>
-        </is>
-      </c>
-      <c r="B22" s="7">
-        <f>SUMIF($A$6:$A$17,$A22,$D$6:$D$17)</f>
-        <v/>
-      </c>
-      <c r="C22" s="7" t="n">
-        <v>18600</v>
-      </c>
-      <c r="D22" s="11">
-        <f>IFERROR(B22/C22,"")</f>
-        <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>5 mi</t>
+          <t>1 mi</t>
         </is>
       </c>
       <c r="B23" s="7">
-        <f>SUMIF($A$6:$A$17,$A23,$D$6:$D$17)</f>
+        <f>SUMIF($A$8:$A$19,$A23,$D$8:$D$19)</f>
         <v/>
       </c>
       <c r="C23" s="7" t="n">
-        <v>41200</v>
+        <v>3140</v>
       </c>
       <c r="D23" s="11">
         <f>IFERROR(B23/C23,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>3 mi</t>
+        </is>
+      </c>
+      <c r="B24" s="7">
+        <f>SUMIF($A$8:$A$19,$A24,$D$8:$D$19)</f>
+        <v/>
+      </c>
+      <c r="C24" s="7" t="n">
+        <v>18600</v>
+      </c>
+      <c r="D24" s="11">
+        <f>IFERROR(B24/C24,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>5 mi</t>
+        </is>
+      </c>
+      <c r="B25" s="7">
+        <f>SUMIF($A$8:$A$19,$A25,$D$8:$D$19)</f>
+        <v/>
+      </c>
+      <c r="C25" s="7" t="n">
+        <v>41200</v>
+      </c>
+      <c r="D25" s="11">
+        <f>IFERROR(B25/C25,"")</f>
         <v/>
       </c>
     </row>
@@ -3853,7 +6006,295 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="110" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Notes and disclosures</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Fixture Park — as of 2026-06-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Every output here is the result of decisions someone made. These are those decisions, including the ones that make the numbers look worse.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n"/>
+      <c r="B4" s="3" t="n"/>
+      <c r="C4" s="3" t="n"/>
+      <c r="D4" s="3" t="n"/>
+      <c r="E4" s="3" t="n"/>
+      <c r="F4" s="3" t="n"/>
+      <c r="G4" s="3" t="n"/>
+      <c r="H4" s="3" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>Topic</t>
+        </is>
+      </c>
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>Applies to</t>
+        </is>
+      </c>
+      <c r="C5" s="14" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Pricing is illustrative</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Deal Summary — Pricing</t>
+        </is>
+      </c>
+      <c r="C6" s="19" t="inlineStr">
+        <is>
+          <t>Every price, per-unit figure and cap rate in this set is illustrative. The per-unit price is a round number chosen to sit inside the band a real per-unit sale price occupies, so the cap-rate arithmetic is realistic. It is not a quote, an offer, a broker's guidance, or a valuation. Cap rates move inversely with the price, so read them as a demonstration of the mechanics rather than a view on the asset.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Licensed data is excluded by design, not by omission</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Rent Comps</t>
+        </is>
+      </c>
+      <c r="C7" s="19" t="inlineStr">
+        <is>
+          <t>No subscription or licensed market-data feed appears anywhere in this set. Comps come only from an operator's own weekly scrape of public leasing pages. That is a deliberate constraint, not a gap: licensed data cannot travel outside the licence, so a portfolio piece built on it could not be shown at all. The cost is coverage, and the coverage is measured and stated rather than assumed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Comp radius is set by measured coverage</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Rent Comps</t>
+        </is>
+      </c>
+      <c r="C8" s="19" t="inlineStr">
+        <is>
+          <t>Three miles, because that is the ring where the operator's own scrape actually holds live rents for enough communities to say something. A wider ring would add distance without adding evidence — it trades real rents for guesses. The coverage sentence on the comp block is measured by a probe against the scraper's own status values, never written by hand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Comps are matched on vintage, and it changes the answer</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Rent Comps — tiers</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="inlineStr">
+        <is>
+          <t>The detailed tiers hold only communities within ten years of the subject's year built. This is not cosmetic. On this deal the flat comp set — every nearby community with rents — averaged a 1981 asset against product built 1994 to 2026 and read the subject as roughly 9% BELOW market. Restricted to same-vintage comps the subject is about 1.5% ABOVE market. The first number was measuring the age gap, not the market. Whenever a comp set is wide enough to include newer product, the spread it reports is partly a renovation and amenity story wearing a rent label.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Year built comes from a free-text note, where it exists at all</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Rent Comps — tiers</t>
+        </is>
+      </c>
+      <c r="C10" s="19" t="inlineStr">
+        <is>
+          <t>The rent tracker has no year-built column. Where a vintage appears here it was parsed out of a free-text note on the community record, and every row carries that as its source. A community with no such note keeps its place in the comp set on distance and product, shows a dash for the year, and the tier header says how many rows the vintage filter could not be applied to. Inventing a year would fabricate the evidence the filter runs on; dropping the community would hide the closest comps for want of a field the source never had.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Market rent is never a blend of new and renewal</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Rent Roll — Summary</t>
+        </is>
+      </c>
+      <c r="C11" s="19" t="inlineStr">
+        <is>
+          <t>Market rent for the model is the new-lease average where a plan has new leases inside the lookback window, and in-place rent where it does not. It is never the average of new and renewal leases together. A blended figure reads as market rent and is not one: renewals are priced off the existing rent, so blending them in drags the number toward where rents used to be and understates the gap the underwriting is trying to measure. On this deal that rule produces a market rent BELOW in-place, which is the correct and uncomfortable answer for an asset whose in-place rents sit above what the market is currently signing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Estimated values are not published as facts</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>throughout</t>
+        </is>
+      </c>
+      <c r="C12" s="19" t="inlineStr">
+        <is>
+          <t>Where a figure is derived rather than read, the audit trail says so and names the inputs. Where a figure is unknown, the cell shows a visible hole rather than a plausible-looking number. A blank that reads as a zero is the most expensive kind of missing data, because nothing downstream flags it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>The lease trade-out report was available and deliberately not used</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Lease Trade-Out</t>
+        </is>
+      </c>
+      <c r="C13" s="19" t="inlineStr">
+        <is>
+          <t>Where a trade-out block appears with no rows, that is because the source report was not used, not because the data does not exist. Trade-out is derived from the rent roll's own lease dates and rents instead, so every figure in this set traces back to one of three raw sources. An output whose provenance forks across more documents than it needs is harder to audit for no analytical gain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Supply coverage is an area of ongoing work</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Supply</t>
+        </is>
+      </c>
+      <c r="C14" s="19" t="inlineStr">
+        <is>
+          <t>The supply section is real and unmodified — the rings, stages and unit counts come from a public permit and entitlement pipeline, and the zeros in the tight rings are genuine rather than missing. Coverage of that pipeline is an area of ongoing work: a ring showing no active supply means nothing was matched in the sources covered so far, which is a weaker statement than nothing being built. This section will be expanded; read it as a floor on competing supply, not a census of it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Checks degrade to NOT CHECKED rather than passing quietly</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Error Checks &amp; Pricing</t>
+        </is>
+      </c>
+      <c r="C15" s="19" t="inlineStr">
+        <is>
+          <t>Every cross-tie on the checks tab reports OK, FAIL, or NOT CHECKED. A check missing one of its inputs reports NOT CHECKED and claims no difference — it never reports OK. A green result that only means 'this check could not run' is worse than a red one, because it buys confidence it has not earned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>This deal does not exist</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>throughout</t>
+        </is>
+      </c>
+      <c r="C16" s="19" t="inlineStr">
+        <is>
+          <t>Fixture Park is fabricated end to end — the property, the operating statement, the rent roll, the comps and the demographics. It exists to exercise every edge the writers handle, so some of its figures are deliberately awkward: a plan with no priced units, a comp community with no published year, a revenue line the source statement never subtotalled.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>The 1-mile demographic ring overstates levels</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Demand</t>
+        </is>
+      </c>
+      <c r="C17" s="19" t="inlineStr">
+        <is>
+          <t>The 1-mile column overstates levels. Ring membership is decided by each census block group's internal point and then the whole block group is counted, so at 1 mile a single large block group can sit mostly outside the ring and still be counted whole. Measured against a commercial source, 1-mile population reads roughly 2.3x and households roughly 1.9x too high; the 3-, 5- and 10-mile columns do not have this problem. Read the 1-mile column for mix and shares, which are ratios and survive the overcount, and read levels off the 3-mile column.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>The rent readback checks transcription, not column choice</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Error Checks &amp; Pricing</t>
+        </is>
+      </c>
+      <c r="C18" s="19" t="inlineStr">
+        <is>
+          <t>Ten units are sampled and their normalized in-place rent is compared against the raw cell it came from, which catches a coercion or transcription error. It cannot catch the wrong rent column having been chosen, because both sides read the same column. The sample is seeded from the roll's as-of date, so the same roll always checks the same units.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3908,7 +6349,7 @@
           <t>Stamped values in this workbook</t>
         </is>
       </c>
-      <c r="B5" s="21" t="n">
+      <c r="B5" s="20" t="n">
         <v>44</v>
       </c>
     </row>
@@ -3962,7 +6403,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="22" t="inlineStr">
+      <c r="A9" s="21" t="inlineStr">
         <is>
           <t>closing_costs.mortgage_tax.amount</t>
         </is>
@@ -3992,14 +6433,14 @@
           <t>closing_costs.loan_amount, summary.state</t>
         </is>
       </c>
-      <c r="G9" s="23" t="inlineStr">
+      <c r="G9" s="19" t="inlineStr">
         <is>
           <t>Computed on the LOAN, never on the price. With no loan amount the line is reported as not asserted rather than inferred at 100% leverage.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="22" t="inlineStr">
+      <c r="A10" s="21" t="inlineStr">
         <is>
           <t>closing_costs.transfer_tax.amount</t>
         </is>
@@ -4029,14 +6470,14 @@
           <t>pricing.price_per_unit, pricing.unit_count, summary.state, closing_costs.price</t>
         </is>
       </c>
-      <c r="G10" s="23" t="inlineStr">
+      <c r="G10" s="19" t="inlineStr">
         <is>
           <t>Rate applied to price_per_unit x unit_count. Per-unit statutes round the consideration up.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="22" t="inlineStr">
+      <c r="A11" s="21" t="inlineStr">
         <is>
           <t>comps.nearby</t>
         </is>
@@ -4066,14 +6507,14 @@
           <t>comps.rows.tier</t>
         </is>
       </c>
-      <c r="G11" s="23" t="inlineStr">
+      <c r="G11" s="19" t="inlineStr">
         <is>
           <t>Every tracked community inside the radius that is not a detail row, with the reason it is not. No rent columns.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="22" t="inlineStr">
+      <c r="A12" s="21" t="inlineStr">
         <is>
           <t>comps.rows</t>
         </is>
@@ -4099,14 +6540,14 @@
         </is>
       </c>
       <c r="F12" s="12" t="n"/>
-      <c r="G12" s="23" t="inlineStr">
+      <c r="G12" s="19" t="inlineStr">
         <is>
           <t>Own weekly scrape; asking and net effective stated separately.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="22" t="inlineStr">
+      <c r="A13" s="21" t="inlineStr">
         <is>
           <t>comps.rows.tier</t>
         </is>
@@ -4136,14 +6577,14 @@
           <t>comps.rows.distance_mi, comps.tiering.subject_product, comps.tiering.subject_year_built, comps.tiering.year_band, comps.tiering.top_n, comps.tiering.additional_n</t>
         </is>
       </c>
-      <c r="G13" s="23" t="inlineStr">
+      <c r="G13" s="19" t="inlineStr">
         <is>
           <t>Tier 1 = the closest 5 matching product and vintage; tier 2 = the next 15; everything else is tier 3, identity only. An unknown year does not disqualify — it is disclosed on the tier header instead.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="22" t="inlineStr">
+      <c r="A14" s="21" t="inlineStr">
         <is>
           <t>demand.rings</t>
         </is>
@@ -4169,14 +6610,14 @@
         </is>
       </c>
       <c r="F14" s="12" t="n"/>
-      <c r="G14" s="23" t="inlineStr">
+      <c r="G14" s="19" t="inlineStr">
         <is>
           <t>Ring demographics.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="22" t="inlineStr">
+      <c r="A15" s="21" t="inlineStr">
         <is>
           <t>pricing.price_per_unit</t>
         </is>
@@ -4202,14 +6643,14 @@
         </is>
       </c>
       <c r="F15" s="12" t="n"/>
-      <c r="G15" s="23" t="inlineStr">
+      <c r="G15" s="19" t="inlineStr">
         <is>
           <t>Illustrative. Inside the band a per-unit sale price occupies.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="22" t="inlineStr">
+      <c r="A16" s="21" t="inlineStr">
         <is>
           <t>pricing.unit_count</t>
         </is>
@@ -4239,10 +6680,10 @@
           <t>summary.unit_count</t>
         </is>
       </c>
-      <c r="G16" s="24" t="n"/>
+      <c r="G16" s="22" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="22" t="inlineStr">
+      <c r="A17" s="21" t="inlineStr">
         <is>
           <t>summary.assessed_value_basis</t>
         </is>
@@ -4268,10 +6709,10 @@
         </is>
       </c>
       <c r="F17" s="12" t="n"/>
-      <c r="G17" s="24" t="n"/>
+      <c r="G17" s="22" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="22" t="inlineStr">
+      <c r="A18" s="21" t="inlineStr">
         <is>
           <t>summary.assessment_ratio</t>
         </is>
@@ -4297,10 +6738,10 @@
         </is>
       </c>
       <c r="F18" s="12" t="n"/>
-      <c r="G18" s="24" t="n"/>
+      <c r="G18" s="22" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="22" t="inlineStr">
+      <c r="A19" s="21" t="inlineStr">
         <is>
           <t>summary.city</t>
         </is>
@@ -4326,10 +6767,10 @@
         </is>
       </c>
       <c r="F19" s="12" t="n"/>
-      <c r="G19" s="24" t="n"/>
+      <c r="G19" s="22" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="22" t="inlineStr">
+      <c r="A20" s="21" t="inlineStr">
         <is>
           <t>summary.construction_status</t>
         </is>
@@ -4355,10 +6796,10 @@
         </is>
       </c>
       <c r="F20" s="12" t="n"/>
-      <c r="G20" s="24" t="n"/>
+      <c r="G20" s="22" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="22" t="inlineStr">
+      <c r="A21" s="21" t="inlineStr">
         <is>
           <t>summary.county</t>
         </is>
@@ -4384,10 +6825,10 @@
         </is>
       </c>
       <c r="F21" s="12" t="n"/>
-      <c r="G21" s="24" t="n"/>
+      <c r="G21" s="22" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="22" t="inlineStr">
+      <c r="A22" s="21" t="inlineStr">
         <is>
           <t>summary.deal_name</t>
         </is>
@@ -4413,14 +6854,14 @@
         </is>
       </c>
       <c r="F22" s="12" t="n"/>
-      <c r="G22" s="23" t="inlineStr">
+      <c r="G22" s="19" t="inlineStr">
         <is>
           <t>Fixture Park</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="22" t="inlineStr">
+      <c r="A23" s="21" t="inlineStr">
         <is>
           <t>summary.deal_status</t>
         </is>
@@ -4446,10 +6887,10 @@
         </is>
       </c>
       <c r="F23" s="12" t="n"/>
-      <c r="G23" s="24" t="n"/>
+      <c r="G23" s="22" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="22" t="inlineStr">
+      <c r="A24" s="21" t="inlineStr">
         <is>
           <t>summary.delivery_date</t>
         </is>
@@ -4475,10 +6916,10 @@
         </is>
       </c>
       <c r="F24" s="12" t="n"/>
-      <c r="G24" s="24" t="n"/>
+      <c r="G24" s="22" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="22" t="inlineStr">
+      <c r="A25" s="21" t="inlineStr">
         <is>
           <t>summary.fair_market_value</t>
         </is>
@@ -4504,14 +6945,14 @@
         </is>
       </c>
       <c r="F25" s="12" t="n"/>
-      <c r="G25" s="23" t="inlineStr">
+      <c r="G25" s="19" t="inlineStr">
         <is>
           <t>Operator's own estimate.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="22" t="inlineStr">
+      <c r="A26" s="21" t="inlineStr">
         <is>
           <t>summary.in_place_rent_avg</t>
         </is>
@@ -4541,14 +6982,14 @@
           <t>rent_roll.units</t>
         </is>
       </c>
-      <c r="G26" s="23" t="inlineStr">
+      <c r="G26" s="19" t="inlineStr">
         <is>
           <t>Occupied units, straight off the roll.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="22" t="inlineStr">
+      <c r="A27" s="21" t="inlineStr">
         <is>
           <t>summary.listing_brokerage</t>
         </is>
@@ -4578,14 +7019,14 @@
           <t>summary.seller_entity</t>
         </is>
       </c>
-      <c r="G27" s="23" t="inlineStr">
+      <c r="G27" s="19" t="inlineStr">
         <is>
           <t>Generic label; no firm or individual is named in a published file.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="22" t="inlineStr">
+      <c r="A28" s="21" t="inlineStr">
         <is>
           <t>summary.market_rent_for_model</t>
         </is>
@@ -4615,14 +7056,14 @@
           <t>rent_roll.units</t>
         </is>
       </c>
-      <c r="G28" s="23" t="inlineStr">
+      <c r="G28" s="19" t="inlineStr">
         <is>
           <t>New-lease average where a plan has new leases in the window, else in-place. Never a blend.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="22" t="inlineStr">
+      <c r="A29" s="21" t="inlineStr">
         <is>
           <t>summary.msa</t>
         </is>
@@ -4652,14 +7093,14 @@
           <t>summary.city, summary.state</t>
         </is>
       </c>
-      <c r="G29" s="23" t="inlineStr">
+      <c r="G29" s="19" t="inlineStr">
         <is>
           <t>Metro assigned from the city/state pair.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="22" t="inlineStr">
+      <c r="A30" s="21" t="inlineStr">
         <is>
           <t>summary.pricing_guidance</t>
         </is>
@@ -4685,14 +7126,14 @@
         </is>
       </c>
       <c r="F30" s="12" t="n"/>
-      <c r="G30" s="23" t="inlineStr">
+      <c r="G30" s="19" t="inlineStr">
         <is>
           <t>Illustrative figure supplied directly; not a quote or an offer.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="22" t="inlineStr">
+      <c r="A31" s="21" t="inlineStr">
         <is>
           <t>summary.product_detail</t>
         </is>
@@ -4718,10 +7159,10 @@
         </is>
       </c>
       <c r="F31" s="12" t="n"/>
-      <c r="G31" s="24" t="n"/>
+      <c r="G31" s="22" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="22" t="inlineStr">
+      <c r="A32" s="21" t="inlineStr">
         <is>
           <t>summary.product_type</t>
         </is>
@@ -4747,10 +7188,10 @@
         </is>
       </c>
       <c r="F32" s="12" t="n"/>
-      <c r="G32" s="24" t="n"/>
+      <c r="G32" s="22" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="22" t="inlineStr">
+      <c r="A33" s="21" t="inlineStr">
         <is>
           <t>summary.school_elementary_name</t>
         </is>
@@ -4776,10 +7217,10 @@
         </is>
       </c>
       <c r="F33" s="12" t="n"/>
-      <c r="G33" s="24" t="n"/>
+      <c r="G33" s="22" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="22" t="inlineStr">
+      <c r="A34" s="21" t="inlineStr">
         <is>
           <t>summary.school_high_name</t>
         </is>
@@ -4805,10 +7246,10 @@
         </is>
       </c>
       <c r="F34" s="12" t="n"/>
-      <c r="G34" s="24" t="n"/>
+      <c r="G34" s="22" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="22" t="inlineStr">
+      <c r="A35" s="21" t="inlineStr">
         <is>
           <t>summary.school_middle_name</t>
         </is>
@@ -4834,10 +7275,10 @@
         </is>
       </c>
       <c r="F35" s="12" t="n"/>
-      <c r="G35" s="24" t="n"/>
+      <c r="G35" s="22" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="22" t="inlineStr">
+      <c r="A36" s="21" t="inlineStr">
         <is>
           <t>summary.seller_entity</t>
         </is>
@@ -4863,10 +7304,10 @@
         </is>
       </c>
       <c r="F36" s="12" t="n"/>
-      <c r="G36" s="24" t="n"/>
+      <c r="G36" s="22" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="22" t="inlineStr">
+      <c r="A37" s="21" t="inlineStr">
         <is>
           <t>summary.state</t>
         </is>
@@ -4892,10 +7333,10 @@
         </is>
       </c>
       <c r="F37" s="12" t="n"/>
-      <c r="G37" s="24" t="n"/>
+      <c r="G37" s="22" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="22" t="inlineStr">
+      <c r="A38" s="21" t="inlineStr">
         <is>
           <t>summary.street_address</t>
         </is>
@@ -4921,14 +7362,14 @@
         </is>
       </c>
       <c r="F38" s="12" t="n"/>
-      <c r="G38" s="23" t="inlineStr">
+      <c r="G38" s="19" t="inlineStr">
         <is>
           <t>1400 Example Parkway</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="22" t="inlineStr">
+      <c r="A39" s="21" t="inlineStr">
         <is>
           <t>summary.structure</t>
         </is>
@@ -4954,14 +7395,14 @@
         </is>
       </c>
       <c r="F39" s="12" t="n"/>
-      <c r="G39" s="23" t="inlineStr">
+      <c r="G39" s="19" t="inlineStr">
         <is>
           <t>Three-story garden, surface parked</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="22" t="inlineStr">
+      <c r="A40" s="21" t="inlineStr">
         <is>
           <t>summary.tax_area_code</t>
         </is>
@@ -4987,10 +7428,10 @@
         </is>
       </c>
       <c r="F40" s="12" t="n"/>
-      <c r="G40" s="24" t="n"/>
+      <c r="G40" s="22" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="22" t="inlineStr">
+      <c r="A41" s="21" t="inlineStr">
         <is>
           <t>summary.tax_basis_label</t>
         </is>
@@ -5016,10 +7457,10 @@
         </is>
       </c>
       <c r="F41" s="12" t="n"/>
-      <c r="G41" s="24" t="n"/>
+      <c r="G41" s="22" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="22" t="inlineStr">
+      <c r="A42" s="21" t="inlineStr">
         <is>
           <t>summary.tax_basis_note</t>
         </is>
@@ -5045,10 +7486,10 @@
         </is>
       </c>
       <c r="F42" s="12" t="n"/>
-      <c r="G42" s="24" t="n"/>
+      <c r="G42" s="22" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="22" t="inlineStr">
+      <c r="A43" s="21" t="inlineStr">
         <is>
           <t>summary.tax_billed_amount</t>
         </is>
@@ -5074,10 +7515,10 @@
         </is>
       </c>
       <c r="F43" s="12" t="n"/>
-      <c r="G43" s="24" t="n"/>
+      <c r="G43" s="22" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="22" t="inlineStr">
+      <c r="A44" s="21" t="inlineStr">
         <is>
           <t>summary.tax_billed_year</t>
         </is>
@@ -5103,10 +7544,10 @@
         </is>
       </c>
       <c r="F44" s="12" t="n"/>
-      <c r="G44" s="24" t="n"/>
+      <c r="G44" s="22" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="22" t="inlineStr">
+      <c r="A45" s="21" t="inlineStr">
         <is>
           <t>summary.tax_divisor</t>
         </is>
@@ -5132,10 +7573,10 @@
         </is>
       </c>
       <c r="F45" s="12" t="n"/>
-      <c r="G45" s="24" t="n"/>
+      <c r="G45" s="22" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="22" t="inlineStr">
+      <c r="A46" s="21" t="inlineStr">
         <is>
           <t>summary.tax_exemption</t>
         </is>
@@ -5161,10 +7602,10 @@
         </is>
       </c>
       <c r="F46" s="12" t="n"/>
-      <c r="G46" s="24" t="n"/>
+      <c r="G46" s="22" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="22" t="inlineStr">
+      <c r="A47" s="21" t="inlineStr">
         <is>
           <t>summary.tax_parcel_id</t>
         </is>
@@ -5190,10 +7631,10 @@
         </is>
       </c>
       <c r="F47" s="12" t="n"/>
-      <c r="G47" s="24" t="n"/>
+      <c r="G47" s="22" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="22" t="inlineStr">
+      <c r="A48" s="21" t="inlineStr">
         <is>
           <t>summary.tax_rate_as_billed</t>
         </is>
@@ -5219,10 +7660,10 @@
         </is>
       </c>
       <c r="F48" s="12" t="n"/>
-      <c r="G48" s="24" t="n"/>
+      <c r="G48" s="22" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="22" t="inlineStr">
+      <c r="A49" s="21" t="inlineStr">
         <is>
           <t>summary.unit_count</t>
         </is>
@@ -5252,14 +7693,14 @@
           <t>rent_roll.units</t>
         </is>
       </c>
-      <c r="G49" s="23" t="inlineStr">
+      <c r="G49" s="19" t="inlineStr">
         <is>
           <t>Distinct unit identifiers on the roll.</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="22" t="inlineStr">
+      <c r="A50" s="21" t="inlineStr">
         <is>
           <t>summary.year_built</t>
         </is>
@@ -5285,10 +7726,10 @@
         </is>
       </c>
       <c r="F50" s="12" t="n"/>
-      <c r="G50" s="24" t="n"/>
+      <c r="G50" s="22" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="22" t="inlineStr">
+      <c r="A51" s="21" t="inlineStr">
         <is>
           <t>summary.zip</t>
         </is>
@@ -5314,10 +7755,10 @@
         </is>
       </c>
       <c r="F51" s="12" t="n"/>
-      <c r="G51" s="24" t="n"/>
+      <c r="G51" s="22" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="22" t="inlineStr">
+      <c r="A52" s="21" t="inlineStr">
         <is>
           <t>supply.rings</t>
         </is>
@@ -5343,7 +7784,7 @@
         </is>
       </c>
       <c r="F52" s="12" t="n"/>
-      <c r="G52" s="23" t="inlineStr">
+      <c r="G52" s="19" t="inlineStr">
         <is>
           <t>Permit and entitlement records.</t>
         </is>

</xml_diff>

<commit_message>
restage the fixture: its Notes tab now describes ITS OWN property
The published fixture was asserting the showcase deal's facts - a 1981 vintage, a
9%/1.5% comp spread, market rent below in-place. All false of Fixture Park, which is
a 2019 build. Notes that quote numbers are now derived from the deal they are
attached to, so the fixture says "built 2019 ... +3.8%" and does not claim a
below-in-place market rent it does not have.

Property tax figures also change here: the tax formula now carries the exemption and
the divisor as cells instead of inlining the divisor, so the workbook computes what
compute.py computes.
</commit_message>
<xml_diff>
--- a/public/downloads/underwriting-demo/sample-deal-summary.xlsx
+++ b/public/downloads/underwriting-demo/sample-deal-summary.xlsx
@@ -3408,7 +3408,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -3530,313 +3530,328 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Rate divisor</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>Synthetic county tax record — Rate table</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
           <t>Rate evidence</t>
         </is>
       </c>
-      <c r="B11" s="12" t="n"/>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="B10" s="12" t="n"/>
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>Rate as billed, 2.148 per $100 of assessed value, read from the synthetic county bill for the 2025 tax year.</t>
         </is>
       </c>
     </row>
-    <row r="12"/>
+    <row r="11"/>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Current year — computed, then checked against the bill</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n"/>
+      <c r="C12" s="4" t="n"/>
+      <c r="D12" s="4" t="n"/>
+    </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>Current year — computed, then checked against the bill</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="n"/>
-      <c r="C13" s="4" t="n"/>
-      <c r="D13" s="4" t="n"/>
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Assessed-value basis</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="n">
+        <v>23000000</v>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>Assessed value (synthetic)</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>Synthetic county tax record — Valuation notice</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Assessed-value basis</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="n">
-        <v>23000000</v>
-      </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>Assessed value (synthetic)</t>
-        </is>
-      </c>
-      <c r="D14" s="6" t="inlineStr">
-        <is>
-          <t>Synthetic county tax record — Valuation notice</t>
-        </is>
+          <t>Assessment ratio</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Assessment ratio</t>
-        </is>
-      </c>
-      <c r="B15" s="11" t="n">
-        <v>1</v>
+          <t>Assessed value</t>
+        </is>
+      </c>
+      <c r="B15" s="7">
+        <f>B13*B14</f>
+        <v/>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>Basis times the legal-class ratio.</t>
+        </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Assessed value</t>
-        </is>
-      </c>
-      <c r="B16" s="7">
-        <f>B14*B15</f>
-        <v/>
-      </c>
-      <c r="C16" s="6" t="inlineStr">
-        <is>
-          <t>Basis times the legal-class ratio.</t>
-        </is>
+          <t>Combined rate</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="n">
+        <v>2.148</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>Combined rate</t>
-        </is>
-      </c>
-      <c r="B17" s="10" t="n">
-        <v>2.148</v>
+          <t>Rate divisor (per)</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>The rate's unit. Never defaulted: it decides whether the rate is per $100 or per $1,000.</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Computed annual tax</t>
-        </is>
-      </c>
-      <c r="B18" s="7">
-        <f>B16*B17/100</f>
-        <v/>
-      </c>
-      <c r="C18" s="6" t="inlineStr">
-        <is>
-          <t>Assessed value times rate, per $100.</t>
+          <t>Exemption</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>Synthetic county tax record — Valuation notice</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>County billed amount</t>
-        </is>
-      </c>
-      <c r="B19" s="7" t="n">
-        <v>494040</v>
+          <t>Computed annual tax</t>
+        </is>
+      </c>
+      <c r="B19" s="7">
+        <f>IF(AND(ISNUMBER(B15),ISNUMBER(B16),ISNUMBER(B17)),MAX(0,B15*B16/B17-B18),"MISSING")</f>
+        <v/>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>As billed for 2025.</t>
-        </is>
-      </c>
-      <c r="D19" s="6" t="inlineStr">
-        <is>
-          <t>Synthetic county tax record — Tax bill</t>
+          <t>Assessed value times rate over the divisor, less any exemption. A missing divisor reads MISSING rather than assuming one.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Computed less billed</t>
-        </is>
-      </c>
-      <c r="B20" s="7">
-        <f>IF(AND(ISNUMBER(B18),ISNUMBER(B19)),B18-B19,"NOT CHECKED")</f>
-        <v/>
+          <t>County billed amount</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="n">
+        <v>494040</v>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>Guarded: a missing input renders NOT CHECKED rather than a difference of zero.</t>
+          <t>As billed for 2025.</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>Synthetic county tax record — Tax bill</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
+          <t>Computed less billed</t>
+        </is>
+      </c>
+      <c r="B21" s="7">
+        <f>IF(AND(ISNUMBER(B19),ISNUMBER(B20)),B19-B20,"NOT CHECKED")</f>
+        <v/>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>Guarded: a missing input renders NOT CHECKED rather than a difference of zero.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
           <t>Check</t>
         </is>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>ties</t>
         </is>
       </c>
-      <c r="C21" s="6" t="inlineStr">
+      <c r="C22" s="6" t="inlineStr">
         <is>
           <t>Ties within 2% of the billed figure.</t>
         </is>
       </c>
     </row>
-    <row r="22"/>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+    <row r="23"/>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>Underwriting assumption at the illustrative price</t>
         </is>
       </c>
-      <c r="B23" s="4" t="n"/>
-      <c r="C23" s="4" t="n"/>
-      <c r="D23" s="4" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>State</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>TX</t>
-        </is>
-      </c>
+      <c r="B24" s="4" t="n"/>
+      <c r="C24" s="4" t="n"/>
+      <c r="D24" s="4" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>Does the basis reset on sale?</t>
+          <t>State</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="C25" s="6" t="inlineStr">
-        <is>
-          <t>TX reassesses toward the transaction price, so the generic pattern applies: assessed value is the purchase price times the statutory assessment ratio.</t>
+          <t>TX</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>Illustrative purchase price (illustrative)</t>
-        </is>
-      </c>
-      <c r="B26" s="7" t="n">
-        <v>38700000</v>
+          <t>Does the basis reset on sale?</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>TX reassesses toward the transaction price, so the generic pattern applies: assessed value is the purchase price times the statutory assessment ratio.</t>
+        </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>Year-one basis</t>
+          <t>Illustrative purchase price (illustrative)</t>
         </is>
       </c>
       <c r="B27" s="7" t="n">
         <v>38700000</v>
       </c>
-      <c r="C27" s="6" t="inlineStr">
-        <is>
-          <t>Purchase price x assessment ratio</t>
-        </is>
-      </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Year-one assessed value</t>
+          <t>Year-one basis</t>
         </is>
       </c>
       <c r="B28" s="7" t="n">
         <v>38700000</v>
       </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>Purchase price x assessment ratio</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>Year-one tax (illustrative)</t>
+          <t>Year-one assessed value</t>
         </is>
       </c>
       <c r="B29" s="7" t="n">
-        <v>831276.0000000001</v>
-      </c>
-      <c r="C29" s="6" t="inlineStr">
-        <is>
-          <t>The figure to carry into the model.</t>
-        </is>
+        <v>38700000</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
+          <t>Year-one tax (illustrative)</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="n">
+        <v>831276.0000000001</v>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>The figure to carry into the model.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
           <t>Year-one tax per unit (illustrative)</t>
         </is>
       </c>
-      <c r="B30" s="7" t="n">
+      <c r="B31" s="7" t="n">
         <v>4618.200000000001</v>
       </c>
     </row>
-    <row r="31"/>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
+    <row r="32"/>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
         <is>
           <t>What the generic shortcut would have said</t>
         </is>
       </c>
-      <c r="B32" s="4" t="n"/>
-      <c r="C32" s="4" t="n"/>
-      <c r="D32" s="4" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="5" t="inlineStr">
-        <is>
-          <t>Assessed value if it reset to the price</t>
-        </is>
-      </c>
-      <c r="B33" s="7" t="n">
-        <v>38700000</v>
-      </c>
-      <c r="C33" s="6" t="inlineStr">
-        <is>
-          <t>Purchase price times the assessment ratio — the pattern that holds in most states.</t>
-        </is>
-      </c>
+      <c r="B33" s="4" t="n"/>
+      <c r="C33" s="4" t="n"/>
+      <c r="D33" s="4" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>Tax on that basis</t>
+          <t>Assessed value if it reset to the price</t>
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>831276.0000000001</v>
+        <v>38700000</v>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>Purchase price times the assessment ratio — the pattern that holds in most states.</t>
+        </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
+          <t>Tax on that basis</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="n">
+        <v>831276.0000000001</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
           <t>Overstatement versus the correct approach</t>
         </is>
       </c>
-      <c r="B35" s="18" t="n">
+      <c r="B36" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="C35" s="6" t="inlineStr">
+      <c r="C36" s="6" t="inlineStr">
         <is>
           <t>Shown because the size of the error is the point. Carrying the generic pattern into an Arizona model does not shade the answer, it changes it: a tax line this far out fails a deal that works.</t>
         </is>
@@ -6012,7 +6027,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -6122,7 +6137,7 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Comps are matched on vintage, and it changes the answer</t>
+          <t>Comps are matched on vintage</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
@@ -6132,7 +6147,7 @@
       </c>
       <c r="C9" s="19" t="inlineStr">
         <is>
-          <t>The detailed tiers hold only communities within ten years of the subject's year built. This is not cosmetic. On this deal the flat comp set — every nearby community with rents — averaged a 1981 asset against product built 1994 to 2026 and read the subject as roughly 9% BELOW market. Restricted to same-vintage comps the subject is about 1.5% ABOVE market. The first number was measuring the age gap, not the market. Whenever a comp set is wide enough to include newer product, the spread it reports is partly a renovation and amenity story wearing a rent label.</t>
+          <t>The detailed tiers hold only communities within ten years of the subject's year built. This is not cosmetic. Whenever a comp set is wide enough to include materially newer product, part of the spread it reports is a renovation and amenity story wearing a rent label — and the wider the vintage range, the more of it is. Where this output set has measured the difference on its own subject, the figures appear in the note below rather than here.</t>
         </is>
       </c>
     </row>
@@ -6166,7 +6181,7 @@
       </c>
       <c r="C11" s="19" t="inlineStr">
         <is>
-          <t>Market rent for the model is the new-lease average where a plan has new leases inside the lookback window, and in-place rent where it does not. It is never the average of new and renewal leases together. A blended figure reads as market rent and is not one: renewals are priced off the existing rent, so blending them in drags the number toward where rents used to be and understates the gap the underwriting is trying to measure. On this deal that rule produces a market rent BELOW in-place, which is the correct and uncomfortable answer for an asset whose in-place rents sit above what the market is currently signing.</t>
+          <t>Market rent for the model is the new-lease average where a plan has new leases inside the lookback window, and in-place rent where it does not. It is never the average of new and renewal leases together. A blended figure reads as market rent and is not one: renewals are priced off the existing rent, so blending them in drags the number toward where rents used to be and understates the gap the underwriting is trying to measure. On an asset whose in-place rents sit above what the market is currently signing, the rule produces a market rent BELOW in-place — which is the correct and uncomfortable answer, and the one a blend would hide.</t>
         </is>
       </c>
     </row>
@@ -6217,7 +6232,7 @@
       </c>
       <c r="C14" s="19" t="inlineStr">
         <is>
-          <t>The supply section is real and unmodified — the rings, stages and unit counts come from a public permit and entitlement pipeline, and the zeros in the tight rings are genuine rather than missing. Coverage of that pipeline is an area of ongoing work: a ring showing no active supply means nothing was matched in the sources covered so far, which is a weaker statement than nothing being built. This section will be expanded; read it as a floor on competing supply, not a census of it.</t>
+          <t>The supply section is real and unmodified — the rings, stages and unit counts come from a public permit and entitlement pipeline, and a zero is a genuine zero rather than a gap left blank. Coverage of that pipeline is an area of ongoing work: a ring showing no active supply means nothing was matched in the sources covered so far, which is a weaker statement than nothing being built. This section will be expanded; read it as a floor on competing supply, not a census of it.</t>
         </is>
       </c>
     </row>
@@ -6241,49 +6256,66 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>This deal does not exist</t>
+          <t>What vintage-matching changed on this deal</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>throughout</t>
+          <t>Rent Comps — tiers</t>
         </is>
       </c>
       <c r="C16" s="19" t="inlineStr">
         <is>
-          <t>Fixture Park is fabricated end to end — the property, the operating statement, the rent roll, the comps and the demographics. It exists to exercise every edge the writers handle, so some of its figures are deliberately awkward: a plan with no priced units, a comp community with no published year, a revenue line the source statement never subtotalled.</t>
+          <t>On this subject — built 2019 — the vintage-matched comp set reads +3.8% against the subject's own rent, while a flat average over every nearby community with rents reads +8.1%. The flat set spans vintages 1998 to 2022; the matched set holds 2009 to 2029, inside the +/-10-year band. The difference between those two numbers is the age gap, not the market.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>The 1-mile demographic ring overstates levels</t>
+          <t>This deal does not exist</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Demand</t>
+          <t>throughout</t>
         </is>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>The 1-mile column overstates levels. Ring membership is decided by each census block group's internal point and then the whole block group is counted, so at 1 mile a single large block group can sit mostly outside the ring and still be counted whole. Measured against a commercial source, 1-mile population reads roughly 2.3x and households roughly 1.9x too high; the 3-, 5- and 10-mile columns do not have this problem. Read the 1-mile column for mix and shares, which are ratios and survive the overcount, and read levels off the 3-mile column.</t>
+          <t>Fixture Park is fabricated end to end — the property, the operating statement, the rent roll, the comps and the demographics. It exists to exercise every edge the writers handle, so some of its figures are deliberately awkward: a plan with no priced units, a comp community with no published year, a revenue line the source statement never subtotalled.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
+          <t>The 1-mile demographic ring overstates levels</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Demand</t>
+        </is>
+      </c>
+      <c r="C18" s="19" t="inlineStr">
+        <is>
+          <t>The 1-mile column overstates levels. Ring membership is decided by each census block group's internal point and then the whole block group is counted, so at 1 mile a single large block group can sit mostly outside the ring and still be counted whole. Measured against a commercial source, 1-mile population reads roughly 2.3x and households roughly 1.9x too high; the 3-, 5- and 10-mile columns do not have this problem. Read the 1-mile column for mix and shares, which are ratios and survive the overcount, and read levels off the 3-mile column.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
           <t>The rent readback checks transcription, not column choice</t>
         </is>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>Error Checks &amp; Pricing</t>
         </is>
       </c>
-      <c r="C18" s="19" t="inlineStr">
+      <c r="C19" s="19" t="inlineStr">
         <is>
           <t>Ten units are sampled and their normalized in-place rent is compared against the raw cell it came from, which catches a coercion or transcription error. It cannot catch the wrong rent column having been chosen, because both sides read the same column. The sample is seeded from the roll's as-of date, so the same roll always checks the same units.</t>
         </is>

</xml_diff>

<commit_message>
restage the fixture: the vintage note now compares vintage, not mix-weighting
The published note claimed a contrast between vintage-matched comps and "every nearby
community with rents". Both figures actually came from the same vintage-filtered rows,
so the second population was never measured - and the sign was inverted, saying the
comp set read against the subject when the ratio is the subject against the comps.

The unrestricted baseline is now measured at selection time (tier 3 publishes no rents
by design, so it could not be derived downstream) and mix-matched identically, so the
only difference between the two figures is which communities are included.

Property tax also gains distinct full-value and assessed-value rows, each labelled for
what it holds, and the exemption cell now carries a number rather than text.
</commit_message>
<xml_diff>
--- a/public/downloads/underwriting-demo/sample-deal-summary.xlsx
+++ b/public/downloads/underwriting-demo/sample-deal-summary.xlsx
@@ -3759,7 +3759,7 @@
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Year-one basis</t>
+          <t>Year-one full value</t>
         </is>
       </c>
       <c r="B28" s="7" t="n">
@@ -3767,7 +3767,7 @@
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>Purchase price x assessment ratio</t>
+          <t>Purchase price (the transaction resets the basis)</t>
         </is>
       </c>
     </row>
@@ -3779,6 +3779,11 @@
       </c>
       <c r="B29" s="7" t="n">
         <v>38700000</v>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>Assessed value = full value x assessment ratio</t>
+        </is>
       </c>
     </row>
     <row r="30">
@@ -6266,7 +6271,7 @@
       </c>
       <c r="C16" s="19" t="inlineStr">
         <is>
-          <t>On this subject — built 2019 — the vintage-matched comp set reads +3.8% against the subject's own rent, while a flat average over every nearby community with rents reads +8.1%. The flat set spans vintages 1998 to 2022; the matched set holds 2009 to 2029, inside the +/-10-year band. The difference between those two numbers is the age gap, not the market.</t>
+          <t>This subject was built 2019. Against comps within +/-10 years of that — 11 communities, vintages 2009 to 2029 — its rent sits 3.8% above the comp set. Against every community in the radius with quoted rent, 14 of them spanning 1998 to 2029, the same rent sits 6.3% below the comp set. Both figures weight the comp side by this property's own unit mix, so the only difference between them is which communities are included: the 10.1% gap is the vintage spread, not the market. A comp set wide enough to include much newer product reports part of a renovation and amenity story as if it were rent.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
restage the fixture: the vintage claim is a measurement of two sets
The note no longer asserts what vintage is worth in a market. It states the
experiment - two comp sets selected identically except for the vintage test, and how
the subject reads against each - plus the direction, and says explicitly that this is
a measurement of these two sets on this date.

Both sets are now shown side by side on the Rent Comps section, since the note points
there: community counts, vintage spans, comp rents, and which communities swap.
</commit_message>
<xml_diff>
--- a/public/downloads/underwriting-demo/sample-deal-summary.xlsx
+++ b/public/downloads/underwriting-demo/sample-deal-summary.xlsx
@@ -69,7 +69,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -84,6 +84,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9D9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -118,7 +123,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -141,6 +146,10 @@
     <xf numFmtId="166" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="169" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -1509,14 +1518,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N58"/>
+  <dimension ref="A1:N69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
     <col width="38" customWidth="1" min="2" max="2"/>
     <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="42" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
@@ -3394,6 +3403,141 @@
       <c r="C58" s="6" t="inlineStr">
         <is>
           <t>Negative means the subject is underwritten BELOW the market — mark-to-market room rather than a stretch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59"/>
+    <row r="60">
+      <c r="A60" s="4" t="inlineStr">
+        <is>
+          <t>Two comp sets, selected identically except for the vintage test</t>
+        </is>
+      </c>
+      <c r="B60" s="4" t="n"/>
+      <c r="C60" s="4" t="n"/>
+      <c r="D60" s="4" t="n"/>
+      <c r="E60" s="4" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="6" t="inlineStr">
+        <is>
+          <t>Held fixed in both: candidate pool, product test, tracker comp exclusions, radius, closest-20 cap, per-community rent rules, mix weighting. Varied: the +/-10-year vintage test only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="14" t="inlineStr">
+        <is>
+          <t>Comp set</t>
+        </is>
+      </c>
+      <c r="B62" s="14" t="inlineStr">
+        <is>
+          <t>Communities</t>
+        </is>
+      </c>
+      <c r="C62" s="14" t="inlineStr">
+        <is>
+          <t>Vintages</t>
+        </is>
+      </c>
+      <c r="D62" s="14" t="inlineStr">
+        <is>
+          <t>Comp net effective</t>
+        </is>
+      </c>
+      <c r="E62" s="14" t="inlineStr">
+        <is>
+          <t>Subject reads</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="5" t="inlineStr">
+        <is>
+          <t>A — vintage test ON</t>
+        </is>
+      </c>
+      <c r="B63" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="C63" s="5" t="inlineStr">
+        <is>
+          <t>2009–2029</t>
+        </is>
+      </c>
+      <c r="D63" s="7" t="n">
+        <v>1767.409090909091</v>
+      </c>
+      <c r="E63" s="11" t="n">
+        <v>0.03811720060466306</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr">
+        <is>
+          <t>B — vintage test OFF</t>
+        </is>
+      </c>
+      <c r="B64" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="C64" s="5" t="inlineStr">
+        <is>
+          <t>1998–2029</t>
+        </is>
+      </c>
+      <c r="D64" s="7" t="n">
+        <v>1957.821666666666</v>
+      </c>
+      <c r="E64" s="11" t="n">
+        <v>-0.06284734252552215</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="18" t="inlineStr">
+        <is>
+          <t>Difference between the two sets</t>
+        </is>
+      </c>
+      <c r="B65" s="19" t="n"/>
+      <c r="C65" s="19" t="n"/>
+      <c r="D65" s="20" t="n">
+        <v>190.4125757575757</v>
+      </c>
+      <c r="E65" s="21" t="n">
+        <v>0.1009645431301852</v>
+      </c>
+    </row>
+    <row r="66"/>
+    <row r="67">
+      <c r="A67" s="5" t="inlineStr">
+        <is>
+          <t>In B but not A</t>
+        </is>
+      </c>
+      <c r="B67" s="5" t="inlineStr">
+        <is>
+          <t>Stonecrest Lofts</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="5" t="inlineStr">
+        <is>
+          <t>In A but not B</t>
+        </is>
+      </c>
+      <c r="B68" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="6" t="inlineStr">
+        <is>
+          <t>Both figures are weighted by this property's own unit mix and computed over the same bed counts, so the two rows describe the same product. This is what these two sets measured on this date; it is not an estimate of what vintage is worth in this market.</t>
         </is>
       </c>
     </row>
@@ -3853,7 +3997,7 @@
           <t>Overstatement versus the correct approach</t>
         </is>
       </c>
-      <c r="B36" s="18" t="n">
+      <c r="B36" s="22" t="n">
         <v>1</v>
       </c>
       <c r="C36" s="6" t="inlineStr">
@@ -6099,7 +6243,7 @@
           <t>Deal Summary — Pricing</t>
         </is>
       </c>
-      <c r="C6" s="19" t="inlineStr">
+      <c r="C6" s="23" t="inlineStr">
         <is>
           <t>Every price, per-unit figure and cap rate in this set is illustrative. The per-unit price is a round number chosen to sit inside the band a real per-unit sale price occupies, so the cap-rate arithmetic is realistic. It is not a quote, an offer, a broker's guidance, or a valuation. Cap rates move inversely with the price, so read them as a demonstration of the mechanics rather than a view on the asset.</t>
         </is>
@@ -6116,7 +6260,7 @@
           <t>Rent Comps</t>
         </is>
       </c>
-      <c r="C7" s="19" t="inlineStr">
+      <c r="C7" s="23" t="inlineStr">
         <is>
           <t>No subscription or licensed market-data feed appears anywhere in this set. Comps come only from an operator's own weekly scrape of public leasing pages. That is a deliberate constraint, not a gap: licensed data cannot travel outside the licence, so a portfolio piece built on it could not be shown at all. The cost is coverage, and the coverage is measured and stated rather than assumed.</t>
         </is>
@@ -6133,7 +6277,7 @@
           <t>Rent Comps</t>
         </is>
       </c>
-      <c r="C8" s="19" t="inlineStr">
+      <c r="C8" s="23" t="inlineStr">
         <is>
           <t>Three miles, because that is the ring where the operator's own scrape actually holds live rents for enough communities to say something. A wider ring would add distance without adding evidence — it trades real rents for guesses. The coverage sentence on the comp block is measured by a probe against the scraper's own status values, never written by hand.</t>
         </is>
@@ -6150,9 +6294,9 @@
           <t>Rent Comps — tiers</t>
         </is>
       </c>
-      <c r="C9" s="19" t="inlineStr">
-        <is>
-          <t>The detailed tiers hold only communities within ten years of the subject's year built. This is not cosmetic. Whenever a comp set is wide enough to include materially newer product, part of the spread it reports is a renovation and amenity story wearing a rent label — and the wider the vintage range, the more of it is. Where this output set has measured the difference on its own subject, the figures appear in the note below rather than here.</t>
+      <c r="C9" s="23" t="inlineStr">
+        <is>
+          <t>The detailed tiers hold only communities within ten years of the subject's year built. Widening that range changes which communities are in the set, and a set that includes materially newer product will generally report a different rent — how much, and in which direction, is a property of the particular submarket and date, not a rule. Where this output set has measured the difference between two otherwise-identical comp sets on its own subject, the figures appear in the note below.</t>
         </is>
       </c>
     </row>
@@ -6167,7 +6311,7 @@
           <t>Rent Comps — tiers</t>
         </is>
       </c>
-      <c r="C10" s="19" t="inlineStr">
+      <c r="C10" s="23" t="inlineStr">
         <is>
           <t>The rent tracker has no year-built column. Where a vintage appears here it was parsed out of a free-text note on the community record, and every row carries that as its source. A community with no such note keeps its place in the comp set on distance and product, shows a dash for the year, and the tier header says how many rows the vintage filter could not be applied to. Inventing a year would fabricate the evidence the filter runs on; dropping the community would hide the closest comps for want of a field the source never had.</t>
         </is>
@@ -6184,7 +6328,7 @@
           <t>Rent Roll — Summary</t>
         </is>
       </c>
-      <c r="C11" s="19" t="inlineStr">
+      <c r="C11" s="23" t="inlineStr">
         <is>
           <t>Market rent for the model is the new-lease average where a plan has new leases inside the lookback window, and in-place rent where it does not. It is never the average of new and renewal leases together. A blended figure reads as market rent and is not one: renewals are priced off the existing rent, so blending them in drags the number toward where rents used to be and understates the gap the underwriting is trying to measure. On an asset whose in-place rents sit above what the market is currently signing, the rule produces a market rent BELOW in-place — which is the correct and uncomfortable answer, and the one a blend would hide.</t>
         </is>
@@ -6201,7 +6345,7 @@
           <t>throughout</t>
         </is>
       </c>
-      <c r="C12" s="19" t="inlineStr">
+      <c r="C12" s="23" t="inlineStr">
         <is>
           <t>Where a figure is derived rather than read, the audit trail says so and names the inputs. Where a figure is unknown, the cell shows a visible hole rather than a plausible-looking number. A blank that reads as a zero is the most expensive kind of missing data, because nothing downstream flags it.</t>
         </is>
@@ -6218,7 +6362,7 @@
           <t>Lease Trade-Out</t>
         </is>
       </c>
-      <c r="C13" s="19" t="inlineStr">
+      <c r="C13" s="23" t="inlineStr">
         <is>
           <t>Where a trade-out block appears with no rows, that is because the source report was not used, not because the data does not exist. Trade-out is derived from the rent roll's own lease dates and rents instead, so every figure in this set traces back to one of three raw sources. An output whose provenance forks across more documents than it needs is harder to audit for no analytical gain.</t>
         </is>
@@ -6235,7 +6379,7 @@
           <t>Supply</t>
         </is>
       </c>
-      <c r="C14" s="19" t="inlineStr">
+      <c r="C14" s="23" t="inlineStr">
         <is>
           <t>The supply section is real and unmodified — the rings, stages and unit counts come from a public permit and entitlement pipeline, and a zero is a genuine zero rather than a gap left blank. Coverage of that pipeline is an area of ongoing work: a ring showing no active supply means nothing was matched in the sources covered so far, which is a weaker statement than nothing being built. This section will be expanded; read it as a floor on competing supply, not a census of it.</t>
         </is>
@@ -6252,7 +6396,7 @@
           <t>Error Checks &amp; Pricing</t>
         </is>
       </c>
-      <c r="C15" s="19" t="inlineStr">
+      <c r="C15" s="23" t="inlineStr">
         <is>
           <t>Every cross-tie on the checks tab reports OK, FAIL, or NOT CHECKED. A check missing one of its inputs reports NOT CHECKED and claims no difference — it never reports OK. A green result that only means 'this check could not run' is worse than a red one, because it buys confidence it has not earned.</t>
         </is>
@@ -6269,9 +6413,9 @@
           <t>Rent Comps — tiers</t>
         </is>
       </c>
-      <c r="C16" s="19" t="inlineStr">
-        <is>
-          <t>This subject was built 2019. Its rent sits 3.8% above a comp set restricted to +/-10 years of that (11 communities, vintages 2009 to 2029). Run the SAME selection with the vintage test switched off and nothing else changed — same product test, same tracker exclusions, same radius, same closest-11 cap, same rent rules, same mix weighting — and 1 communities swap in (vintages now 1998 to 2029), putting the same rent 6.3% below the comp set instead. Both figures are weighted by this property's own unit mix and computed over the same bed counts (100% of its units), so the 10.1 point difference is the vintage effect and not a mixture of criteria. A comp set wide enough to include much newer product reports part of a renovation and amenity story as if it were rent.</t>
+      <c r="C16" s="23" t="inlineStr">
+        <is>
+          <t>This subject was built 2019. Two comp sets were selected by identical criteria — same candidate pool, same product test, same tracker exclusions, same radius, same closest-11 cap, same rent rules, same mix weighting — differing only in whether the +/-10-year vintage test was applied. Set A, vintage test ON: 11 communities, vintages 2009 to 2029; this subject's rent reads 3.8% above it. Set B, vintage test OFF: 1 of those communities are replaced (vintages 1998 to 2029); the same rent reads 6.3% below it. Both figures are weighted by this property's own unit mix and computed over the same bed counts (100% of its units), so the two sets differ by 10.1 points. Direction: the newer communities nearby rent above this subject's own vintage cohort. Both sets are listed on the Rent Comps section — this is a measurement of these two sets on this date, not an estimate of what vintage is worth in this market.</t>
         </is>
       </c>
     </row>
@@ -6286,7 +6430,7 @@
           <t>throughout</t>
         </is>
       </c>
-      <c r="C17" s="19" t="inlineStr">
+      <c r="C17" s="23" t="inlineStr">
         <is>
           <t>Fixture Park is fabricated end to end — the property, the operating statement, the rent roll, the comps and the demographics. It exists to exercise every edge the writers handle, so some of its figures are deliberately awkward: a plan with no priced units, a comp community with no published year, a revenue line the source statement never subtotalled.</t>
         </is>
@@ -6303,7 +6447,7 @@
           <t>Demand</t>
         </is>
       </c>
-      <c r="C18" s="19" t="inlineStr">
+      <c r="C18" s="23" t="inlineStr">
         <is>
           <t>The 1-mile column overstates levels. Ring membership is decided by each census block group's internal point and then the whole block group is counted, so at 1 mile a single large block group can sit mostly outside the ring and still be counted whole. Measured against a commercial source, 1-mile population reads roughly 2.3x and households roughly 1.9x too high; the 3-, 5- and 10-mile columns do not have this problem. Read the 1-mile column for mix and shares, which are ratios and survive the overcount, and read levels off the 3-mile column.</t>
         </is>
@@ -6320,7 +6464,7 @@
           <t>Error Checks &amp; Pricing</t>
         </is>
       </c>
-      <c r="C19" s="19" t="inlineStr">
+      <c r="C19" s="23" t="inlineStr">
         <is>
           <t>Ten units are sampled and their normalized in-place rent is compared against the raw cell it came from, which catches a coercion or transcription error. It cannot catch the wrong rent column having been chosen, because both sides read the same column. The sample is seeded from the roll's as-of date, so the same roll always checks the same units.</t>
         </is>
@@ -6386,7 +6530,7 @@
           <t>Stamped values in this workbook</t>
         </is>
       </c>
-      <c r="B5" s="20" t="n">
+      <c r="B5" s="24" t="n">
         <v>44</v>
       </c>
     </row>
@@ -6440,7 +6584,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="21" t="inlineStr">
+      <c r="A9" s="25" t="inlineStr">
         <is>
           <t>closing_costs.mortgage_tax.amount</t>
         </is>
@@ -6470,14 +6614,14 @@
           <t>closing_costs.loan_amount, summary.state</t>
         </is>
       </c>
-      <c r="G9" s="19" t="inlineStr">
+      <c r="G9" s="23" t="inlineStr">
         <is>
           <t>Computed on the LOAN, never on the price. With no loan amount the line is reported as not asserted rather than inferred at 100% leverage.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="21" t="inlineStr">
+      <c r="A10" s="25" t="inlineStr">
         <is>
           <t>closing_costs.transfer_tax.amount</t>
         </is>
@@ -6507,14 +6651,14 @@
           <t>pricing.price_per_unit, pricing.unit_count, summary.state, closing_costs.price</t>
         </is>
       </c>
-      <c r="G10" s="19" t="inlineStr">
+      <c r="G10" s="23" t="inlineStr">
         <is>
           <t>Rate applied to price_per_unit x unit_count. Per-unit statutes round the consideration up.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="21" t="inlineStr">
+      <c r="A11" s="25" t="inlineStr">
         <is>
           <t>comps.nearby</t>
         </is>
@@ -6544,14 +6688,14 @@
           <t>comps.rows.tier</t>
         </is>
       </c>
-      <c r="G11" s="19" t="inlineStr">
+      <c r="G11" s="23" t="inlineStr">
         <is>
           <t>Every tracked community inside the radius that is not a detail row, with the reason it is not. No rent columns.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="21" t="inlineStr">
+      <c r="A12" s="25" t="inlineStr">
         <is>
           <t>comps.rows</t>
         </is>
@@ -6577,14 +6721,14 @@
         </is>
       </c>
       <c r="F12" s="12" t="n"/>
-      <c r="G12" s="19" t="inlineStr">
+      <c r="G12" s="23" t="inlineStr">
         <is>
           <t>Own weekly scrape; asking and net effective stated separately.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="21" t="inlineStr">
+      <c r="A13" s="25" t="inlineStr">
         <is>
           <t>comps.rows.tier</t>
         </is>
@@ -6614,14 +6758,14 @@
           <t>comps.rows.distance_mi, comps.tiering.subject_product, comps.tiering.subject_year_built, comps.tiering.year_band, comps.tiering.top_n, comps.tiering.additional_n</t>
         </is>
       </c>
-      <c r="G13" s="19" t="inlineStr">
+      <c r="G13" s="23" t="inlineStr">
         <is>
           <t>Tier 1 = the closest 5 matching product and vintage; tier 2 = the next 15; everything else is tier 3, identity only. An unknown year does not disqualify — it is disclosed on the tier header instead.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="21" t="inlineStr">
+      <c r="A14" s="25" t="inlineStr">
         <is>
           <t>demand.rings</t>
         </is>
@@ -6647,14 +6791,14 @@
         </is>
       </c>
       <c r="F14" s="12" t="n"/>
-      <c r="G14" s="19" t="inlineStr">
+      <c r="G14" s="23" t="inlineStr">
         <is>
           <t>Ring demographics.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="21" t="inlineStr">
+      <c r="A15" s="25" t="inlineStr">
         <is>
           <t>pricing.price_per_unit</t>
         </is>
@@ -6680,14 +6824,14 @@
         </is>
       </c>
       <c r="F15" s="12" t="n"/>
-      <c r="G15" s="19" t="inlineStr">
+      <c r="G15" s="23" t="inlineStr">
         <is>
           <t>Illustrative. Inside the band a per-unit sale price occupies.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="21" t="inlineStr">
+      <c r="A16" s="25" t="inlineStr">
         <is>
           <t>pricing.unit_count</t>
         </is>
@@ -6717,10 +6861,10 @@
           <t>summary.unit_count</t>
         </is>
       </c>
-      <c r="G16" s="22" t="n"/>
+      <c r="G16" s="26" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="21" t="inlineStr">
+      <c r="A17" s="25" t="inlineStr">
         <is>
           <t>summary.assessed_value_basis</t>
         </is>
@@ -6746,10 +6890,10 @@
         </is>
       </c>
       <c r="F17" s="12" t="n"/>
-      <c r="G17" s="22" t="n"/>
+      <c r="G17" s="26" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="21" t="inlineStr">
+      <c r="A18" s="25" t="inlineStr">
         <is>
           <t>summary.assessment_ratio</t>
         </is>
@@ -6775,10 +6919,10 @@
         </is>
       </c>
       <c r="F18" s="12" t="n"/>
-      <c r="G18" s="22" t="n"/>
+      <c r="G18" s="26" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="21" t="inlineStr">
+      <c r="A19" s="25" t="inlineStr">
         <is>
           <t>summary.city</t>
         </is>
@@ -6804,10 +6948,10 @@
         </is>
       </c>
       <c r="F19" s="12" t="n"/>
-      <c r="G19" s="22" t="n"/>
+      <c r="G19" s="26" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="21" t="inlineStr">
+      <c r="A20" s="25" t="inlineStr">
         <is>
           <t>summary.construction_status</t>
         </is>
@@ -6833,10 +6977,10 @@
         </is>
       </c>
       <c r="F20" s="12" t="n"/>
-      <c r="G20" s="22" t="n"/>
+      <c r="G20" s="26" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="21" t="inlineStr">
+      <c r="A21" s="25" t="inlineStr">
         <is>
           <t>summary.county</t>
         </is>
@@ -6862,10 +7006,10 @@
         </is>
       </c>
       <c r="F21" s="12" t="n"/>
-      <c r="G21" s="22" t="n"/>
+      <c r="G21" s="26" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="21" t="inlineStr">
+      <c r="A22" s="25" t="inlineStr">
         <is>
           <t>summary.deal_name</t>
         </is>
@@ -6891,14 +7035,14 @@
         </is>
       </c>
       <c r="F22" s="12" t="n"/>
-      <c r="G22" s="19" t="inlineStr">
+      <c r="G22" s="23" t="inlineStr">
         <is>
           <t>Fixture Park</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="21" t="inlineStr">
+      <c r="A23" s="25" t="inlineStr">
         <is>
           <t>summary.deal_status</t>
         </is>
@@ -6924,10 +7068,10 @@
         </is>
       </c>
       <c r="F23" s="12" t="n"/>
-      <c r="G23" s="22" t="n"/>
+      <c r="G23" s="26" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="21" t="inlineStr">
+      <c r="A24" s="25" t="inlineStr">
         <is>
           <t>summary.delivery_date</t>
         </is>
@@ -6953,10 +7097,10 @@
         </is>
       </c>
       <c r="F24" s="12" t="n"/>
-      <c r="G24" s="22" t="n"/>
+      <c r="G24" s="26" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="21" t="inlineStr">
+      <c r="A25" s="25" t="inlineStr">
         <is>
           <t>summary.fair_market_value</t>
         </is>
@@ -6982,14 +7126,14 @@
         </is>
       </c>
       <c r="F25" s="12" t="n"/>
-      <c r="G25" s="19" t="inlineStr">
+      <c r="G25" s="23" t="inlineStr">
         <is>
           <t>Operator's own estimate.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="21" t="inlineStr">
+      <c r="A26" s="25" t="inlineStr">
         <is>
           <t>summary.in_place_rent_avg</t>
         </is>
@@ -7019,14 +7163,14 @@
           <t>rent_roll.units</t>
         </is>
       </c>
-      <c r="G26" s="19" t="inlineStr">
+      <c r="G26" s="23" t="inlineStr">
         <is>
           <t>Occupied units, straight off the roll.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="21" t="inlineStr">
+      <c r="A27" s="25" t="inlineStr">
         <is>
           <t>summary.listing_brokerage</t>
         </is>
@@ -7056,14 +7200,14 @@
           <t>summary.seller_entity</t>
         </is>
       </c>
-      <c r="G27" s="19" t="inlineStr">
+      <c r="G27" s="23" t="inlineStr">
         <is>
           <t>Generic label; no firm or individual is named in a published file.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="21" t="inlineStr">
+      <c r="A28" s="25" t="inlineStr">
         <is>
           <t>summary.market_rent_for_model</t>
         </is>
@@ -7093,14 +7237,14 @@
           <t>rent_roll.units</t>
         </is>
       </c>
-      <c r="G28" s="19" t="inlineStr">
+      <c r="G28" s="23" t="inlineStr">
         <is>
           <t>New-lease average where a plan has new leases in the window, else in-place. Never a blend.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="21" t="inlineStr">
+      <c r="A29" s="25" t="inlineStr">
         <is>
           <t>summary.msa</t>
         </is>
@@ -7130,14 +7274,14 @@
           <t>summary.city, summary.state</t>
         </is>
       </c>
-      <c r="G29" s="19" t="inlineStr">
+      <c r="G29" s="23" t="inlineStr">
         <is>
           <t>Metro assigned from the city/state pair.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="21" t="inlineStr">
+      <c r="A30" s="25" t="inlineStr">
         <is>
           <t>summary.pricing_guidance</t>
         </is>
@@ -7163,14 +7307,14 @@
         </is>
       </c>
       <c r="F30" s="12" t="n"/>
-      <c r="G30" s="19" t="inlineStr">
+      <c r="G30" s="23" t="inlineStr">
         <is>
           <t>Illustrative figure supplied directly; not a quote or an offer.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="21" t="inlineStr">
+      <c r="A31" s="25" t="inlineStr">
         <is>
           <t>summary.product_detail</t>
         </is>
@@ -7196,10 +7340,10 @@
         </is>
       </c>
       <c r="F31" s="12" t="n"/>
-      <c r="G31" s="22" t="n"/>
+      <c r="G31" s="26" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="21" t="inlineStr">
+      <c r="A32" s="25" t="inlineStr">
         <is>
           <t>summary.product_type</t>
         </is>
@@ -7225,10 +7369,10 @@
         </is>
       </c>
       <c r="F32" s="12" t="n"/>
-      <c r="G32" s="22" t="n"/>
+      <c r="G32" s="26" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="21" t="inlineStr">
+      <c r="A33" s="25" t="inlineStr">
         <is>
           <t>summary.school_elementary_name</t>
         </is>
@@ -7254,10 +7398,10 @@
         </is>
       </c>
       <c r="F33" s="12" t="n"/>
-      <c r="G33" s="22" t="n"/>
+      <c r="G33" s="26" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="21" t="inlineStr">
+      <c r="A34" s="25" t="inlineStr">
         <is>
           <t>summary.school_high_name</t>
         </is>
@@ -7283,10 +7427,10 @@
         </is>
       </c>
       <c r="F34" s="12" t="n"/>
-      <c r="G34" s="22" t="n"/>
+      <c r="G34" s="26" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="21" t="inlineStr">
+      <c r="A35" s="25" t="inlineStr">
         <is>
           <t>summary.school_middle_name</t>
         </is>
@@ -7312,10 +7456,10 @@
         </is>
       </c>
       <c r="F35" s="12" t="n"/>
-      <c r="G35" s="22" t="n"/>
+      <c r="G35" s="26" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="21" t="inlineStr">
+      <c r="A36" s="25" t="inlineStr">
         <is>
           <t>summary.seller_entity</t>
         </is>
@@ -7341,10 +7485,10 @@
         </is>
       </c>
       <c r="F36" s="12" t="n"/>
-      <c r="G36" s="22" t="n"/>
+      <c r="G36" s="26" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="21" t="inlineStr">
+      <c r="A37" s="25" t="inlineStr">
         <is>
           <t>summary.state</t>
         </is>
@@ -7370,10 +7514,10 @@
         </is>
       </c>
       <c r="F37" s="12" t="n"/>
-      <c r="G37" s="22" t="n"/>
+      <c r="G37" s="26" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="21" t="inlineStr">
+      <c r="A38" s="25" t="inlineStr">
         <is>
           <t>summary.street_address</t>
         </is>
@@ -7399,14 +7543,14 @@
         </is>
       </c>
       <c r="F38" s="12" t="n"/>
-      <c r="G38" s="19" t="inlineStr">
+      <c r="G38" s="23" t="inlineStr">
         <is>
           <t>1400 Example Parkway</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="21" t="inlineStr">
+      <c r="A39" s="25" t="inlineStr">
         <is>
           <t>summary.structure</t>
         </is>
@@ -7432,14 +7576,14 @@
         </is>
       </c>
       <c r="F39" s="12" t="n"/>
-      <c r="G39" s="19" t="inlineStr">
+      <c r="G39" s="23" t="inlineStr">
         <is>
           <t>Three-story garden, surface parked</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="21" t="inlineStr">
+      <c r="A40" s="25" t="inlineStr">
         <is>
           <t>summary.tax_area_code</t>
         </is>
@@ -7465,10 +7609,10 @@
         </is>
       </c>
       <c r="F40" s="12" t="n"/>
-      <c r="G40" s="22" t="n"/>
+      <c r="G40" s="26" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="21" t="inlineStr">
+      <c r="A41" s="25" t="inlineStr">
         <is>
           <t>summary.tax_basis_label</t>
         </is>
@@ -7494,10 +7638,10 @@
         </is>
       </c>
       <c r="F41" s="12" t="n"/>
-      <c r="G41" s="22" t="n"/>
+      <c r="G41" s="26" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="21" t="inlineStr">
+      <c r="A42" s="25" t="inlineStr">
         <is>
           <t>summary.tax_basis_note</t>
         </is>
@@ -7523,10 +7667,10 @@
         </is>
       </c>
       <c r="F42" s="12" t="n"/>
-      <c r="G42" s="22" t="n"/>
+      <c r="G42" s="26" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="21" t="inlineStr">
+      <c r="A43" s="25" t="inlineStr">
         <is>
           <t>summary.tax_billed_amount</t>
         </is>
@@ -7552,10 +7696,10 @@
         </is>
       </c>
       <c r="F43" s="12" t="n"/>
-      <c r="G43" s="22" t="n"/>
+      <c r="G43" s="26" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="21" t="inlineStr">
+      <c r="A44" s="25" t="inlineStr">
         <is>
           <t>summary.tax_billed_year</t>
         </is>
@@ -7581,10 +7725,10 @@
         </is>
       </c>
       <c r="F44" s="12" t="n"/>
-      <c r="G44" s="22" t="n"/>
+      <c r="G44" s="26" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="21" t="inlineStr">
+      <c r="A45" s="25" t="inlineStr">
         <is>
           <t>summary.tax_divisor</t>
         </is>
@@ -7610,10 +7754,10 @@
         </is>
       </c>
       <c r="F45" s="12" t="n"/>
-      <c r="G45" s="22" t="n"/>
+      <c r="G45" s="26" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="21" t="inlineStr">
+      <c r="A46" s="25" t="inlineStr">
         <is>
           <t>summary.tax_exemption</t>
         </is>
@@ -7639,10 +7783,10 @@
         </is>
       </c>
       <c r="F46" s="12" t="n"/>
-      <c r="G46" s="22" t="n"/>
+      <c r="G46" s="26" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="21" t="inlineStr">
+      <c r="A47" s="25" t="inlineStr">
         <is>
           <t>summary.tax_parcel_id</t>
         </is>
@@ -7668,10 +7812,10 @@
         </is>
       </c>
       <c r="F47" s="12" t="n"/>
-      <c r="G47" s="22" t="n"/>
+      <c r="G47" s="26" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="21" t="inlineStr">
+      <c r="A48" s="25" t="inlineStr">
         <is>
           <t>summary.tax_rate_as_billed</t>
         </is>
@@ -7697,10 +7841,10 @@
         </is>
       </c>
       <c r="F48" s="12" t="n"/>
-      <c r="G48" s="22" t="n"/>
+      <c r="G48" s="26" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="21" t="inlineStr">
+      <c r="A49" s="25" t="inlineStr">
         <is>
           <t>summary.unit_count</t>
         </is>
@@ -7730,14 +7874,14 @@
           <t>rent_roll.units</t>
         </is>
       </c>
-      <c r="G49" s="19" t="inlineStr">
+      <c r="G49" s="23" t="inlineStr">
         <is>
           <t>Distinct unit identifiers on the roll.</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="21" t="inlineStr">
+      <c r="A50" s="25" t="inlineStr">
         <is>
           <t>summary.year_built</t>
         </is>
@@ -7763,10 +7907,10 @@
         </is>
       </c>
       <c r="F50" s="12" t="n"/>
-      <c r="G50" s="22" t="n"/>
+      <c r="G50" s="26" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="21" t="inlineStr">
+      <c r="A51" s="25" t="inlineStr">
         <is>
           <t>summary.zip</t>
         </is>
@@ -7792,10 +7936,10 @@
         </is>
       </c>
       <c r="F51" s="12" t="n"/>
-      <c r="G51" s="22" t="n"/>
+      <c r="G51" s="26" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="21" t="inlineStr">
+      <c r="A52" s="25" t="inlineStr">
         <is>
           <t>supply.rings</t>
         </is>
@@ -7821,7 +7965,7 @@
         </is>
       </c>
       <c r="F52" s="12" t="n"/>
-      <c r="G52" s="19" t="inlineStr">
+      <c r="G52" s="23" t="inlineStr">
         <is>
           <t>Permit and entitlement records.</t>
         </is>

</xml_diff>